<commit_message>
Avances 18/03 PRE REUNIÓN: prueba de algoritmos de optimización.
</commit_message>
<xml_diff>
--- a/Optimizacion/Resultados optimizadores.xlsx
+++ b/Optimizacion/Resultados optimizadores.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uccl0-my.sharepoint.com/personal/mfernandafolch_uc_cl/Documents/Escritorio/Concha y Toro/Proyecto_Tintos_CyT_P2/Optimizacion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="894" documentId="11_AD4D2F04E46CFB4ACB3E20395551EF76693EDF1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D80D664C-0605-4EBC-81C8-2056D54ED004}"/>
+  <xr:revisionPtr revIDLastSave="1478" documentId="11_AD4D2F04E46CFB4ACB3E20395551EF76693EDF1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AA2D608-32F6-4684-9161-6EF88E76B899}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="45">
   <si>
     <t>Set de datos:</t>
   </si>
@@ -53,12 +54,6 @@
     <t>popsize</t>
   </si>
   <si>
-    <t>n_particles</t>
-  </si>
-  <si>
-    <t>n_iter</t>
-  </si>
-  <si>
     <t>differential evolution</t>
   </si>
   <si>
@@ -107,9 +102,6 @@
     <t>Los métodos da y de en sus mejores versiones según lo evaluado con el set de datos anterior, no entrega buenos resultados.</t>
   </si>
   <si>
-    <t>Probé coon PSO de mealpy, se demora mucho y como que no funciona</t>
-  </si>
-  <si>
     <t>Data CS 24 AGROCAUQ estanque 68.xlsx</t>
   </si>
   <si>
@@ -123,18 +115,77 @@
   </si>
   <si>
     <t>Cambié C1 C2 y w</t>
+  </si>
+  <si>
+    <t>Probé con PSO de mealpy, se demora mucho y como que no funciona</t>
+  </si>
+  <si>
+    <t>en otros casos azúcar es de 20, y etanol de 0,4, por ejemplo</t>
+  </si>
+  <si>
+    <t>PSO mealpy</t>
+  </si>
+  <si>
+    <t>n_iter (epoch)</t>
+  </si>
+  <si>
+    <t>n_particles (pop_size)</t>
+  </si>
+  <si>
+    <t>PSO mealpy PSO.OriginalPSO</t>
+  </si>
+  <si>
+    <t>PSO mealpy PSO.HPSO_TVAC</t>
+  </si>
+  <si>
+    <t>PSO mealpy pso.originalpso</t>
+  </si>
+  <si>
+    <t>Tiempo (min)</t>
+  </si>
+  <si>
+    <t>Dual annealing funciona peor con esta función objetivo</t>
+  </si>
+  <si>
+    <t>con termination en it = 219</t>
+  </si>
+  <si>
+    <t>con termination en  it = 129</t>
+  </si>
+  <si>
+    <t>10000, eps = 1e-6</t>
+  </si>
+  <si>
+    <t>con termination en  it = 113</t>
+  </si>
+  <si>
+    <t>Set de datos</t>
+  </si>
+  <si>
+    <t>PROBAR CON C1 = 1,5, C2 = 1,5 y w = 0,7</t>
+  </si>
+  <si>
+    <t>10000, eps = 1e-7</t>
+  </si>
+  <si>
+    <t>Debe ser más exigente el criterio para cortar optimización</t>
+  </si>
+  <si>
+    <t>Mas de una hora corriendo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0.0000000"/>
     <numFmt numFmtId="165" formatCode="#,##0.00000000"/>
-    <numFmt numFmtId="170" formatCode="#,##0.000000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.000000"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="0.000000000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -157,8 +208,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -183,8 +240,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="19">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -440,11 +503,57 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -474,6 +583,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -495,7 +607,51 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -504,12 +660,31 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="168" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -525,6 +700,236 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>72762</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>52917</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>489480</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="CuadroTexto 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9CC596AA-74E9-D4D1-99B6-39E63ED29CE4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14294116" y="11396927"/>
+          <a:ext cx="4067968" cy="1627188"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100"/>
+            <a:t>Notas/observaciones:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100"/>
+            <a:t>-</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100" baseline="0"/>
+            <a:t> PSO es el que "mejor" ajusta en algunos, pero no en todos. </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100" baseline="0"/>
+            <a:t>- Cuando se obtiene un buen ajuste visual con un costo bajo (he visto casos con f.o. &lt;100), el costo de la función objetivo tiende a ser la mayoría de los datos de azúcares, es decir, el costo del etanol tiende a de entre 0 y 2, aprox. </a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>99219</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>145521</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>398730</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>13076</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A61F78B0-A91E-511D-596A-1165341536D1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14320573" y="13169636"/>
+          <a:ext cx="7602011" cy="800212"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>290375</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>32281</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>251647</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>52801</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="7" name="Entrada de lápiz 6">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8C01B987-261C-0388-EA04-D360A93B2B5D}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="16945896" y="13797229"/>
+            <a:ext cx="2395440" cy="20520"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="7" name="Entrada de lápiz 6">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8C01B987-261C-0388-EA04-D360A93B2B5D}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="16909896" y="13726470"/>
+              <a:ext cx="2467080" cy="161683"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/ink/ink1.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-17T12:47:28.692"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.2" units="cm"/>
+      <inkml:brushProperty name="height" value="0.4" units="cm"/>
+      <inkml:brushProperty name="color" value="#FFFC00"/>
+      <inkml:brushProperty name="tip" value="rectangle"/>
+      <inkml:brushProperty name="rasterOp" value="maskPen"/>
+      <inkml:brushProperty name="ignorePressure" value="1"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">6653 57,'-32'-1,"-51"-10,17 2,-560-26,-773 37,815-3,566 1</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2433.25">3364 21,'-152'0,"-797"14,383-9,337-6,83-9,-1 1,69 10,-15 0,-121-13,126 4,-134 6,104 4,-227-2,328 0</inkml:trace>
+</inkml:ink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -790,16 +1195,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:T83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.453125" customWidth="1"/>
     <col min="3" max="3" width="9.36328125" customWidth="1"/>
-    <col min="5" max="5" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.08984375" customWidth="1"/>
     <col min="10" max="10" width="9.90625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="52.7265625" customWidth="1"/>
   </cols>
@@ -809,60 +1215,60 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="32" t="s">
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="65" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="65" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="65" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="60" t="s">
+        <v>6</v>
+      </c>
+      <c r="L2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="L2" t="s">
-        <v>16</v>
-      </c>
     </row>
     <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="36"/>
+      <c r="B3" s="64"/>
       <c r="C3" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>5</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="38"/>
+      <c r="E3" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
+      <c r="J3" s="67"/>
       <c r="L3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B4" s="8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C4" s="9">
         <v>8</v>
@@ -873,7 +1279,7 @@
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
       <c r="G4" s="9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H4" s="10">
         <v>82.549381118790606</v>
@@ -885,7 +1291,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B5" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C5" s="2">
         <v>8</v>
@@ -896,7 +1302,7 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H5" s="3">
         <v>204.12437459632801</v>
@@ -908,7 +1314,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B6" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C6" s="2">
         <v>8</v>
@@ -919,7 +1325,7 @@
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H6" s="3">
         <v>538.65830215846302</v>
@@ -931,7 +1337,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B7" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C7" s="2">
         <v>14</v>
@@ -942,7 +1348,7 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H7" s="3">
         <v>81.804288393525695</v>
@@ -954,7 +1360,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B8" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C8" s="2">
         <v>14</v>
@@ -965,7 +1371,7 @@
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H8" s="3">
         <v>84.980454925729703</v>
@@ -977,7 +1383,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B9" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C9" s="2">
         <v>14</v>
@@ -988,7 +1394,7 @@
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H9" s="4">
         <v>55.270130124821399</v>
@@ -1000,7 +1406,7 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B10" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C10" s="2">
         <v>20</v>
@@ -1011,7 +1417,7 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H10" s="3">
         <v>81.842917511313502</v>
@@ -1024,7 +1430,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B11" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C11" s="2">
         <v>20</v>
@@ -1035,7 +1441,7 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H11" s="5">
         <v>63.049160766663</v>
@@ -1047,7 +1453,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B12" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C12" s="2">
         <v>20</v>
@@ -1058,7 +1464,7 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H12" s="3">
         <v>93.389411925614297</v>
@@ -1070,7 +1476,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B13" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C13" s="2">
         <v>8</v>
@@ -1081,7 +1487,7 @@
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H13" s="3">
         <v>82.549381118790606</v>
@@ -1095,7 +1501,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B14" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C14" s="2">
         <v>8</v>
@@ -1106,7 +1512,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H14" s="3">
         <v>204.12437459632801</v>
@@ -1120,7 +1526,7 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B15" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C15" s="2">
         <v>8</v>
@@ -1131,7 +1537,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H15" s="3">
         <v>538.65830215846302</v>
@@ -1145,7 +1551,7 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B16" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C16" s="2">
         <v>14</v>
@@ -1156,7 +1562,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H16" s="3">
         <v>81.804288393525695</v>
@@ -1170,7 +1576,7 @@
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B17" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C17" s="2">
         <v>14</v>
@@ -1181,7 +1587,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H17" s="3">
         <v>84.980454925729703</v>
@@ -1195,7 +1601,7 @@
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B18" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C18" s="2">
         <v>14</v>
@@ -1206,7 +1612,7 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H18" s="4">
         <v>55.270130124821399</v>
@@ -1220,7 +1626,7 @@
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B19" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C19" s="2">
         <v>20</v>
@@ -1231,7 +1637,7 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H19" s="3">
         <v>81.842917511313502</v>
@@ -1245,7 +1651,7 @@
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B20" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C20" s="2">
         <v>20</v>
@@ -1256,7 +1662,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H20" s="5">
         <v>63.049160766663</v>
@@ -1270,7 +1676,7 @@
     </row>
     <row r="21" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B21" s="22" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C21" s="23">
         <v>20</v>
@@ -1281,7 +1687,7 @@
       <c r="E21" s="23"/>
       <c r="F21" s="23"/>
       <c r="G21" s="23" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H21" s="21">
         <v>93.389411925614297</v>
@@ -1295,7 +1701,7 @@
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B22" s="8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C22" s="9">
         <v>10</v>
@@ -1304,7 +1710,7 @@
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
       <c r="G22" s="17" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H22" s="10">
         <v>59.072205394945499</v>
@@ -1316,7 +1722,7 @@
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B23" s="12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C23" s="2">
         <v>20</v>
@@ -1325,7 +1731,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H23" s="3">
         <v>59.072205394945499</v>
@@ -1337,7 +1743,7 @@
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B24" s="12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C24" s="2">
         <v>40</v>
@@ -1346,7 +1752,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
       <c r="G24" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H24" s="3">
         <v>59.072205394945499</v>
@@ -1358,7 +1764,7 @@
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B25" s="12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C25" s="2">
         <v>60</v>
@@ -1367,7 +1773,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
       <c r="G25" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H25" s="3">
         <v>59.072205394945499</v>
@@ -1379,7 +1785,7 @@
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B26" s="12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C26" s="2">
         <v>10</v>
@@ -1388,7 +1794,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
       <c r="G26" s="18" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H26" s="3">
         <v>59.072205394945499</v>
@@ -1402,7 +1808,7 @@
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B27" s="12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C27" s="2">
         <v>20</v>
@@ -1411,7 +1817,7 @@
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
       <c r="G27" s="18" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H27" s="3">
         <v>59.072205394945499</v>
@@ -1425,7 +1831,7 @@
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B28" s="12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C28" s="2">
         <v>40</v>
@@ -1434,7 +1840,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
       <c r="G28" s="18" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H28" s="3">
         <v>59.072205394945499</v>
@@ -1448,7 +1854,7 @@
     </row>
     <row r="29" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B29" s="22" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C29" s="23">
         <v>60</v>
@@ -1457,7 +1863,7 @@
       <c r="E29" s="23"/>
       <c r="F29" s="23"/>
       <c r="G29" s="25" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H29" s="21">
         <v>59.072205394945499</v>
@@ -1471,7 +1877,7 @@
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B30" s="8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
@@ -1482,7 +1888,7 @@
         <v>50</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H30" s="10">
         <v>76.496085191314805</v>
@@ -1494,7 +1900,7 @@
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B31" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -1505,7 +1911,7 @@
         <v>50</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H31" s="3">
         <v>34.156916731388499</v>
@@ -1517,7 +1923,7 @@
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B32" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -1528,7 +1934,7 @@
         <v>50</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H32" s="3">
         <v>21.866985737151001</v>
@@ -1540,7 +1946,7 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B33" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -1551,7 +1957,7 @@
         <v>50</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H33" s="3">
         <v>21.598196097453801</v>
@@ -1563,7 +1969,7 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B34" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -1574,7 +1980,7 @@
         <v>80</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H34" s="3">
         <v>68.838314256654002</v>
@@ -1586,7 +1992,7 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B35" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -1597,7 +2003,7 @@
         <v>80</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H35" s="3">
         <v>33.383979815760597</v>
@@ -1609,7 +2015,7 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B36" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -1620,7 +2026,7 @@
         <v>80</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H36" s="3">
         <v>21.115469552137299</v>
@@ -1632,7 +2038,7 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B37" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -1643,7 +2049,7 @@
         <v>80</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H37" s="3">
         <v>21.152551459206698</v>
@@ -1655,7 +2061,7 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B38" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -1666,7 +2072,7 @@
         <v>100</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H38" s="4">
         <v>21.096195547588302</v>
@@ -1678,7 +2084,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B39" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -1689,7 +2095,7 @@
         <v>150</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H39" s="3">
         <v>20.933555214239501</v>
@@ -1701,7 +2107,7 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B40" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -1712,7 +2118,7 @@
         <v>80</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H40" s="3">
         <v>21.152551459206698</v>
@@ -1726,7 +2132,7 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B41" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -1737,7 +2143,7 @@
         <v>100</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H41" s="4">
         <v>21.096195547588302</v>
@@ -1749,185 +2155,160 @@
         <v>35.68</v>
       </c>
       <c r="L41" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B42" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B42" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C42" s="23"/>
+      <c r="D42" s="23"/>
+      <c r="E42" s="23">
         <v>25</v>
       </c>
-      <c r="F42" s="6">
+      <c r="F42" s="23">
         <v>150</v>
       </c>
-      <c r="G42" s="6" t="s">
+      <c r="G42" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="H42" s="21">
+        <v>20.933555214239501</v>
+      </c>
+      <c r="I42" s="21">
+        <v>20.913852644711</v>
+      </c>
+      <c r="J42" s="24">
+        <v>63.56</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B43" s="42" t="s">
+        <v>31</v>
+      </c>
+      <c r="C43" s="43"/>
+      <c r="D43" s="43"/>
+      <c r="E43" s="43">
         <v>10</v>
       </c>
-      <c r="H42" s="14">
-        <v>20.933555214239501</v>
-      </c>
-      <c r="I42" s="14">
-        <v>20.913852644711</v>
-      </c>
-      <c r="J42" s="27">
-        <v>63.56</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A45" t="s">
+      <c r="F43" s="43">
+        <v>500</v>
+      </c>
+      <c r="G43" s="43" t="s">
+        <v>7</v>
+      </c>
+      <c r="H43" s="44">
+        <v>14.1130851162229</v>
+      </c>
+      <c r="I43" s="43"/>
+      <c r="J43" s="45">
+        <f>2*60+57.83</f>
+        <v>177.82999999999998</v>
+      </c>
+      <c r="K43">
+        <f>J43/60</f>
+        <v>2.9638333333333331</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B44" s="48" t="s">
+        <v>32</v>
+      </c>
+      <c r="E44" s="49">
+        <v>10</v>
+      </c>
+      <c r="F44" s="49">
+        <v>500</v>
+      </c>
+      <c r="G44" s="43" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A48" t="s">
         <v>0</v>
       </c>
-      <c r="B45" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B46" s="29" t="s">
+      <c r="B48" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" spans="2:20" ht="29" x14ac:dyDescent="0.35">
+      <c r="B49" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="C46" s="31" t="s">
+      <c r="C49" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="D46" s="31"/>
-      <c r="E46" s="31"/>
-      <c r="F46" s="31"/>
-      <c r="G46" s="32" t="s">
-        <v>14</v>
-      </c>
-      <c r="H46" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="I46" s="32" t="s">
+      <c r="D49" s="34"/>
+      <c r="E49" s="34"/>
+      <c r="F49" s="34"/>
+      <c r="G49" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="J46" s="34" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B47" s="30"/>
-      <c r="C47" s="7" t="s">
+      <c r="H49" s="35" t="s">
+        <v>9</v>
+      </c>
+      <c r="I49" s="35" t="s">
+        <v>10</v>
+      </c>
+      <c r="J49" s="37" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B50" s="33"/>
+      <c r="C50" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D47" s="7" t="s">
+      <c r="D50" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E47" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="F47" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="G47" s="33"/>
-      <c r="H47" s="33"/>
-      <c r="I47" s="33"/>
-      <c r="J47" s="35"/>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B48" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="2">
+      <c r="E50" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G50" s="36"/>
+      <c r="H50" s="36"/>
+      <c r="I50" s="36"/>
+      <c r="J50" s="38"/>
+    </row>
+    <row r="51" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B51" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="39">
         <v>25</v>
       </c>
-      <c r="F48" s="2">
-        <v>50</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H48" s="28">
-        <v>39.402122681394601</v>
-      </c>
-      <c r="I48" s="2"/>
-      <c r="J48" s="2">
-        <v>48.38</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B49" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2">
-        <v>25</v>
-      </c>
-      <c r="F49" s="2">
-        <v>80</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H49" s="28">
-        <v>26.1017589545019</v>
-      </c>
-      <c r="I49" s="2"/>
-      <c r="J49" s="2">
-        <f>60+17.06</f>
-        <v>77.06</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B50" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2">
-        <v>25</v>
-      </c>
-      <c r="F50" s="2">
+      <c r="F51" s="39">
         <v>100</v>
       </c>
-      <c r="G50" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H50" s="39">
-        <v>26.036020305426099</v>
-      </c>
-      <c r="I50" s="2"/>
-      <c r="J50" s="2">
-        <f>60+32.74</f>
-        <v>92.740000000000009</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B51" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2">
-        <v>25</v>
-      </c>
-      <c r="F51" s="2">
-        <v>120</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H51" s="28">
-        <v>26.036020305426099</v>
-      </c>
-      <c r="I51" s="2"/>
-      <c r="J51" s="2">
-        <f>60+52.17</f>
-        <v>112.17</v>
+      <c r="G51" s="39" t="s">
+        <v>7</v>
+      </c>
+      <c r="H51" s="40">
+        <v>642.85640012476097</v>
+      </c>
+      <c r="I51" s="9"/>
+      <c r="J51" s="11">
+        <f>2*60+14.52</f>
+        <v>134.52000000000001</v>
+      </c>
+      <c r="K51" s="41">
+        <f>J51/60</f>
+        <v>2.242</v>
       </c>
       <c r="L51" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B52" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="52" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B52" s="12" t="s">
+        <v>16</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
@@ -1935,25 +2316,30 @@
         <v>25</v>
       </c>
       <c r="F52" s="2">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H52" s="28">
-        <v>26.1017589545019</v>
-      </c>
-      <c r="I52" s="3">
-        <v>26.1014646021309</v>
-      </c>
-      <c r="J52" s="2">
-        <f>60+13.62</f>
-        <v>73.62</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B53" s="2" t="s">
-        <v>18</v>
+        <v>7</v>
+      </c>
+      <c r="H52" s="29">
+        <v>642.66116140171596</v>
+      </c>
+      <c r="I52" s="2"/>
+      <c r="J52" s="13">
+        <f>2*60+21.53</f>
+        <v>141.53</v>
+      </c>
+      <c r="K52" s="41">
+        <f t="shared" ref="K52:K60" si="0">J52/60</f>
+        <v>2.3588333333333336</v>
+      </c>
+      <c r="L52" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="53" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B53" s="12" t="s">
+        <v>16</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
@@ -1961,398 +2347,1640 @@
         <v>25</v>
       </c>
       <c r="F53" s="2">
+        <v>150</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H53" s="29">
+        <v>642.66116140171596</v>
+      </c>
+      <c r="I53" s="2"/>
+      <c r="J53" s="13">
+        <f>2*60+41.42</f>
+        <v>161.42000000000002</v>
+      </c>
+      <c r="K53" s="41">
+        <f t="shared" si="0"/>
+        <v>2.6903333333333337</v>
+      </c>
+    </row>
+    <row r="54" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B54" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2">
+        <v>25</v>
+      </c>
+      <c r="F54" s="2">
+        <v>150</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H54" s="29">
+        <v>642.66116140171596</v>
+      </c>
+      <c r="I54" s="30">
+        <v>642.92712592794396</v>
+      </c>
+      <c r="J54" s="13">
+        <f>2*60+40.53</f>
+        <v>160.53</v>
+      </c>
+      <c r="K54" s="41">
+        <f t="shared" si="0"/>
+        <v>2.6755</v>
+      </c>
+      <c r="L54" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="55" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B55" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2">
+        <v>30</v>
+      </c>
+      <c r="F55" s="2">
+        <v>150</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H55" s="28">
+        <v>376.02775723511297</v>
+      </c>
+      <c r="I55" s="2"/>
+      <c r="J55" s="13">
+        <f>60+36.33</f>
+        <v>96.33</v>
+      </c>
+      <c r="K55" s="41">
+        <f t="shared" si="0"/>
+        <v>1.6054999999999999</v>
+      </c>
+    </row>
+    <row r="56" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B56" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2">
+        <v>30</v>
+      </c>
+      <c r="F56" s="2">
+        <v>200</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H56" s="28">
+        <v>375.67459265584</v>
+      </c>
+      <c r="I56" s="2"/>
+      <c r="J56" s="13">
+        <f>60+50.99</f>
+        <v>110.99000000000001</v>
+      </c>
+      <c r="K56" s="41">
+        <f t="shared" si="0"/>
+        <v>1.8498333333333334</v>
+      </c>
+    </row>
+    <row r="57" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B57" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2">
+        <v>35</v>
+      </c>
+      <c r="F57" s="2">
+        <v>200</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H57" s="28">
+        <v>642.68328820100896</v>
+      </c>
+      <c r="I57" s="2"/>
+      <c r="J57" s="13">
+        <f>5*60+13.72</f>
+        <v>313.72000000000003</v>
+      </c>
+      <c r="K57" s="41">
+        <f t="shared" si="0"/>
+        <v>5.2286666666666672</v>
+      </c>
+    </row>
+    <row r="58" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B58" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="31">
+        <v>25</v>
+      </c>
+      <c r="F58" s="31">
         <v>100</v>
       </c>
-      <c r="G53" s="2" t="s">
+      <c r="G58" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="H58" s="28">
+        <v>642.65825516787504</v>
+      </c>
+      <c r="I58" s="2"/>
+      <c r="J58" s="13">
+        <f>5*60+38.17</f>
+        <v>338.17</v>
+      </c>
+      <c r="K58" s="41">
+        <f t="shared" si="0"/>
+        <v>5.636166666666667</v>
+      </c>
+      <c r="L58" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="59" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B59" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2">
+        <v>25</v>
+      </c>
+      <c r="F59" s="2">
+        <v>500</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H59" s="28">
+        <v>642.48339335654896</v>
+      </c>
+      <c r="I59" s="2"/>
+      <c r="J59" s="13">
+        <f>16*60+24.41</f>
+        <v>984.41</v>
+      </c>
+      <c r="K59" s="41">
+        <f t="shared" si="0"/>
+        <v>16.406833333333331</v>
+      </c>
+    </row>
+    <row r="60" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B60" s="42" t="s">
+        <v>28</v>
+      </c>
+      <c r="C60" s="43"/>
+      <c r="D60" s="43"/>
+      <c r="E60" s="43">
         <v>10</v>
       </c>
-      <c r="H53" s="39">
+      <c r="F60" s="43">
+        <v>500</v>
+      </c>
+      <c r="G60" s="43" t="s">
+        <v>7</v>
+      </c>
+      <c r="H60" s="46">
+        <v>98.115554496124503</v>
+      </c>
+      <c r="I60" s="43"/>
+      <c r="J60" s="45">
+        <f>16*60+20.41</f>
+        <v>980.41</v>
+      </c>
+      <c r="K60" s="41">
+        <f t="shared" si="0"/>
+        <v>16.340166666666665</v>
+      </c>
+    </row>
+    <row r="61" spans="2:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B61" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C61" s="9">
+        <v>10</v>
+      </c>
+      <c r="D61" s="9"/>
+      <c r="E61" s="9"/>
+      <c r="F61" s="9"/>
+      <c r="G61" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H61" s="10">
+        <v>1627.2112119826199</v>
+      </c>
+      <c r="I61" s="10"/>
+      <c r="J61" s="11">
+        <f>60+18.43</f>
+        <v>78.430000000000007</v>
+      </c>
+      <c r="K61" s="41">
+        <f t="shared" ref="K61:K67" si="1">J61/60</f>
+        <v>1.3071666666666668</v>
+      </c>
+    </row>
+    <row r="62" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B62" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C62" s="2">
+        <v>20</v>
+      </c>
+      <c r="D62" s="2"/>
+      <c r="E62" s="2"/>
+      <c r="F62" s="2"/>
+      <c r="G62" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H62" s="3">
+        <v>270.86726147910599</v>
+      </c>
+      <c r="I62" s="3"/>
+      <c r="J62" s="13">
+        <f>4*60+16</f>
+        <v>256</v>
+      </c>
+      <c r="K62" s="41">
+        <f t="shared" si="1"/>
+        <v>4.2666666666666666</v>
+      </c>
+    </row>
+    <row r="63" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B63" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C63" s="2">
+        <v>40</v>
+      </c>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2"/>
+      <c r="F63" s="2"/>
+      <c r="G63" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H63" s="4">
+        <v>80.891270066865701</v>
+      </c>
+      <c r="I63" s="3"/>
+      <c r="J63" s="13">
+        <f>6*60+32.9</f>
+        <v>392.9</v>
+      </c>
+      <c r="K63" s="41">
+        <f t="shared" si="1"/>
+        <v>6.5483333333333329</v>
+      </c>
+    </row>
+    <row r="64" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B64" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C64" s="6">
+        <v>60</v>
+      </c>
+      <c r="D64" s="6"/>
+      <c r="E64" s="6"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="H64" s="47">
+        <v>80.891270066865701</v>
+      </c>
+      <c r="I64" s="14"/>
+      <c r="J64" s="27">
+        <f>8*60+48.35</f>
+        <v>528.35</v>
+      </c>
+      <c r="K64" s="41">
+        <f t="shared" si="1"/>
+        <v>8.8058333333333341</v>
+      </c>
+      <c r="T64" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B65" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C65" s="9">
+        <v>14</v>
+      </c>
+      <c r="D65" s="9">
+        <v>8</v>
+      </c>
+      <c r="E65" s="9"/>
+      <c r="F65" s="9"/>
+      <c r="G65" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H65" s="10">
+        <v>778.393043419641</v>
+      </c>
+      <c r="I65" s="9"/>
+      <c r="J65" s="11">
+        <f>60+33.35</f>
+        <v>93.35</v>
+      </c>
+      <c r="K65" s="41">
+        <f t="shared" si="1"/>
+        <v>1.5558333333333332</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B66" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C66" s="2">
+        <v>20</v>
+      </c>
+      <c r="D66" s="2">
+        <v>6</v>
+      </c>
+      <c r="E66" s="2"/>
+      <c r="F66" s="2"/>
+      <c r="G66" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H66" s="3">
+        <v>631.09160994058198</v>
+      </c>
+      <c r="I66" s="2"/>
+      <c r="J66" s="13">
+        <f>60+13.3</f>
+        <v>73.3</v>
+      </c>
+      <c r="K66" s="41">
+        <f t="shared" si="1"/>
+        <v>1.2216666666666667</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B67" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C67" s="6">
+        <v>20</v>
+      </c>
+      <c r="D67" s="6">
+        <v>8</v>
+      </c>
+      <c r="E67" s="6"/>
+      <c r="F67" s="6"/>
+      <c r="G67" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="H67" s="14">
+        <v>537.62630440488795</v>
+      </c>
+      <c r="I67" s="6"/>
+      <c r="J67" s="27">
+        <f>2*60+25.47</f>
+        <v>145.47</v>
+      </c>
+      <c r="K67" s="41">
+        <f t="shared" si="1"/>
+        <v>2.4245000000000001</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A70" t="s">
+        <v>0</v>
+      </c>
+      <c r="B70" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B71" s="63" t="s">
+        <v>1</v>
+      </c>
+      <c r="C71" s="62" t="s">
+        <v>2</v>
+      </c>
+      <c r="D71" s="62"/>
+      <c r="E71" s="62"/>
+      <c r="F71" s="62"/>
+      <c r="G71" s="65" t="s">
+        <v>12</v>
+      </c>
+      <c r="H71" s="65" t="s">
+        <v>9</v>
+      </c>
+      <c r="I71" s="65" t="s">
+        <v>10</v>
+      </c>
+      <c r="J71" s="60" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B72" s="68"/>
+      <c r="C72" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D72" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E72" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F72" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G72" s="69"/>
+      <c r="H72" s="69"/>
+      <c r="I72" s="69"/>
+      <c r="J72" s="61"/>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B73" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C73" s="9"/>
+      <c r="D73" s="9"/>
+      <c r="E73" s="9">
+        <v>25</v>
+      </c>
+      <c r="F73" s="9">
+        <v>50</v>
+      </c>
+      <c r="G73" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H73" s="40">
+        <v>39.402122681394601</v>
+      </c>
+      <c r="I73" s="9"/>
+      <c r="J73" s="11">
+        <v>48.38</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B74" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C74" s="2"/>
+      <c r="D74" s="2"/>
+      <c r="E74" s="2">
+        <v>25</v>
+      </c>
+      <c r="F74" s="2">
+        <v>80</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H74" s="28">
+        <v>26.1017589545019</v>
+      </c>
+      <c r="I74" s="2"/>
+      <c r="J74" s="13">
+        <f>60+17.06</f>
+        <v>77.06</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B75" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C75" s="2"/>
+      <c r="D75" s="2"/>
+      <c r="E75" s="2">
+        <v>25</v>
+      </c>
+      <c r="F75" s="2">
+        <v>100</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H75" s="29">
         <v>26.036020305426099</v>
       </c>
-      <c r="I53" s="4">
+      <c r="I75" s="2"/>
+      <c r="J75" s="13">
+        <f>60+32.74</f>
+        <v>92.740000000000009</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B76" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C76" s="2"/>
+      <c r="D76" s="2"/>
+      <c r="E76" s="2">
+        <v>25</v>
+      </c>
+      <c r="F76" s="2">
+        <v>120</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H76" s="28">
+        <v>26.036020305426099</v>
+      </c>
+      <c r="I76" s="2"/>
+      <c r="J76" s="13">
+        <f>60+52.17</f>
+        <v>112.17</v>
+      </c>
+      <c r="L76" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B77" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C77" s="2"/>
+      <c r="D77" s="2"/>
+      <c r="E77" s="2">
+        <v>25</v>
+      </c>
+      <c r="F77" s="2">
+        <v>80</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H77" s="28">
+        <v>26.1017589545019</v>
+      </c>
+      <c r="I77" s="3">
+        <v>26.1014646021309</v>
+      </c>
+      <c r="J77" s="13">
+        <f>60+13.62</f>
+        <v>73.62</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B78" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C78" s="2"/>
+      <c r="D78" s="2"/>
+      <c r="E78" s="2">
+        <v>25</v>
+      </c>
+      <c r="F78" s="2">
+        <v>100</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H78" s="29">
+        <v>26.036020305426099</v>
+      </c>
+      <c r="I78" s="4">
         <v>26.028892560451698</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J78" s="13">
         <f>60+33.08</f>
         <v>93.08</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B57" t="s">
-        <v>22</v>
-      </c>
-      <c r="K57" s="1"/>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B58" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B60" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B61" s="29" t="s">
-        <v>1</v>
-      </c>
-      <c r="C61" s="31" t="s">
-        <v>2</v>
-      </c>
-      <c r="D61" s="31"/>
-      <c r="E61" s="31"/>
-      <c r="F61" s="31"/>
-      <c r="G61" s="32" t="s">
-        <v>14</v>
-      </c>
-      <c r="H61" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="I61" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="J61" s="34" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B62" s="30"/>
-      <c r="C62" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="D62" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="E62" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="F62" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="G62" s="33"/>
-      <c r="H62" s="33"/>
-      <c r="I62" s="33"/>
-      <c r="J62" s="35"/>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B63" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C63" s="2"/>
-      <c r="D63" s="2"/>
-      <c r="E63" s="44">
-        <v>25</v>
-      </c>
-      <c r="F63" s="44">
-        <v>100</v>
-      </c>
-      <c r="G63" s="44" t="s">
-        <v>9</v>
-      </c>
-      <c r="H63" s="40">
-        <v>642.85640012476097</v>
-      </c>
-      <c r="I63" s="2"/>
-      <c r="J63" s="2">
-        <f>2*60+14.52</f>
-        <v>134.52000000000001</v>
-      </c>
-      <c r="L63" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B64" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
-      <c r="E64" s="2">
-        <v>25</v>
-      </c>
-      <c r="F64" s="2">
-        <v>120</v>
-      </c>
-      <c r="G64" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H64" s="39">
-        <v>642.66116140171596</v>
-      </c>
-      <c r="I64" s="2"/>
-      <c r="J64" s="2">
-        <f>2*60+21.53</f>
-        <v>141.53</v>
-      </c>
-      <c r="L64" t="s">
+    <row r="79" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B79" s="42" t="s">
+        <v>28</v>
+      </c>
+      <c r="C79" s="43"/>
+      <c r="D79" s="43"/>
+      <c r="E79" s="43">
+        <v>10</v>
+      </c>
+      <c r="F79" s="43">
+        <v>500</v>
+      </c>
+      <c r="G79" s="43" t="s">
+        <v>7</v>
+      </c>
+      <c r="H79" s="46">
+        <v>45.923361985594603</v>
+      </c>
+      <c r="I79" s="43"/>
+      <c r="J79" s="45">
+        <f>13*60+9.75</f>
+        <v>789.75</v>
+      </c>
+      <c r="K79">
+        <f>J79/60</f>
+        <v>13.1625</v>
+      </c>
+    </row>
+    <row r="82" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B82" t="s">
+        <v>20</v>
+      </c>
+      <c r="K82" s="1"/>
+    </row>
+    <row r="83" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B83" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B65" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2">
-        <v>25</v>
-      </c>
-      <c r="F65" s="2">
-        <v>150</v>
-      </c>
-      <c r="G65" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H65" s="39">
-        <v>642.66116140171596</v>
-      </c>
-      <c r="I65" s="2"/>
-      <c r="J65" s="2">
-        <f>2*60+41.42</f>
-        <v>161.42000000000002</v>
-      </c>
-    </row>
-    <row r="66" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B66" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
-      <c r="E66" s="2">
-        <v>25</v>
-      </c>
-      <c r="F66" s="2">
-        <v>150</v>
-      </c>
-      <c r="G66" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="H66" s="39">
-        <v>642.66116140171596</v>
-      </c>
-      <c r="I66" s="42">
-        <v>642.92712592794396</v>
-      </c>
-      <c r="J66" s="2">
-        <f>2*60+40.53</f>
-        <v>160.53</v>
-      </c>
-      <c r="L66" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="67" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B67" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-      <c r="E67" s="2">
-        <v>30</v>
-      </c>
-      <c r="F67" s="2">
-        <v>150</v>
-      </c>
-      <c r="G67" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H67" s="40">
-        <v>376.02775723511297</v>
-      </c>
-      <c r="I67" s="2"/>
-      <c r="J67" s="2">
-        <f>60+36.33</f>
-        <v>96.33</v>
-      </c>
-    </row>
-    <row r="68" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B68" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2"/>
-      <c r="E68" s="41">
-        <v>30</v>
-      </c>
-      <c r="F68" s="41">
-        <v>200</v>
-      </c>
-      <c r="G68" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H68" s="28">
-        <v>375.67459265584</v>
-      </c>
-      <c r="I68" s="2"/>
-      <c r="J68" s="2">
-        <f>60+50.99</f>
-        <v>110.99000000000001</v>
-      </c>
-    </row>
-    <row r="69" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B69" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2">
-        <v>35</v>
-      </c>
-      <c r="F69" s="2">
-        <v>200</v>
-      </c>
-      <c r="G69" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H69" s="28">
-        <v>642.68328820100896</v>
-      </c>
-      <c r="I69" s="2"/>
-      <c r="J69" s="2">
-        <f>5*60+13.72</f>
-        <v>313.72000000000003</v>
-      </c>
-    </row>
-    <row r="70" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B70" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
-      <c r="E70" s="43">
-        <v>25</v>
-      </c>
-      <c r="F70" s="43">
-        <v>100</v>
-      </c>
-      <c r="G70" s="44" t="s">
-        <v>9</v>
-      </c>
-      <c r="H70" s="28">
-        <v>642.65825516787504</v>
-      </c>
-      <c r="I70" s="2"/>
-      <c r="J70" s="2">
-        <f>5*60+38.17</f>
-        <v>338.17</v>
-      </c>
-      <c r="L70" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="72" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="73" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B73" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C73" s="9">
-        <v>10</v>
-      </c>
-      <c r="D73" s="9"/>
-      <c r="E73" s="9"/>
-      <c r="F73" s="9"/>
-      <c r="G73" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="H73" s="10">
-        <v>1627.2112119826199</v>
-      </c>
-      <c r="I73" s="10"/>
-      <c r="J73" s="11">
-        <f>60+18.43</f>
-        <v>78.430000000000007</v>
-      </c>
-    </row>
-    <row r="74" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B74" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C74" s="2">
-        <v>20</v>
-      </c>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
-      <c r="F74" s="2"/>
-      <c r="G74" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H74" s="3">
-        <v>270.86726147910599</v>
-      </c>
-      <c r="I74" s="3"/>
-      <c r="J74" s="13">
-        <f>4*60+16</f>
-        <v>256</v>
-      </c>
-    </row>
-    <row r="75" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B75" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C75" s="2">
-        <v>40</v>
-      </c>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
-      <c r="F75" s="2"/>
-      <c r="G75" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H75" s="3">
-        <v>80.891270066865701</v>
-      </c>
-      <c r="I75" s="3"/>
-      <c r="J75" s="13">
-        <f>6*60+32.9</f>
-        <v>392.9</v>
-      </c>
-    </row>
-    <row r="76" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B76" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C76" s="6">
-        <v>60</v>
-      </c>
-      <c r="D76" s="6"/>
-      <c r="E76" s="6"/>
-      <c r="F76" s="6"/>
-      <c r="G76" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H76" s="14">
-        <v>80.891270066865701</v>
-      </c>
-      <c r="I76" s="14"/>
-      <c r="J76" s="27">
-        <f>8*60+48.35</f>
-        <v>528.35</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="C61:F61"/>
-    <mergeCell ref="G61:G62"/>
-    <mergeCell ref="H61:H62"/>
-    <mergeCell ref="I61:I62"/>
-    <mergeCell ref="J61:J62"/>
-    <mergeCell ref="J46:J47"/>
+  <mergeCells count="12">
+    <mergeCell ref="J71:J72"/>
     <mergeCell ref="C2:F2"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="I2:I3"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:F46"/>
-    <mergeCell ref="G46:G47"/>
-    <mergeCell ref="H46:H47"/>
-    <mergeCell ref="I46:I47"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="C71:F71"/>
+    <mergeCell ref="G71:G72"/>
+    <mergeCell ref="H71:H72"/>
+    <mergeCell ref="I71:I72"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C75CEB36-15CC-49A5-922D-23CCF4F0347B}">
+  <dimension ref="A1:W46"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.7265625" customWidth="1"/>
+    <col min="5" max="5" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.36328125" customWidth="1"/>
+    <col min="7" max="7" width="16.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="14" max="14" width="38.08984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.08984375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B2" s="57" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="57" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="57" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="57" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" s="57" t="s">
+        <v>40</v>
+      </c>
+      <c r="O2" s="77" t="s">
+        <v>1</v>
+      </c>
+      <c r="P2" s="74" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="75"/>
+      <c r="R2" s="75"/>
+      <c r="S2" s="76"/>
+      <c r="T2" s="69" t="s">
+        <v>9</v>
+      </c>
+      <c r="U2" s="69" t="s">
+        <v>6</v>
+      </c>
+      <c r="V2" s="69" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B3" s="57"/>
+      <c r="C3" s="50" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="77"/>
+      <c r="P3" s="50" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q3" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="R3" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="S3" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="T3" s="73"/>
+      <c r="U3" s="73"/>
+      <c r="V3" s="73"/>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2">
+        <v>150</v>
+      </c>
+      <c r="G4" s="54">
+        <v>3.54059150007205E-4</v>
+      </c>
+      <c r="H4" s="2">
+        <f>60+18.28</f>
+        <v>78.28</v>
+      </c>
+      <c r="I4" s="51">
+        <f>H4/60</f>
+        <v>1.3046666666666666</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2">
+        <v>25</v>
+      </c>
+      <c r="S4" s="2">
+        <v>200</v>
+      </c>
+      <c r="T4" s="54">
+        <f>G5</f>
+        <v>3.5386864122503397E-4</v>
+      </c>
+      <c r="U4" s="2">
+        <f t="shared" ref="U4:V6" si="0">H5</f>
+        <v>84.3</v>
+      </c>
+      <c r="V4" s="2">
+        <f t="shared" si="0"/>
+        <v>1.405</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2">
+        <v>25</v>
+      </c>
+      <c r="F5" s="2">
+        <v>200</v>
+      </c>
+      <c r="G5" s="54">
+        <v>3.5386864122503397E-4</v>
+      </c>
+      <c r="H5" s="2">
+        <f>60+24.3</f>
+        <v>84.3</v>
+      </c>
+      <c r="I5" s="51">
+        <f t="shared" ref="I5:I9" si="1">H5/60</f>
+        <v>1.405</v>
+      </c>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2">
+        <v>25</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T5" s="2">
+        <v>1.3251362658287199E-3</v>
+      </c>
+      <c r="U5" s="2">
+        <f>6*60+41.95</f>
+        <v>401.95</v>
+      </c>
+      <c r="V5" s="51">
+        <f>U5/60</f>
+        <v>6.6991666666666667</v>
+      </c>
+      <c r="W5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="51">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2">
+        <v>25</v>
+      </c>
+      <c r="F7" s="2">
+        <v>150</v>
+      </c>
+      <c r="G7" s="2">
+        <v>7.47298733256553E-4</v>
+      </c>
+      <c r="H7" s="2">
+        <f>60+39.4</f>
+        <v>99.4</v>
+      </c>
+      <c r="I7" s="51">
+        <f t="shared" si="1"/>
+        <v>1.6566666666666667</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2">
+        <v>25</v>
+      </c>
+      <c r="S7" s="2">
+        <v>500</v>
+      </c>
+      <c r="T7" s="54">
+        <f>G25</f>
+        <v>1.10137530548398E-2</v>
+      </c>
+      <c r="U7" s="2">
+        <f t="shared" ref="U7:V7" si="2">H25</f>
+        <v>983.38</v>
+      </c>
+      <c r="V7" s="78">
+        <f t="shared" si="2"/>
+        <v>16.389666666666667</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2">
+        <v>25</v>
+      </c>
+      <c r="F8" s="2">
+        <v>200</v>
+      </c>
+      <c r="G8" s="2">
+        <v>7.4539462925004598E-4</v>
+      </c>
+      <c r="H8" s="2">
+        <f>60*2+16.43</f>
+        <v>136.43</v>
+      </c>
+      <c r="I8" s="51">
+        <f t="shared" si="1"/>
+        <v>2.2738333333333336</v>
+      </c>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="2"/>
+      <c r="W8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2">
+        <v>20</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G9" s="56">
+        <v>7.1734287866433903E-4</v>
+      </c>
+      <c r="H9" s="2">
+        <f>4*60+58.9</f>
+        <v>298.89999999999998</v>
+      </c>
+      <c r="I9" s="51">
+        <f t="shared" si="1"/>
+        <v>4.9816666666666665</v>
+      </c>
+      <c r="J9" s="55" t="s">
+        <v>39</v>
+      </c>
+      <c r="K9" s="55"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="2"/>
+      <c r="T9" s="2"/>
+      <c r="U9" s="2"/>
+      <c r="V9" s="2"/>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="2">
+        <v>14</v>
+      </c>
+      <c r="D10" s="2">
+        <v>8</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2">
+        <v>1.0140708323287399E-3</v>
+      </c>
+      <c r="H10" s="2">
+        <v>23.59</v>
+      </c>
+      <c r="I10" s="51">
+        <f>H10/60</f>
+        <v>0.39316666666666666</v>
+      </c>
+      <c r="J10" s="71"/>
+      <c r="K10" s="71"/>
+      <c r="N10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2">
+        <v>25</v>
+      </c>
+      <c r="S10" s="2">
+        <v>200</v>
+      </c>
+      <c r="T10" s="54">
+        <f>G43</f>
+        <v>4.96373772906626E-4</v>
+      </c>
+      <c r="U10" s="2">
+        <f t="shared" ref="U10:V10" si="3">H43</f>
+        <v>297.94</v>
+      </c>
+      <c r="V10" s="51">
+        <f t="shared" si="3"/>
+        <v>4.9656666666666665</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="2">
+        <v>20</v>
+      </c>
+      <c r="D11" s="2">
+        <v>8</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2">
+        <v>2.6214962503612101E-3</v>
+      </c>
+      <c r="H11" s="2">
+        <v>35.130000000000003</v>
+      </c>
+      <c r="I11" s="51">
+        <f>H11/60</f>
+        <v>0.58550000000000002</v>
+      </c>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
+      <c r="S11" s="2"/>
+      <c r="T11" s="2"/>
+      <c r="U11" s="2"/>
+      <c r="V11" s="2"/>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="2">
+        <v>50</v>
+      </c>
+      <c r="D12" s="2">
+        <v>10</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2">
+        <v>7.2968812345856502E-4</v>
+      </c>
+      <c r="H12" s="2">
+        <f>60+39.66</f>
+        <v>99.66</v>
+      </c>
+      <c r="I12" s="51">
+        <f>H12/60</f>
+        <v>1.661</v>
+      </c>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
+      <c r="S12" s="2"/>
+      <c r="T12" s="2"/>
+      <c r="U12" s="2"/>
+      <c r="V12" s="2"/>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="2">
+        <v>20</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2">
+        <v>2.9707312987521901E-2</v>
+      </c>
+      <c r="H13" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="I13" s="51">
+        <f>H13/60</f>
+        <v>0.39833333333333332</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2">
+        <v>50</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2">
+        <v>3.2673059442356002E-3</v>
+      </c>
+      <c r="H14" s="2">
+        <v>50.34</v>
+      </c>
+      <c r="I14" s="51">
+        <f>H14/60</f>
+        <v>0.83900000000000008</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="G16">
+        <f>MIN(G4:G14)</f>
+        <v>3.5386864122503397E-4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B21" s="57" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="58" t="s">
+        <v>2</v>
+      </c>
+      <c r="D21" s="58"/>
+      <c r="E21" s="58"/>
+      <c r="F21" s="58"/>
+      <c r="G21" s="57" t="s">
+        <v>9</v>
+      </c>
+      <c r="H21" s="57" t="s">
+        <v>6</v>
+      </c>
+      <c r="I21" s="57" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B22" s="57"/>
+      <c r="C22" s="50" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E22" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F22" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="G22" s="57"/>
+      <c r="H22" s="57"/>
+      <c r="I22" s="57"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2">
+        <v>25</v>
+      </c>
+      <c r="F23" s="2">
+        <v>150</v>
+      </c>
+      <c r="G23" s="72">
+        <v>1.10227895476947E-2</v>
+      </c>
+      <c r="H23" s="18">
+        <f>3*60+59.05</f>
+        <v>239.05</v>
+      </c>
+      <c r="I23" s="51">
+        <f t="shared" ref="I23:I25" si="4">H23/60</f>
+        <v>3.9841666666666669</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2">
+        <v>25</v>
+      </c>
+      <c r="F24" s="2">
+        <v>200</v>
+      </c>
+      <c r="G24" s="54">
+        <v>1.1022084456943E-2</v>
+      </c>
+      <c r="H24" s="18">
+        <f>5*60+36.45</f>
+        <v>336.45</v>
+      </c>
+      <c r="I24" s="51">
+        <f t="shared" si="4"/>
+        <v>5.6074999999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2">
+        <v>25</v>
+      </c>
+      <c r="F25" s="2">
+        <v>500</v>
+      </c>
+      <c r="G25" s="54">
+        <v>1.10137530548398E-2</v>
+      </c>
+      <c r="H25" s="2">
+        <f>16*60+23.38</f>
+        <v>983.38</v>
+      </c>
+      <c r="I25" s="51">
+        <f t="shared" si="4"/>
+        <v>16.389666666666667</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B27" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="C27" s="52"/>
+      <c r="D27" s="52"/>
+      <c r="E27" s="52">
+        <v>25</v>
+      </c>
+      <c r="F27" s="52">
+        <v>150</v>
+      </c>
+      <c r="G27" s="52">
+        <v>5.0054474380338103E-2</v>
+      </c>
+      <c r="H27" s="52">
+        <f>2*60+57.09</f>
+        <v>177.09</v>
+      </c>
+      <c r="I27" s="53">
+        <f>H27/60</f>
+        <v>2.9515000000000002</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B28" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="52"/>
+      <c r="D28" s="52"/>
+      <c r="E28" s="52">
+        <v>25</v>
+      </c>
+      <c r="F28" s="52">
+        <v>200</v>
+      </c>
+      <c r="G28" s="52">
+        <v>8.3019029328971292E-3</v>
+      </c>
+      <c r="H28" s="52">
+        <f>4*60+16.62</f>
+        <v>256.62</v>
+      </c>
+      <c r="I28" s="53">
+        <f>H28/60</f>
+        <v>4.2770000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B29" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="C29" s="52"/>
+      <c r="D29" s="52"/>
+      <c r="E29" s="52">
+        <v>20</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G29" s="70">
+        <v>1.34035214624097E-3</v>
+      </c>
+      <c r="H29" s="52">
+        <f>5*60+36.08</f>
+        <v>336.08</v>
+      </c>
+      <c r="I29" s="53">
+        <f>H29/60</f>
+        <v>5.6013333333333328</v>
+      </c>
+      <c r="J29" s="55" t="s">
+        <v>36</v>
+      </c>
+      <c r="K29" s="55"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B30" s="52"/>
+      <c r="C30" s="52"/>
+      <c r="D30" s="52"/>
+      <c r="E30" s="52"/>
+      <c r="F30" s="52"/>
+      <c r="G30" s="52"/>
+      <c r="H30" s="52"/>
+      <c r="I30" s="53">
+        <f>H30/60</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B31" s="52"/>
+      <c r="C31" s="52"/>
+      <c r="D31" s="52"/>
+      <c r="E31" s="52"/>
+      <c r="F31" s="52"/>
+      <c r="G31" s="52"/>
+      <c r="H31" s="52"/>
+      <c r="I31" s="53">
+        <f>H31/60</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B32" s="52" t="s">
+        <v>13</v>
+      </c>
+      <c r="C32" s="52">
+        <v>50</v>
+      </c>
+      <c r="D32" s="52"/>
+      <c r="E32" s="52"/>
+      <c r="F32" s="52"/>
+      <c r="G32" s="52">
+        <v>1.4277277173853299E-2</v>
+      </c>
+      <c r="H32" s="52">
+        <f>60+48.03</f>
+        <v>108.03</v>
+      </c>
+      <c r="I32" s="53">
+        <f>H32/60</f>
+        <v>1.8005</v>
+      </c>
+      <c r="K32" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B33" s="52"/>
+      <c r="C33" s="52"/>
+      <c r="D33" s="52"/>
+      <c r="E33" s="52"/>
+      <c r="F33" s="52"/>
+      <c r="G33" s="52"/>
+      <c r="H33" s="52"/>
+      <c r="I33" s="53">
+        <f>H33/60</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B34" s="52"/>
+      <c r="C34" s="52"/>
+      <c r="D34" s="52"/>
+      <c r="E34" s="52"/>
+      <c r="F34" s="52"/>
+      <c r="G34" s="52"/>
+      <c r="H34" s="52"/>
+      <c r="I34" s="53">
+        <f>H34/60</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G35">
+        <f>MIN(G23:G34)</f>
+        <v>1.34035214624097E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B40" s="57" t="s">
+        <v>1</v>
+      </c>
+      <c r="C40" s="58" t="s">
+        <v>2</v>
+      </c>
+      <c r="D40" s="58"/>
+      <c r="E40" s="58"/>
+      <c r="F40" s="58"/>
+      <c r="G40" s="57" t="s">
+        <v>9</v>
+      </c>
+      <c r="H40" s="57" t="s">
+        <v>6</v>
+      </c>
+      <c r="I40" s="57" t="s">
+        <v>34</v>
+      </c>
+      <c r="J40" s="59"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B41" s="57"/>
+      <c r="C41" s="50" t="s">
+        <v>3</v>
+      </c>
+      <c r="D41" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E41" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F41" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="G41" s="57"/>
+      <c r="H41" s="57"/>
+      <c r="I41" s="57"/>
+      <c r="J41" s="59"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B42" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2">
+        <v>25</v>
+      </c>
+      <c r="F42" s="2">
+        <v>150</v>
+      </c>
+      <c r="G42" s="54">
+        <v>4.9674920623337304E-4</v>
+      </c>
+      <c r="H42" s="18">
+        <f>3*60+30.56</f>
+        <v>210.56</v>
+      </c>
+      <c r="I42" s="51">
+        <f t="shared" ref="I42:I44" si="5">H42/60</f>
+        <v>3.5093333333333332</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B43" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2">
+        <v>25</v>
+      </c>
+      <c r="F43" s="2">
+        <v>200</v>
+      </c>
+      <c r="G43" s="54">
+        <v>4.96373772906626E-4</v>
+      </c>
+      <c r="H43" s="18">
+        <f>4*60+57.94</f>
+        <v>297.94</v>
+      </c>
+      <c r="I43" s="51">
+        <f t="shared" si="5"/>
+        <v>4.9656666666666665</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B44" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2">
+        <v>20</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G44" s="56">
+        <v>5.3459457337247504E-4</v>
+      </c>
+      <c r="H44" s="2">
+        <f>11*60+36.44</f>
+        <v>696.44</v>
+      </c>
+      <c r="I44" s="51">
+        <f t="shared" si="5"/>
+        <v>11.607333333333335</v>
+      </c>
+      <c r="J44" s="55" t="s">
+        <v>37</v>
+      </c>
+      <c r="K44" s="55"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G46">
+        <f>MIN(G42:G44)</f>
+        <v>4.96373772906626E-4</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="22">
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="T2:T3"/>
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="J40:J41"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:H22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:F40"/>
+    <mergeCell ref="G40:G41"/>
+    <mergeCell ref="H40:H41"/>
+    <mergeCell ref="I40:I41"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Avances 18/03: post reunión, avances en pruebas con PSO.
</commit_message>
<xml_diff>
--- a/Optimizacion/Resultados optimizadores.xlsx
+++ b/Optimizacion/Resultados optimizadores.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
-  <workbookPr/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uccl0-my.sharepoint.com/personal/mfernandafolch_uc_cl/Documents/Escritorio/Concha y Toro/Proyecto_Tintos_CyT_P2/Optimizacion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1478" documentId="11_AD4D2F04E46CFB4ACB3E20395551EF76693EDF1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AA2D608-32F6-4684-9161-6EF88E76B899}"/>
+  <xr:revisionPtr revIDLastSave="2080" documentId="11_AD4D2F04E46CFB4ACB3E20395551EF76693EDF1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5C88990-6139-4981-B232-B2EFB61D2B00}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="71">
   <si>
     <t>Set de datos:</t>
   </si>
@@ -172,20 +173,99 @@
   </si>
   <si>
     <t>Mas de una hora corriendo</t>
+  </si>
+  <si>
+    <t>Método PSO</t>
+  </si>
+  <si>
+    <t>pop_size</t>
+  </si>
+  <si>
+    <t>epoch</t>
+  </si>
+  <si>
+    <t>c1</t>
+  </si>
+  <si>
+    <t>c2</t>
+  </si>
+  <si>
+    <t>w</t>
+  </si>
+  <si>
+    <t>Parámetros</t>
+  </si>
+  <si>
+    <t>mu0</t>
+  </si>
+  <si>
+    <t>betaG0</t>
+  </si>
+  <si>
+    <t>betaF0</t>
+  </si>
+  <si>
+    <t>Kn0</t>
+  </si>
+  <si>
+    <t>Kg0</t>
+  </si>
+  <si>
+    <t>Kf0</t>
+  </si>
+  <si>
+    <t>Kig0</t>
+  </si>
+  <si>
+    <t>Kie0</t>
+  </si>
+  <si>
+    <t>Kd0</t>
+  </si>
+  <si>
+    <t>Yxn</t>
+  </si>
+  <si>
+    <t>Yxf</t>
+  </si>
+  <si>
+    <t>Yeg</t>
+  </si>
+  <si>
+    <t>Yef</t>
+  </si>
+  <si>
+    <t>Yxg</t>
+  </si>
+  <si>
+    <t>PSO_gpt</t>
+  </si>
+  <si>
+    <t>Parámetros fijados</t>
+  </si>
+  <si>
+    <t>PSO_pyswarms</t>
+  </si>
+  <si>
+    <t>PSO_mealpy</t>
+  </si>
+  <si>
+    <t>PSO_pymoo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0.0000000"/>
     <numFmt numFmtId="165" formatCode="#,##0.00000000"/>
     <numFmt numFmtId="166" formatCode="#,##0.000000"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.000000000"/>
+    <numFmt numFmtId="170" formatCode="0.0000000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -214,8 +294,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -246,6 +348,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="23">
     <border>
@@ -553,7 +661,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -628,13 +736,36 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -663,28 +794,22 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="168" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1219,25 +1344,25 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="62" t="s">
+      <c r="C2" s="71" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="65" t="s">
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="74" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="65" t="s">
+      <c r="H2" s="74" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="65" t="s">
+      <c r="I2" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="60" t="s">
+      <c r="J2" s="69" t="s">
         <v>6</v>
       </c>
       <c r="L2" t="s">
@@ -1245,7 +1370,7 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="64"/>
+      <c r="B3" s="73"/>
       <c r="C3" s="16" t="s">
         <v>3</v>
       </c>
@@ -1258,10 +1383,10 @@
       <c r="F3" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="67"/>
+      <c r="G3" s="75"/>
+      <c r="H3" s="75"/>
+      <c r="I3" s="75"/>
+      <c r="J3" s="76"/>
       <c r="L3" t="s">
         <v>15</v>
       </c>
@@ -2769,30 +2894,30 @@
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B71" s="63" t="s">
+      <c r="B71" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="C71" s="62" t="s">
+      <c r="C71" s="71" t="s">
         <v>2</v>
       </c>
-      <c r="D71" s="62"/>
-      <c r="E71" s="62"/>
-      <c r="F71" s="62"/>
-      <c r="G71" s="65" t="s">
+      <c r="D71" s="71"/>
+      <c r="E71" s="71"/>
+      <c r="F71" s="71"/>
+      <c r="G71" s="74" t="s">
         <v>12</v>
       </c>
-      <c r="H71" s="65" t="s">
+      <c r="H71" s="74" t="s">
         <v>9</v>
       </c>
-      <c r="I71" s="65" t="s">
+      <c r="I71" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="J71" s="60" t="s">
+      <c r="J71" s="69" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="72" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B72" s="68"/>
+      <c r="B72" s="77"/>
       <c r="C72" s="7" t="s">
         <v>3</v>
       </c>
@@ -2805,10 +2930,10 @@
       <c r="F72" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G72" s="69"/>
-      <c r="H72" s="69"/>
-      <c r="I72" s="69"/>
-      <c r="J72" s="61"/>
+      <c r="G72" s="60"/>
+      <c r="H72" s="60"/>
+      <c r="I72" s="60"/>
+      <c r="J72" s="70"/>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B73" s="8" t="s">
@@ -3052,48 +3177,48 @@
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="58" t="s">
+      <c r="C2" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="57" t="s">
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="57" t="s">
+      <c r="H2" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="57" t="s">
+      <c r="I2" s="65" t="s">
         <v>34</v>
       </c>
-      <c r="N2" s="57" t="s">
+      <c r="N2" s="65" t="s">
         <v>40</v>
       </c>
-      <c r="O2" s="77" t="s">
+      <c r="O2" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="P2" s="74" t="s">
+      <c r="P2" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="75"/>
-      <c r="R2" s="75"/>
-      <c r="S2" s="76"/>
-      <c r="T2" s="69" t="s">
+      <c r="Q2" s="63"/>
+      <c r="R2" s="63"/>
+      <c r="S2" s="64"/>
+      <c r="T2" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="U2" s="69" t="s">
+      <c r="U2" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="V2" s="69" t="s">
+      <c r="V2" s="60" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="B3" s="57"/>
+      <c r="B3" s="65"/>
       <c r="C3" s="50" t="s">
         <v>3</v>
       </c>
@@ -3106,11 +3231,11 @@
       <c r="F3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="N3" s="57"/>
-      <c r="O3" s="77"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
+      <c r="I3" s="65"/>
+      <c r="N3" s="65"/>
+      <c r="O3" s="66"/>
       <c r="P3" s="50" t="s">
         <v>3</v>
       </c>
@@ -3123,9 +3248,9 @@
       <c r="S3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="T3" s="73"/>
-      <c r="U3" s="73"/>
-      <c r="V3" s="73"/>
+      <c r="T3" s="61"/>
+      <c r="U3" s="61"/>
+      <c r="V3" s="61"/>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="B4" s="2" t="s">
@@ -3169,7 +3294,7 @@
         <v>3.5386864122503397E-4</v>
       </c>
       <c r="U4" s="2">
-        <f t="shared" ref="U4:V6" si="0">H5</f>
+        <f t="shared" ref="U4:V4" si="0">H5</f>
         <v>84.3</v>
       </c>
       <c r="V4" s="2">
@@ -3294,7 +3419,7 @@
         <f t="shared" ref="U7:V7" si="2">H25</f>
         <v>983.38</v>
       </c>
-      <c r="V7" s="78">
+      <c r="V7" s="59">
         <f t="shared" si="2"/>
         <v>16.389666666666667</v>
       </c>
@@ -3396,8 +3521,6 @@
         <f>H10/60</f>
         <v>0.39316666666666666</v>
       </c>
-      <c r="J10" s="71"/>
-      <c r="K10" s="71"/>
       <c r="N10" s="2" t="s">
         <v>18</v>
       </c>
@@ -3549,27 +3672,27 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B21" s="57" t="s">
+      <c r="B21" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C21" s="58" t="s">
+      <c r="C21" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="58"/>
-      <c r="E21" s="58"/>
-      <c r="F21" s="58"/>
-      <c r="G21" s="57" t="s">
+      <c r="D21" s="68"/>
+      <c r="E21" s="68"/>
+      <c r="F21" s="68"/>
+      <c r="G21" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="H21" s="57" t="s">
+      <c r="H21" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="I21" s="57" t="s">
+      <c r="I21" s="65" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B22" s="57"/>
+      <c r="B22" s="65"/>
       <c r="C22" s="50" t="s">
         <v>3</v>
       </c>
@@ -3582,9 +3705,9 @@
       <c r="F22" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G22" s="57"/>
-      <c r="H22" s="57"/>
-      <c r="I22" s="57"/>
+      <c r="G22" s="65"/>
+      <c r="H22" s="65"/>
+      <c r="I22" s="65"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B23" s="2" t="s">
@@ -3598,7 +3721,7 @@
       <c r="F23" s="2">
         <v>150</v>
       </c>
-      <c r="G23" s="72">
+      <c r="G23" s="58">
         <v>1.10227895476947E-2</v>
       </c>
       <c r="H23" s="18">
@@ -3688,7 +3811,7 @@
         <v>177.09</v>
       </c>
       <c r="I27" s="53">
-        <f>H27/60</f>
+        <f t="shared" ref="I27:I34" si="5">H27/60</f>
         <v>2.9515000000000002</v>
       </c>
     </row>
@@ -3712,7 +3835,7 @@
         <v>256.62</v>
       </c>
       <c r="I28" s="53">
-        <f>H28/60</f>
+        <f t="shared" si="5"/>
         <v>4.2770000000000001</v>
       </c>
     </row>
@@ -3728,7 +3851,7 @@
       <c r="F29" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G29" s="70">
+      <c r="G29" s="31">
         <v>1.34035214624097E-3</v>
       </c>
       <c r="H29" s="52">
@@ -3736,7 +3859,7 @@
         <v>336.08</v>
       </c>
       <c r="I29" s="53">
-        <f>H29/60</f>
+        <f t="shared" si="5"/>
         <v>5.6013333333333328</v>
       </c>
       <c r="J29" s="55" t="s">
@@ -3753,7 +3876,7 @@
       <c r="G30" s="52"/>
       <c r="H30" s="52"/>
       <c r="I30" s="53">
-        <f>H30/60</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -3766,7 +3889,7 @@
       <c r="G31" s="52"/>
       <c r="H31" s="52"/>
       <c r="I31" s="53">
-        <f>H31/60</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -3788,7 +3911,7 @@
         <v>108.03</v>
       </c>
       <c r="I32" s="53">
-        <f>H32/60</f>
+        <f t="shared" si="5"/>
         <v>1.8005</v>
       </c>
       <c r="K32" t="s">
@@ -3804,7 +3927,7 @@
       <c r="G33" s="52"/>
       <c r="H33" s="52"/>
       <c r="I33" s="53">
-        <f>H33/60</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -3817,7 +3940,7 @@
       <c r="G34" s="52"/>
       <c r="H34" s="52"/>
       <c r="I34" s="53">
-        <f>H34/60</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -3836,28 +3959,28 @@
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B40" s="57" t="s">
+      <c r="B40" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C40" s="58" t="s">
+      <c r="C40" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="D40" s="58"/>
-      <c r="E40" s="58"/>
-      <c r="F40" s="58"/>
-      <c r="G40" s="57" t="s">
+      <c r="D40" s="68"/>
+      <c r="E40" s="68"/>
+      <c r="F40" s="68"/>
+      <c r="G40" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="H40" s="57" t="s">
+      <c r="H40" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="I40" s="57" t="s">
+      <c r="I40" s="65" t="s">
         <v>34</v>
       </c>
-      <c r="J40" s="59"/>
+      <c r="J40" s="67"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B41" s="57"/>
+      <c r="B41" s="65"/>
       <c r="C41" s="50" t="s">
         <v>3</v>
       </c>
@@ -3870,10 +3993,10 @@
       <c r="F41" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G41" s="57"/>
-      <c r="H41" s="57"/>
-      <c r="I41" s="57"/>
-      <c r="J41" s="59"/>
+      <c r="G41" s="65"/>
+      <c r="H41" s="65"/>
+      <c r="I41" s="65"/>
+      <c r="J41" s="67"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B42" s="2" t="s">
@@ -3895,7 +4018,7 @@
         <v>210.56</v>
       </c>
       <c r="I42" s="51">
-        <f t="shared" ref="I42:I44" si="5">H42/60</f>
+        <f t="shared" ref="I42:I44" si="6">H42/60</f>
         <v>3.5093333333333332</v>
       </c>
     </row>
@@ -3919,7 +4042,7 @@
         <v>297.94</v>
       </c>
       <c r="I43" s="51">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>4.9656666666666665</v>
       </c>
     </row>
@@ -3943,7 +4066,7 @@
         <v>696.44</v>
       </c>
       <c r="I44" s="51">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>11.607333333333335</v>
       </c>
       <c r="J44" s="55" t="s">
@@ -3959,12 +4082,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="T2:T3"/>
-    <mergeCell ref="P2:S2"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
     <mergeCell ref="J40:J41"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="B21:B22"/>
@@ -3981,6 +4098,1089 @@
     <mergeCell ref="G40:G41"/>
     <mergeCell ref="H40:H41"/>
     <mergeCell ref="I40:I41"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="T2:T3"/>
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F024A9F-720A-4384-9592-EDD81D7A1CFE}">
+  <dimension ref="A1:Z21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="37.26953125" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7265625" customWidth="1"/>
+    <col min="4" max="4" width="9.1796875" customWidth="1"/>
+    <col min="5" max="5" width="8.36328125" customWidth="1"/>
+    <col min="6" max="7" width="6.90625" customWidth="1"/>
+    <col min="8" max="8" width="15.08984375" customWidth="1"/>
+    <col min="9" max="9" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.7265625" customWidth="1"/>
+    <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="16.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="60" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="60" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="62" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="60" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="60" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="60" t="s">
+        <v>34</v>
+      </c>
+      <c r="K1" s="62" t="s">
+        <v>51</v>
+      </c>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
+      <c r="Q1" s="63"/>
+      <c r="R1" s="63"/>
+      <c r="S1" s="63"/>
+      <c r="T1" s="63"/>
+      <c r="U1" s="63"/>
+      <c r="V1" s="63"/>
+      <c r="W1" s="63"/>
+      <c r="X1" s="64"/>
+      <c r="Z1" s="55" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="57" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" s="57" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" s="57" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" s="57" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" s="57" t="s">
+        <v>50</v>
+      </c>
+      <c r="H2" s="61"/>
+      <c r="I2" s="61"/>
+      <c r="J2" s="61"/>
+      <c r="K2" s="82" t="s">
+        <v>52</v>
+      </c>
+      <c r="L2" s="82" t="s">
+        <v>53</v>
+      </c>
+      <c r="M2" s="82" t="s">
+        <v>54</v>
+      </c>
+      <c r="N2" s="79" t="s">
+        <v>55</v>
+      </c>
+      <c r="O2" s="79" t="s">
+        <v>56</v>
+      </c>
+      <c r="P2" s="79" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q2" s="79" t="s">
+        <v>58</v>
+      </c>
+      <c r="R2" s="79" t="s">
+        <v>59</v>
+      </c>
+      <c r="S2" s="79" t="s">
+        <v>60</v>
+      </c>
+      <c r="T2" s="82" t="s">
+        <v>61</v>
+      </c>
+      <c r="U2" s="82" t="s">
+        <v>65</v>
+      </c>
+      <c r="V2" s="81" t="s">
+        <v>62</v>
+      </c>
+      <c r="W2" s="82" t="s">
+        <v>63</v>
+      </c>
+      <c r="X2" s="82" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="2">
+        <v>150</v>
+      </c>
+      <c r="D3" s="2">
+        <v>20</v>
+      </c>
+      <c r="E3" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="H3" s="78">
+        <v>2.9472175802249201E-4</v>
+      </c>
+      <c r="I3" s="2">
+        <f>60+13.49</f>
+        <v>73.489999999999995</v>
+      </c>
+      <c r="J3" s="51">
+        <f>I3/60</f>
+        <v>1.2248333333333332</v>
+      </c>
+      <c r="K3" s="83">
+        <v>2.1924339239705899E-2</v>
+      </c>
+      <c r="L3" s="83">
+        <v>5.3243124688619803</v>
+      </c>
+      <c r="M3" s="83">
+        <v>10</v>
+      </c>
+      <c r="N3" s="80">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O3" s="80">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P3" s="80">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q3" s="80">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R3" s="80">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S3" s="80">
+        <v>1E-4</v>
+      </c>
+      <c r="T3" s="83">
+        <v>2.1598443591871601</v>
+      </c>
+      <c r="U3" s="83">
+        <v>9.4242283395423598</v>
+      </c>
+      <c r="V3" s="80">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W3" s="83">
+        <v>0.1</v>
+      </c>
+      <c r="X3" s="83">
+        <v>0.66937281186906705</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="2">
+        <v>150</v>
+      </c>
+      <c r="D4" s="2">
+        <v>20</v>
+      </c>
+      <c r="E4" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="H4" s="78">
+        <v>1.40375181209925E-2</v>
+      </c>
+      <c r="I4" s="2">
+        <f>60+6.44</f>
+        <v>66.44</v>
+      </c>
+      <c r="J4" s="51">
+        <f t="shared" ref="J4:J14" si="0">I4/60</f>
+        <v>1.1073333333333333</v>
+      </c>
+      <c r="K4" s="84">
+        <v>2.13935160996067</v>
+      </c>
+      <c r="L4" s="84">
+        <v>3.7720314524367198</v>
+      </c>
+      <c r="M4" s="84">
+        <v>7.0774441190072404</v>
+      </c>
+      <c r="N4" s="80">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O4" s="80">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P4" s="80">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q4" s="80">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R4" s="80">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S4" s="80">
+        <v>1E-4</v>
+      </c>
+      <c r="T4" s="84">
+        <v>1.8888019984842901</v>
+      </c>
+      <c r="U4" s="84">
+        <v>6.3974765814129801</v>
+      </c>
+      <c r="V4" s="80">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W4" s="83">
+        <v>0.83091291134603795</v>
+      </c>
+      <c r="X4" s="83">
+        <v>0.11175654744772601</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="2">
+        <v>150</v>
+      </c>
+      <c r="D5" s="2">
+        <v>20</v>
+      </c>
+      <c r="E5" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="H5" s="78">
+        <v>1.32701286472156E-3</v>
+      </c>
+      <c r="I5" s="2">
+        <f>5*60+48.41</f>
+        <v>348.40999999999997</v>
+      </c>
+      <c r="J5" s="51">
+        <f t="shared" si="0"/>
+        <v>5.8068333333333326</v>
+      </c>
+      <c r="K5" s="84">
+        <v>3.0051333747301801</v>
+      </c>
+      <c r="L5" s="84">
+        <v>5.0528684093825298</v>
+      </c>
+      <c r="M5" s="84">
+        <v>4.8710938159898802</v>
+      </c>
+      <c r="N5" s="80">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O5" s="80">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P5" s="80">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q5" s="80">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R5" s="80">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S5" s="80">
+        <v>1E-4</v>
+      </c>
+      <c r="T5" s="84">
+        <v>1.06812478247408</v>
+      </c>
+      <c r="U5" s="84">
+        <v>3.3029168292772599</v>
+      </c>
+      <c r="V5" s="80">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W5" s="83">
+        <v>0.29242188148853998</v>
+      </c>
+      <c r="X5" s="83">
+        <v>0.47648836606682399</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="2">
+        <v>150</v>
+      </c>
+      <c r="D6" s="2">
+        <v>20</v>
+      </c>
+      <c r="E6" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="H6" s="78">
+        <v>7.04873626723777E-4</v>
+      </c>
+      <c r="I6" s="2">
+        <f>60+14.51</f>
+        <v>74.510000000000005</v>
+      </c>
+      <c r="J6" s="51">
+        <f t="shared" si="0"/>
+        <v>1.2418333333333333</v>
+      </c>
+      <c r="K6" s="83">
+        <v>0.232102232392803</v>
+      </c>
+      <c r="L6" s="84">
+        <v>4.1297069928879102</v>
+      </c>
+      <c r="M6" s="84">
+        <v>6.0078738386920403</v>
+      </c>
+      <c r="N6" s="80">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O6" s="80">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P6" s="80">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q6" s="80">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R6" s="80">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S6" s="80">
+        <v>1E-4</v>
+      </c>
+      <c r="T6" s="84">
+        <v>1.1019035329447</v>
+      </c>
+      <c r="U6" s="84">
+        <v>2.97276558235572</v>
+      </c>
+      <c r="V6" s="80">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W6" s="83">
+        <v>0.20748440650441199</v>
+      </c>
+      <c r="X6" s="83">
+        <v>0.59401552721599604</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="2">
+        <v>200</v>
+      </c>
+      <c r="D7" s="2">
+        <v>20</v>
+      </c>
+      <c r="E7" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="F7" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="H7" s="78">
+        <v>2.9328842498517401E-4</v>
+      </c>
+      <c r="I7" s="2">
+        <f>60+15.12</f>
+        <v>75.12</v>
+      </c>
+      <c r="J7" s="51">
+        <f t="shared" si="0"/>
+        <v>1.252</v>
+      </c>
+      <c r="K7" s="83">
+        <v>2.1763903293888599E-2</v>
+      </c>
+      <c r="L7" s="83">
+        <v>5.3320005646842601</v>
+      </c>
+      <c r="M7" s="83">
+        <v>10</v>
+      </c>
+      <c r="N7" s="80">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O7" s="80">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P7" s="80">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q7" s="80">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R7" s="80">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S7" s="80">
+        <v>1E-4</v>
+      </c>
+      <c r="T7" s="84">
+        <v>2.7464836815839999</v>
+      </c>
+      <c r="U7" s="84">
+        <v>9.4217689488491896</v>
+      </c>
+      <c r="V7" s="80">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W7" s="83">
+        <v>0.1</v>
+      </c>
+      <c r="X7" s="83">
+        <v>0.66954694007881499</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" s="2">
+        <v>200</v>
+      </c>
+      <c r="D8" s="2">
+        <v>20</v>
+      </c>
+      <c r="E8" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="H8" s="86">
+        <v>3.3229795416845E-3</v>
+      </c>
+      <c r="I8" s="2">
+        <f>60+30.34</f>
+        <v>90.34</v>
+      </c>
+      <c r="J8" s="51">
+        <f t="shared" si="0"/>
+        <v>1.5056666666666667</v>
+      </c>
+      <c r="K8" s="84">
+        <v>5.3708635632974699</v>
+      </c>
+      <c r="L8" s="84">
+        <v>1.91711370869458</v>
+      </c>
+      <c r="M8" s="84">
+        <v>1.21894257791956</v>
+      </c>
+      <c r="N8" s="80">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O8" s="80">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P8" s="80">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q8" s="80">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R8" s="80">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S8" s="80">
+        <v>1E-4</v>
+      </c>
+      <c r="T8" s="84">
+        <v>5.0621300467977699</v>
+      </c>
+      <c r="U8" s="84">
+        <v>4.3662737525307698</v>
+      </c>
+      <c r="V8" s="80">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W8" s="83">
+        <v>0.32173344505856499</v>
+      </c>
+      <c r="X8" s="83">
+        <v>0.41579920796990599</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="2">
+        <v>200</v>
+      </c>
+      <c r="D9" s="2">
+        <v>20</v>
+      </c>
+      <c r="E9" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="F9" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="H9" s="78">
+        <v>1.3251362658287199E-3</v>
+      </c>
+      <c r="I9" s="2">
+        <f>60*7+25.26</f>
+        <v>445.26</v>
+      </c>
+      <c r="J9" s="51">
+        <f t="shared" si="0"/>
+        <v>7.4210000000000003</v>
+      </c>
+      <c r="K9" s="84">
+        <v>3.01506522825153</v>
+      </c>
+      <c r="L9" s="84">
+        <v>5.05925344685207</v>
+      </c>
+      <c r="M9" s="83">
+        <v>4.86872801688311</v>
+      </c>
+      <c r="N9" s="80">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O9" s="80">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P9" s="80">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q9" s="80">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R9" s="80">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S9" s="80">
+        <v>1E-4</v>
+      </c>
+      <c r="T9" s="84">
+        <v>1.06792904742284</v>
+      </c>
+      <c r="U9" s="84">
+        <v>3.30384536377028</v>
+      </c>
+      <c r="V9" s="80">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W9" s="83">
+        <v>0.29253732272668498</v>
+      </c>
+      <c r="X9" s="83">
+        <v>0.47645758028965701</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="2">
+        <v>200</v>
+      </c>
+      <c r="D10" s="2">
+        <v>20</v>
+      </c>
+      <c r="E10" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="F10" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="H10" s="2">
+        <v>7.04243140314323E-4</v>
+      </c>
+      <c r="I10" s="2">
+        <f>60+30.12</f>
+        <v>90.12</v>
+      </c>
+      <c r="J10" s="51">
+        <f t="shared" si="0"/>
+        <v>1.502</v>
+      </c>
+      <c r="K10" s="83">
+        <v>0.23198883475251</v>
+      </c>
+      <c r="L10" s="83">
+        <v>4.13163737355673</v>
+      </c>
+      <c r="M10" s="83">
+        <v>6.0033822043910199</v>
+      </c>
+      <c r="N10" s="80">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O10" s="80">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P10" s="80">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q10" s="80">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R10" s="80">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S10" s="80">
+        <v>1E-4</v>
+      </c>
+      <c r="T10" s="84">
+        <v>1.10164214051543</v>
+      </c>
+      <c r="U10" s="84">
+        <v>3.12238469928359</v>
+      </c>
+      <c r="V10" s="80">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W10" s="83">
+        <v>0.207546998368103</v>
+      </c>
+      <c r="X10" s="83">
+        <v>0.59565351370611197</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="2">
+        <v>500</v>
+      </c>
+      <c r="D11" s="2">
+        <v>20</v>
+      </c>
+      <c r="E11" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="F11" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2">
+        <v>0</v>
+      </c>
+      <c r="J11" s="51">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K11" s="85">
+        <v>0</v>
+      </c>
+      <c r="L11" s="85">
+        <v>0</v>
+      </c>
+      <c r="M11" s="85">
+        <v>0</v>
+      </c>
+      <c r="N11" s="80">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O11" s="80">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P11" s="80">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q11" s="80">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R11" s="80">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S11" s="80">
+        <v>1E-4</v>
+      </c>
+      <c r="T11" s="85">
+        <v>0</v>
+      </c>
+      <c r="U11" s="85">
+        <v>0</v>
+      </c>
+      <c r="V11" s="80">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W11" s="85">
+        <v>0</v>
+      </c>
+      <c r="X11" s="85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="2">
+        <v>500</v>
+      </c>
+      <c r="D12" s="2">
+        <v>20</v>
+      </c>
+      <c r="E12" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="F12" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0</v>
+      </c>
+      <c r="J12" s="51">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K12" s="85">
+        <v>0</v>
+      </c>
+      <c r="L12" s="85">
+        <v>0</v>
+      </c>
+      <c r="M12" s="85">
+        <v>0</v>
+      </c>
+      <c r="N12" s="80">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O12" s="80">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P12" s="80">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q12" s="80">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R12" s="80">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S12" s="80">
+        <v>1E-4</v>
+      </c>
+      <c r="T12" s="85">
+        <v>0</v>
+      </c>
+      <c r="U12" s="85">
+        <v>0</v>
+      </c>
+      <c r="V12" s="80">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W12" s="85">
+        <v>0</v>
+      </c>
+      <c r="X12" s="85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="2">
+        <v>500</v>
+      </c>
+      <c r="D13" s="2">
+        <v>20</v>
+      </c>
+      <c r="E13" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="F13" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G13" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="H13" s="2">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0</v>
+      </c>
+      <c r="J13" s="51">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K13" s="85">
+        <v>0</v>
+      </c>
+      <c r="L13" s="85">
+        <v>0</v>
+      </c>
+      <c r="M13" s="85">
+        <v>0</v>
+      </c>
+      <c r="N13" s="80">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O13" s="80">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P13" s="80">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q13" s="80">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R13" s="80">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S13" s="80">
+        <v>1E-4</v>
+      </c>
+      <c r="T13" s="85">
+        <v>0</v>
+      </c>
+      <c r="U13" s="85">
+        <v>0</v>
+      </c>
+      <c r="V13" s="80">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W13" s="85">
+        <v>0</v>
+      </c>
+      <c r="X13" s="85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="2">
+        <v>500</v>
+      </c>
+      <c r="D14" s="2">
+        <v>20</v>
+      </c>
+      <c r="E14" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="F14" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="H14" s="2">
+        <v>7.0311620720228901E-4</v>
+      </c>
+      <c r="I14" s="2">
+        <f>4*60+9.5</f>
+        <v>249.5</v>
+      </c>
+      <c r="J14" s="51">
+        <f t="shared" si="0"/>
+        <v>4.1583333333333332</v>
+      </c>
+      <c r="K14" s="83">
+        <v>0.230277928812854</v>
+      </c>
+      <c r="L14" s="84">
+        <v>4.1471160732970196</v>
+      </c>
+      <c r="M14" s="84">
+        <v>6.0025562868090301</v>
+      </c>
+      <c r="N14" s="80">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O14" s="80">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P14" s="80">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q14" s="80">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R14" s="80">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S14" s="80">
+        <v>1E-4</v>
+      </c>
+      <c r="T14" s="84">
+        <v>1.1015287199813399</v>
+      </c>
+      <c r="U14" s="84">
+        <v>2.49443328688508</v>
+      </c>
+      <c r="V14" s="80">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W14" s="83">
+        <v>0.20757536882927899</v>
+      </c>
+      <c r="X14" s="83">
+        <v>0.59564622966884795</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A17" s="2"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" s="2"/>
+      <c r="H18" s="87"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20" s="2"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A21" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="C1:G1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:J2"/>
+    <mergeCell ref="K1:X1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Avances 19/03: Pruebas PSO, pymoo es el mejor.
</commit_message>
<xml_diff>
--- a/Optimizacion/Resultados optimizadores.xlsx
+++ b/Optimizacion/Resultados optimizadores.xlsx
@@ -1,22 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uccl0-my.sharepoint.com/personal/mfernandafolch_uc_cl/Documents/Escritorio/Concha y Toro/Proyecto_Tintos_CyT_P2/Optimizacion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2080" documentId="11_AD4D2F04E46CFB4ACB3E20395551EF76693EDF1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5C88990-6139-4981-B232-B2EFB61D2B00}"/>
+  <xr:revisionPtr revIDLastSave="3259" documentId="11_AD4D2F04E46CFB4ACB3E20395551EF76693EDF1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DB6260E-9F20-4E87-BA24-4468EF55AE14}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
-    <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
+    <sheet name="Pruebas PSO" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pruebas PSO'!$A$2:$X$36</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -37,8 +40,35 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={D3BE4DB7-6357-44ED-AFF7-727C0C991779}</author>
+    <author>tc={C19F6259-C0C9-43B5-BDBC-3757C13DADEC}</author>
+  </authors>
+  <commentList>
+    <comment ref="J18" authorId="0" shapeId="0" xr:uid="{D3BE4DB7-6357-44ED-AFF7-727C0C991779}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    MUY LENTO</t>
+      </text>
+    </comment>
+    <comment ref="J28" authorId="1" shapeId="0" xr:uid="{C19F6259-C0C9-43B5-BDBC-3757C13DADEC}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    MUY LENTO</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="71">
   <si>
     <t>Set de datos:</t>
   </si>
@@ -257,13 +287,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0.0000000"/>
     <numFmt numFmtId="165" formatCode="#,##0.00000000"/>
     <numFmt numFmtId="166" formatCode="#,##0.000000"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.000000000"/>
-    <numFmt numFmtId="170" formatCode="0.0000000"/>
+    <numFmt numFmtId="169" formatCode="0.0000000"/>
+    <numFmt numFmtId="170" formatCode="0.00000000"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -309,15 +340,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -354,8 +383,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="23">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -657,11 +698,74 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -735,11 +839,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="168" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -753,18 +858,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -794,22 +887,88 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1055,6 +1214,12 @@
   <inkml:trace contextRef="#ctx0" brushRef="#br0">6653 57,'-32'-1,"-51"-10,17 2,-560-26,-773 37,815-3,566 1</inkml:trace>
   <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2433.25">3364 21,'-152'0,"-797"14,383-9,337-6,83-9,-1 1,69 10,-15 0,-121-13,126 4,-134 6,104 4,-227-2,328 0</inkml:trace>
 </inkml:ink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="María Fernanda Folch Díaz" id="{5D4D3F9D-C31C-4FEE-ADBF-F3914B8EBD59}" userId="S::mfernandafolch@uc.cl::0edf900c-c7cc-461f-97c7-8fa0d92641eb" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1318,6 +1483,17 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="J18" dT="2026-03-19T14:12:16.14" personId="{5D4D3F9D-C31C-4FEE-ADBF-F3914B8EBD59}" id="{D3BE4DB7-6357-44ED-AFF7-727C0C991779}">
+    <text>MUY LENTO</text>
+  </threadedComment>
+  <threadedComment ref="J28" dT="2026-03-19T15:49:42.54" personId="{5D4D3F9D-C31C-4FEE-ADBF-F3914B8EBD59}" id="{C19F6259-C0C9-43B5-BDBC-3757C13DADEC}">
+    <text>MUY LENTO</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T83"/>
@@ -1344,25 +1520,25 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B2" s="72" t="s">
+      <c r="B2" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="71" t="s">
+      <c r="C2" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="74" t="s">
+      <c r="D2" s="70"/>
+      <c r="E2" s="70"/>
+      <c r="F2" s="70"/>
+      <c r="G2" s="73" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="74" t="s">
+      <c r="H2" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="74" t="s">
+      <c r="I2" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="69" t="s">
+      <c r="J2" s="68" t="s">
         <v>6</v>
       </c>
       <c r="L2" t="s">
@@ -1370,7 +1546,7 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="73"/>
+      <c r="B3" s="72"/>
       <c r="C3" s="16" t="s">
         <v>3</v>
       </c>
@@ -1383,10 +1559,10 @@
       <c r="F3" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="75"/>
-      <c r="H3" s="75"/>
-      <c r="I3" s="75"/>
-      <c r="J3" s="76"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="74"/>
+      <c r="I3" s="74"/>
+      <c r="J3" s="75"/>
       <c r="L3" t="s">
         <v>15</v>
       </c>
@@ -2894,30 +3070,30 @@
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B71" s="72" t="s">
+      <c r="B71" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="C71" s="71" t="s">
+      <c r="C71" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="D71" s="71"/>
-      <c r="E71" s="71"/>
-      <c r="F71" s="71"/>
-      <c r="G71" s="74" t="s">
+      <c r="D71" s="70"/>
+      <c r="E71" s="70"/>
+      <c r="F71" s="70"/>
+      <c r="G71" s="73" t="s">
         <v>12</v>
       </c>
-      <c r="H71" s="74" t="s">
+      <c r="H71" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="I71" s="74" t="s">
+      <c r="I71" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="J71" s="69" t="s">
+      <c r="J71" s="68" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="72" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B72" s="77"/>
+      <c r="B72" s="76"/>
       <c r="C72" s="7" t="s">
         <v>3</v>
       </c>
@@ -2930,10 +3106,10 @@
       <c r="F72" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G72" s="60"/>
-      <c r="H72" s="60"/>
-      <c r="I72" s="60"/>
-      <c r="J72" s="70"/>
+      <c r="G72" s="63"/>
+      <c r="H72" s="63"/>
+      <c r="I72" s="63"/>
+      <c r="J72" s="69"/>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B73" s="8" t="s">
@@ -3177,48 +3353,48 @@
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="B2" s="65" t="s">
+      <c r="B2" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="68" t="s">
+      <c r="C2" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="65" t="s">
+      <c r="D2" s="80"/>
+      <c r="E2" s="80"/>
+      <c r="F2" s="80"/>
+      <c r="G2" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="65" t="s">
+      <c r="H2" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="65" t="s">
+      <c r="I2" s="77" t="s">
         <v>34</v>
       </c>
-      <c r="N2" s="65" t="s">
+      <c r="N2" s="77" t="s">
         <v>40</v>
       </c>
-      <c r="O2" s="66" t="s">
+      <c r="O2" s="78" t="s">
         <v>1</v>
       </c>
-      <c r="P2" s="62" t="s">
+      <c r="P2" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="63"/>
-      <c r="R2" s="63"/>
-      <c r="S2" s="64"/>
-      <c r="T2" s="60" t="s">
+      <c r="Q2" s="66"/>
+      <c r="R2" s="66"/>
+      <c r="S2" s="67"/>
+      <c r="T2" s="63" t="s">
         <v>9</v>
       </c>
-      <c r="U2" s="60" t="s">
+      <c r="U2" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="V2" s="60" t="s">
+      <c r="V2" s="63" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="B3" s="65"/>
+      <c r="B3" s="77"/>
       <c r="C3" s="50" t="s">
         <v>3</v>
       </c>
@@ -3231,11 +3407,11 @@
       <c r="F3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="65"/>
-      <c r="H3" s="65"/>
-      <c r="I3" s="65"/>
-      <c r="N3" s="65"/>
-      <c r="O3" s="66"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+      <c r="I3" s="77"/>
+      <c r="N3" s="77"/>
+      <c r="O3" s="78"/>
       <c r="P3" s="50" t="s">
         <v>3</v>
       </c>
@@ -3248,9 +3424,9 @@
       <c r="S3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="T3" s="61"/>
-      <c r="U3" s="61"/>
-      <c r="V3" s="61"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="B4" s="2" t="s">
@@ -3419,7 +3595,7 @@
         <f t="shared" ref="U7:V7" si="2">H25</f>
         <v>983.38</v>
       </c>
-      <c r="V7" s="59">
+      <c r="V7" s="58">
         <f t="shared" si="2"/>
         <v>16.389666666666667</v>
       </c>
@@ -3672,27 +3848,27 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B21" s="65" t="s">
+      <c r="B21" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="C21" s="68" t="s">
+      <c r="C21" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="68"/>
-      <c r="E21" s="68"/>
-      <c r="F21" s="68"/>
-      <c r="G21" s="65" t="s">
+      <c r="D21" s="80"/>
+      <c r="E21" s="80"/>
+      <c r="F21" s="80"/>
+      <c r="G21" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="H21" s="65" t="s">
+      <c r="H21" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="I21" s="65" t="s">
+      <c r="I21" s="77" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B22" s="65"/>
+      <c r="B22" s="77"/>
       <c r="C22" s="50" t="s">
         <v>3</v>
       </c>
@@ -3705,9 +3881,9 @@
       <c r="F22" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G22" s="65"/>
-      <c r="H22" s="65"/>
-      <c r="I22" s="65"/>
+      <c r="G22" s="77"/>
+      <c r="H22" s="77"/>
+      <c r="I22" s="77"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B23" s="2" t="s">
@@ -3721,7 +3897,7 @@
       <c r="F23" s="2">
         <v>150</v>
       </c>
-      <c r="G23" s="58">
+      <c r="G23" s="57">
         <v>1.10227895476947E-2</v>
       </c>
       <c r="H23" s="18">
@@ -3959,28 +4135,28 @@
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B40" s="65" t="s">
+      <c r="B40" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="C40" s="68" t="s">
+      <c r="C40" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="D40" s="68"/>
-      <c r="E40" s="68"/>
-      <c r="F40" s="68"/>
-      <c r="G40" s="65" t="s">
+      <c r="D40" s="80"/>
+      <c r="E40" s="80"/>
+      <c r="F40" s="80"/>
+      <c r="G40" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="H40" s="65" t="s">
+      <c r="H40" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="I40" s="65" t="s">
+      <c r="I40" s="77" t="s">
         <v>34</v>
       </c>
-      <c r="J40" s="67"/>
+      <c r="J40" s="79"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B41" s="65"/>
+      <c r="B41" s="77"/>
       <c r="C41" s="50" t="s">
         <v>3</v>
       </c>
@@ -3993,10 +4169,10 @@
       <c r="F41" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G41" s="65"/>
-      <c r="H41" s="65"/>
-      <c r="I41" s="65"/>
-      <c r="J41" s="67"/>
+      <c r="G41" s="77"/>
+      <c r="H41" s="77"/>
+      <c r="I41" s="77"/>
+      <c r="J41" s="79"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B42" s="2" t="s">
@@ -4110,18 +4286,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F024A9F-720A-4384-9592-EDD81D7A1CFE}">
-  <dimension ref="A1:Z21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F024A9F-720A-4384-9592-EDD81D7A1CFE}">
+  <dimension ref="A1:Z36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="37.26953125" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7265625" customWidth="1"/>
-    <col min="4" max="4" width="9.1796875" customWidth="1"/>
-    <col min="5" max="5" width="8.36328125" customWidth="1"/>
+    <col min="1" max="1" width="40.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="6.90625" customWidth="1"/>
     <col min="8" max="8" width="15.08984375" customWidth="1"/>
-    <col min="9" max="9" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.54296875" customWidth="1"/>
     <col min="10" max="10" width="12.7265625" customWidth="1"/>
     <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.26953125" bestFit="1" customWidth="1"/>
@@ -4133,1055 +4308,2695 @@
     <col min="26" max="27" width="16.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="60" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" s="60" t="s">
-        <v>45</v>
-      </c>
-      <c r="C1" s="62" t="s">
+    <row r="1" spans="1:26" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C1" s="128" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="60" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" s="60" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" s="60" t="s">
-        <v>34</v>
-      </c>
-      <c r="K1" s="62" t="s">
+      <c r="D1" s="129"/>
+      <c r="E1" s="129"/>
+      <c r="F1" s="129"/>
+      <c r="G1" s="130"/>
+      <c r="K1" s="128" t="s">
         <v>51</v>
       </c>
-      <c r="L1" s="63"/>
-      <c r="M1" s="63"/>
-      <c r="N1" s="63"/>
-      <c r="O1" s="63"/>
-      <c r="P1" s="63"/>
-      <c r="Q1" s="63"/>
-      <c r="R1" s="63"/>
-      <c r="S1" s="63"/>
-      <c r="T1" s="63"/>
-      <c r="U1" s="63"/>
-      <c r="V1" s="63"/>
-      <c r="W1" s="63"/>
-      <c r="X1" s="64"/>
+      <c r="L1" s="129"/>
+      <c r="M1" s="129"/>
+      <c r="N1" s="129"/>
+      <c r="O1" s="129"/>
+      <c r="P1" s="129"/>
+      <c r="Q1" s="129"/>
+      <c r="R1" s="129"/>
+      <c r="S1" s="129"/>
+      <c r="T1" s="129"/>
+      <c r="U1" s="129"/>
+      <c r="V1" s="129"/>
+      <c r="W1" s="129"/>
+      <c r="X1" s="131"/>
       <c r="Z1" s="55" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="61"/>
-      <c r="B2" s="61"/>
-      <c r="C2" s="57" t="s">
+    <row r="2" spans="1:26" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="133" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="132" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="98" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="57" t="s">
+      <c r="D2" s="98" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="57" t="s">
+      <c r="E2" s="98" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="57" t="s">
+      <c r="F2" s="98" t="s">
         <v>49</v>
       </c>
-      <c r="G2" s="57" t="s">
+      <c r="G2" s="98" t="s">
         <v>50</v>
       </c>
-      <c r="H2" s="61"/>
-      <c r="I2" s="61"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="82" t="s">
+      <c r="H2" s="132" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="132" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="132" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" s="99" t="s">
         <v>52</v>
       </c>
-      <c r="L2" s="82" t="s">
+      <c r="L2" s="99" t="s">
         <v>53</v>
       </c>
-      <c r="M2" s="82" t="s">
+      <c r="M2" s="99" t="s">
         <v>54</v>
       </c>
-      <c r="N2" s="79" t="s">
+      <c r="N2" s="100" t="s">
         <v>55</v>
       </c>
-      <c r="O2" s="79" t="s">
+      <c r="O2" s="100" t="s">
         <v>56</v>
       </c>
-      <c r="P2" s="79" t="s">
+      <c r="P2" s="100" t="s">
         <v>57</v>
       </c>
-      <c r="Q2" s="79" t="s">
+      <c r="Q2" s="100" t="s">
         <v>58</v>
       </c>
-      <c r="R2" s="79" t="s">
+      <c r="R2" s="100" t="s">
         <v>59</v>
       </c>
-      <c r="S2" s="79" t="s">
+      <c r="S2" s="100" t="s">
         <v>60</v>
       </c>
-      <c r="T2" s="82" t="s">
+      <c r="T2" s="99" t="s">
         <v>61</v>
       </c>
-      <c r="U2" s="82" t="s">
+      <c r="U2" s="99" t="s">
         <v>65</v>
       </c>
-      <c r="V2" s="81" t="s">
+      <c r="V2" s="101" t="s">
         <v>62</v>
       </c>
-      <c r="W2" s="82" t="s">
+      <c r="W2" s="99" t="s">
         <v>63</v>
       </c>
-      <c r="X2" s="82" t="s">
+      <c r="X2" s="102" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="9">
         <v>150</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="9">
         <v>20</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="9">
         <v>1.5</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="9">
         <v>1.5</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="9">
         <v>0.7</v>
       </c>
-      <c r="H3" s="78">
+      <c r="H3" s="9">
         <v>2.9472175802249201E-4</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="9">
         <f>60+13.49</f>
         <v>73.489999999999995</v>
       </c>
-      <c r="J3" s="51">
+      <c r="J3" s="89">
         <f>I3/60</f>
         <v>1.2248333333333332</v>
       </c>
-      <c r="K3" s="83">
+      <c r="K3" s="90">
         <v>2.1924339239705899E-2</v>
       </c>
-      <c r="L3" s="83">
+      <c r="L3" s="90">
         <v>5.3243124688619803</v>
       </c>
-      <c r="M3" s="83">
+      <c r="M3" s="90">
         <v>10</v>
       </c>
-      <c r="N3" s="80">
+      <c r="N3" s="91">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="O3" s="80">
+      <c r="O3" s="91">
         <v>8.5518540000000005</v>
       </c>
-      <c r="P3" s="80">
+      <c r="P3" s="91">
         <v>7.1656500000000003</v>
       </c>
-      <c r="Q3" s="80">
+      <c r="Q3" s="91">
         <v>44.150669999999998</v>
       </c>
-      <c r="R3" s="80">
+      <c r="R3" s="91">
         <v>42.528283999999999</v>
       </c>
-      <c r="S3" s="80">
+      <c r="S3" s="91">
         <v>1E-4</v>
       </c>
-      <c r="T3" s="83">
+      <c r="T3" s="90">
         <v>2.1598443591871601</v>
       </c>
-      <c r="U3" s="83">
+      <c r="U3" s="90">
         <v>9.4242283395423598</v>
       </c>
-      <c r="V3" s="80">
+      <c r="V3" s="91">
         <v>1.6426339999999999</v>
       </c>
-      <c r="W3" s="83">
+      <c r="W3" s="90">
         <v>0.1</v>
       </c>
-      <c r="X3" s="83">
+      <c r="X3" s="92">
         <v>0.66937281186906705</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:26" s="86" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="81">
         <v>150</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="81">
         <v>20</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="81">
         <v>1.5</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="81">
         <v>1.5</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="81">
         <v>0.7</v>
       </c>
-      <c r="H4" s="78">
-        <v>1.40375181209925E-2</v>
-      </c>
-      <c r="I4" s="2">
-        <f>60+6.44</f>
-        <v>66.44</v>
-      </c>
-      <c r="J4" s="51">
-        <f t="shared" ref="J4:J14" si="0">I4/60</f>
-        <v>1.1073333333333333</v>
-      </c>
-      <c r="K4" s="84">
-        <v>2.13935160996067</v>
-      </c>
-      <c r="L4" s="84">
-        <v>3.7720314524367198</v>
-      </c>
-      <c r="M4" s="84">
-        <v>7.0774441190072404</v>
-      </c>
-      <c r="N4" s="80">
+      <c r="H4" s="81">
+        <v>2.3513880843272501E-2</v>
+      </c>
+      <c r="I4" s="81">
+        <f>60+7.64</f>
+        <v>67.64</v>
+      </c>
+      <c r="J4" s="82">
+        <f t="shared" ref="J4" si="0">I4/60</f>
+        <v>1.1273333333333333</v>
+      </c>
+      <c r="K4" s="83">
+        <v>6.9239735242755502</v>
+      </c>
+      <c r="L4" s="83">
+        <v>1.82078102654331</v>
+      </c>
+      <c r="M4" s="83">
+        <v>9.9329324700275592</v>
+      </c>
+      <c r="N4" s="84">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="O4" s="80">
+      <c r="O4" s="84">
         <v>8.5518540000000005</v>
       </c>
-      <c r="P4" s="80">
+      <c r="P4" s="84">
         <v>7.1656500000000003</v>
       </c>
-      <c r="Q4" s="80">
+      <c r="Q4" s="84">
         <v>44.150669999999998</v>
       </c>
-      <c r="R4" s="80">
+      <c r="R4" s="84">
         <v>42.528283999999999</v>
       </c>
-      <c r="S4" s="80">
+      <c r="S4" s="84">
         <v>1E-4</v>
       </c>
-      <c r="T4" s="84">
-        <v>1.8888019984842901</v>
-      </c>
-      <c r="U4" s="84">
-        <v>6.3974765814129801</v>
-      </c>
-      <c r="V4" s="80">
+      <c r="T4" s="83">
+        <v>2.2496431130169099</v>
+      </c>
+      <c r="U4" s="83">
+        <v>3.90148636909132</v>
+      </c>
+      <c r="V4" s="84">
         <v>1.6426339999999999</v>
       </c>
-      <c r="W4" s="83">
-        <v>0.83091291134603795</v>
-      </c>
-      <c r="X4" s="83">
-        <v>0.11175654744772601</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="W4" s="85">
+        <v>1.4863468597450999</v>
+      </c>
+      <c r="X4" s="94">
+        <v>0.26736379732660398</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" s="86" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="81">
         <v>150</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="81">
         <v>20</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="81">
         <v>1.5</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="81">
         <v>1.5</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="81">
         <v>0.7</v>
       </c>
-      <c r="H5" s="78">
+      <c r="H5" s="81">
         <v>1.32701286472156E-3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="81">
         <f>5*60+48.41</f>
         <v>348.40999999999997</v>
       </c>
-      <c r="J5" s="51">
-        <f t="shared" si="0"/>
+      <c r="J5" s="126">
+        <f>I5/60</f>
         <v>5.8068333333333326</v>
       </c>
-      <c r="K5" s="84">
+      <c r="K5" s="83">
         <v>3.0051333747301801</v>
       </c>
-      <c r="L5" s="84">
+      <c r="L5" s="83">
         <v>5.0528684093825298</v>
       </c>
-      <c r="M5" s="84">
+      <c r="M5" s="83">
         <v>4.8710938159898802</v>
       </c>
-      <c r="N5" s="80">
+      <c r="N5" s="84">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="O5" s="80">
+      <c r="O5" s="84">
         <v>8.5518540000000005</v>
       </c>
-      <c r="P5" s="80">
+      <c r="P5" s="84">
         <v>7.1656500000000003</v>
       </c>
-      <c r="Q5" s="80">
+      <c r="Q5" s="84">
         <v>44.150669999999998</v>
       </c>
-      <c r="R5" s="80">
+      <c r="R5" s="84">
         <v>42.528283999999999</v>
       </c>
-      <c r="S5" s="80">
+      <c r="S5" s="84">
         <v>1E-4</v>
       </c>
-      <c r="T5" s="84">
+      <c r="T5" s="83">
         <v>1.06812478247408</v>
       </c>
-      <c r="U5" s="84">
+      <c r="U5" s="83">
         <v>3.3029168292772599</v>
       </c>
-      <c r="V5" s="80">
+      <c r="V5" s="84">
         <v>1.6426339999999999</v>
       </c>
-      <c r="W5" s="83">
+      <c r="W5" s="85">
         <v>0.29242188148853998</v>
       </c>
-      <c r="X5" s="83">
+      <c r="X5" s="94">
         <v>0.47648836606682399</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:26" s="86" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="81" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="81">
         <v>150</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="81">
         <v>20</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="81">
         <v>1.5</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="81">
         <v>1.5</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="81">
         <v>0.7</v>
       </c>
-      <c r="H6" s="78">
+      <c r="H6" s="54">
         <v>7.04873626723777E-4</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="54">
         <f>60+14.51</f>
         <v>74.510000000000005</v>
       </c>
-      <c r="J6" s="51">
-        <f t="shared" si="0"/>
+      <c r="J6" s="111">
+        <f>I6/60</f>
         <v>1.2418333333333333</v>
       </c>
-      <c r="K6" s="83">
+      <c r="K6" s="112">
         <v>0.232102232392803</v>
       </c>
-      <c r="L6" s="84">
+      <c r="L6" s="113">
         <v>4.1297069928879102</v>
       </c>
-      <c r="M6" s="84">
+      <c r="M6" s="113">
         <v>6.0078738386920403</v>
       </c>
-      <c r="N6" s="80">
+      <c r="N6" s="115">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="O6" s="80">
+      <c r="O6" s="115">
         <v>8.5518540000000005</v>
       </c>
-      <c r="P6" s="80">
+      <c r="P6" s="115">
         <v>7.1656500000000003</v>
       </c>
-      <c r="Q6" s="80">
+      <c r="Q6" s="115">
         <v>44.150669999999998</v>
       </c>
-      <c r="R6" s="80">
+      <c r="R6" s="115">
         <v>42.528283999999999</v>
       </c>
-      <c r="S6" s="80">
+      <c r="S6" s="115">
         <v>1E-4</v>
       </c>
-      <c r="T6" s="84">
+      <c r="T6" s="113">
         <v>1.1019035329447</v>
       </c>
-      <c r="U6" s="84">
+      <c r="U6" s="113">
         <v>2.97276558235572</v>
       </c>
-      <c r="V6" s="80">
+      <c r="V6" s="115">
         <v>1.6426339999999999</v>
       </c>
-      <c r="W6" s="83">
+      <c r="W6" s="112">
         <v>0.20748440650441199</v>
       </c>
-      <c r="X6" s="83">
+      <c r="X6" s="114">
         <v>0.59401552721599604</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:26" s="86" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="81" t="s">
         <v>66</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="81">
         <v>200</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="81">
         <v>20</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="81">
         <v>1.5</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="81">
         <v>1.5</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="81">
         <v>0.7</v>
       </c>
-      <c r="H7" s="78">
+      <c r="H7" s="81">
         <v>2.9328842498517401E-4</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="81">
         <f>60+15.12</f>
         <v>75.12</v>
       </c>
-      <c r="J7" s="51">
-        <f t="shared" si="0"/>
+      <c r="J7" s="82">
+        <f>I7/60</f>
         <v>1.252</v>
       </c>
-      <c r="K7" s="83">
+      <c r="K7" s="85">
         <v>2.1763903293888599E-2</v>
       </c>
-      <c r="L7" s="83">
+      <c r="L7" s="85">
         <v>5.3320005646842601</v>
       </c>
-      <c r="M7" s="83">
+      <c r="M7" s="85">
         <v>10</v>
       </c>
-      <c r="N7" s="80">
+      <c r="N7" s="84">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="O7" s="80">
+      <c r="O7" s="84">
         <v>8.5518540000000005</v>
       </c>
-      <c r="P7" s="80">
+      <c r="P7" s="84">
         <v>7.1656500000000003</v>
       </c>
-      <c r="Q7" s="80">
+      <c r="Q7" s="84">
         <v>44.150669999999998</v>
       </c>
-      <c r="R7" s="80">
+      <c r="R7" s="84">
         <v>42.528283999999999</v>
       </c>
-      <c r="S7" s="80">
+      <c r="S7" s="84">
         <v>1E-4</v>
       </c>
-      <c r="T7" s="84">
+      <c r="T7" s="83">
         <v>2.7464836815839999</v>
       </c>
-      <c r="U7" s="84">
+      <c r="U7" s="83">
         <v>9.4217689488491896</v>
       </c>
-      <c r="V7" s="80">
+      <c r="V7" s="84">
         <v>1.6426339999999999</v>
       </c>
-      <c r="W7" s="83">
+      <c r="W7" s="85">
         <v>0.1</v>
       </c>
-      <c r="X7" s="83">
+      <c r="X7" s="94">
         <v>0.66954694007881499</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:26" s="86" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="81">
         <v>200</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="81">
         <v>20</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="81">
         <v>1.5</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="81">
         <v>1.5</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="81">
         <v>0.7</v>
       </c>
-      <c r="H8" s="86">
-        <v>3.3229795416845E-3</v>
-      </c>
-      <c r="I8" s="2">
-        <f>60+30.34</f>
-        <v>90.34</v>
-      </c>
-      <c r="J8" s="51">
-        <f t="shared" si="0"/>
-        <v>1.5056666666666667</v>
-      </c>
-      <c r="K8" s="84">
-        <v>5.3708635632974699</v>
-      </c>
-      <c r="L8" s="84">
-        <v>1.91711370869458</v>
-      </c>
-      <c r="M8" s="84">
-        <v>1.21894257791956</v>
-      </c>
-      <c r="N8" s="80">
+      <c r="H8" s="87">
+        <v>2.3513880843272501E-2</v>
+      </c>
+      <c r="I8" s="81">
+        <f>60+31.97</f>
+        <v>91.97</v>
+      </c>
+      <c r="J8" s="82">
+        <f>I8/60</f>
+        <v>1.5328333333333333</v>
+      </c>
+      <c r="K8" s="83">
+        <v>6.9239735242755502</v>
+      </c>
+      <c r="L8" s="83">
+        <v>1.82078102654331</v>
+      </c>
+      <c r="M8" s="83">
+        <v>9.9329324700275592</v>
+      </c>
+      <c r="N8" s="84">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="O8" s="80">
+      <c r="O8" s="84">
         <v>8.5518540000000005</v>
       </c>
-      <c r="P8" s="80">
+      <c r="P8" s="84">
         <v>7.1656500000000003</v>
       </c>
-      <c r="Q8" s="80">
+      <c r="Q8" s="84">
         <v>44.150669999999998</v>
       </c>
-      <c r="R8" s="80">
+      <c r="R8" s="84">
         <v>42.528283999999999</v>
       </c>
-      <c r="S8" s="80">
+      <c r="S8" s="84">
         <v>1E-4</v>
       </c>
-      <c r="T8" s="84">
-        <v>5.0621300467977699</v>
-      </c>
-      <c r="U8" s="84">
-        <v>4.3662737525307698</v>
-      </c>
-      <c r="V8" s="80">
+      <c r="T8" s="83">
+        <v>2.2496431130169099</v>
+      </c>
+      <c r="U8" s="83">
+        <v>3.90148636909132</v>
+      </c>
+      <c r="V8" s="84">
         <v>1.6426339999999999</v>
       </c>
-      <c r="W8" s="83">
-        <v>0.32173344505856499</v>
-      </c>
-      <c r="X8" s="83">
-        <v>0.41579920796990599</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+      <c r="W8" s="85">
+        <v>1.4863468597450999</v>
+      </c>
+      <c r="X8" s="94">
+        <v>0.26736379732660398</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" s="86" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="81">
         <v>200</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="81">
         <v>20</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="81">
         <v>1.5</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="81">
         <v>1.5</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="81">
         <v>0.7</v>
       </c>
-      <c r="H9" s="78">
+      <c r="H9" s="81">
         <v>1.3251362658287199E-3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="81">
         <f>60*7+25.26</f>
         <v>445.26</v>
       </c>
-      <c r="J9" s="51">
-        <f t="shared" si="0"/>
+      <c r="J9" s="126">
+        <f>I9/60</f>
         <v>7.4210000000000003</v>
       </c>
-      <c r="K9" s="84">
+      <c r="K9" s="83">
         <v>3.01506522825153</v>
       </c>
-      <c r="L9" s="84">
+      <c r="L9" s="83">
         <v>5.05925344685207</v>
       </c>
-      <c r="M9" s="83">
+      <c r="M9" s="85">
         <v>4.86872801688311</v>
       </c>
-      <c r="N9" s="80">
+      <c r="N9" s="84">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="O9" s="80">
+      <c r="O9" s="84">
         <v>8.5518540000000005</v>
       </c>
-      <c r="P9" s="80">
+      <c r="P9" s="84">
         <v>7.1656500000000003</v>
       </c>
-      <c r="Q9" s="80">
+      <c r="Q9" s="84">
         <v>44.150669999999998</v>
       </c>
-      <c r="R9" s="80">
+      <c r="R9" s="84">
         <v>42.528283999999999</v>
       </c>
-      <c r="S9" s="80">
+      <c r="S9" s="84">
         <v>1E-4</v>
       </c>
-      <c r="T9" s="84">
+      <c r="T9" s="83">
         <v>1.06792904742284</v>
       </c>
-      <c r="U9" s="84">
+      <c r="U9" s="83">
         <v>3.30384536377028</v>
       </c>
-      <c r="V9" s="80">
+      <c r="V9" s="84">
         <v>1.6426339999999999</v>
       </c>
-      <c r="W9" s="83">
+      <c r="W9" s="85">
         <v>0.29253732272668498</v>
       </c>
-      <c r="X9" s="83">
+      <c r="X9" s="94">
         <v>0.47645758028965701</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:26" s="86" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="81" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="81">
         <v>200</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="81">
         <v>20</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="81">
         <v>1.5</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="81">
         <v>1.5</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="81">
         <v>0.7</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="54">
         <v>7.04243140314323E-4</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="54">
         <f>60+30.12</f>
         <v>90.12</v>
       </c>
-      <c r="J10" s="51">
-        <f t="shared" si="0"/>
+      <c r="J10" s="111">
+        <f>I10/60</f>
         <v>1.502</v>
       </c>
-      <c r="K10" s="83">
+      <c r="K10" s="112">
         <v>0.23198883475251</v>
       </c>
-      <c r="L10" s="83">
+      <c r="L10" s="112">
         <v>4.13163737355673</v>
       </c>
-      <c r="M10" s="83">
+      <c r="M10" s="112">
         <v>6.0033822043910199</v>
       </c>
-      <c r="N10" s="80">
+      <c r="N10" s="115">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="O10" s="80">
+      <c r="O10" s="115">
         <v>8.5518540000000005</v>
       </c>
-      <c r="P10" s="80">
+      <c r="P10" s="115">
         <v>7.1656500000000003</v>
       </c>
-      <c r="Q10" s="80">
+      <c r="Q10" s="115">
         <v>44.150669999999998</v>
       </c>
-      <c r="R10" s="80">
+      <c r="R10" s="115">
         <v>42.528283999999999</v>
       </c>
-      <c r="S10" s="80">
+      <c r="S10" s="115">
         <v>1E-4</v>
       </c>
-      <c r="T10" s="84">
+      <c r="T10" s="113">
         <v>1.10164214051543</v>
       </c>
-      <c r="U10" s="84">
+      <c r="U10" s="113">
         <v>3.12238469928359</v>
       </c>
-      <c r="V10" s="80">
+      <c r="V10" s="115">
         <v>1.6426339999999999</v>
       </c>
-      <c r="W10" s="83">
+      <c r="W10" s="112">
         <v>0.207546998368103</v>
       </c>
-      <c r="X10" s="83">
+      <c r="X10" s="114">
         <v>0.59565351370611197</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:26" s="86" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="81" t="s">
         <v>66</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="81">
         <v>500</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="81">
         <v>20</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="81">
         <v>1.5</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="81">
         <v>1.5</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="81">
         <v>0.7</v>
       </c>
-      <c r="H11" s="2">
-        <v>0</v>
-      </c>
-      <c r="I11" s="2">
-        <v>0</v>
-      </c>
-      <c r="J11" s="51">
-        <f t="shared" si="0"/>
-        <v>0</v>
+      <c r="H11" s="81">
+        <v>2.9106327802450499E-4</v>
+      </c>
+      <c r="I11" s="81">
+        <f>3*60+9.3</f>
+        <v>189.3</v>
+      </c>
+      <c r="J11" s="82">
+        <f>I11/60</f>
+        <v>3.1550000000000002</v>
       </c>
       <c r="K11" s="85">
-        <v>0</v>
+        <v>2.1502308919205501E-2</v>
       </c>
       <c r="L11" s="85">
-        <v>0</v>
+        <v>5.3545334420611397</v>
       </c>
       <c r="M11" s="85">
-        <v>0</v>
-      </c>
-      <c r="N11" s="80">
+        <v>10</v>
+      </c>
+      <c r="N11" s="84">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="O11" s="80">
+      <c r="O11" s="84">
         <v>8.5518540000000005</v>
       </c>
-      <c r="P11" s="80">
+      <c r="P11" s="84">
         <v>7.1656500000000003</v>
       </c>
-      <c r="Q11" s="80">
+      <c r="Q11" s="84">
         <v>44.150669999999998</v>
       </c>
-      <c r="R11" s="80">
+      <c r="R11" s="84">
         <v>42.528283999999999</v>
       </c>
-      <c r="S11" s="80">
+      <c r="S11" s="84">
         <v>1E-4</v>
       </c>
       <c r="T11" s="85">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U11" s="85">
-        <v>0</v>
-      </c>
-      <c r="V11" s="80">
+        <v>9.5278443260242494</v>
+      </c>
+      <c r="V11" s="84">
         <v>1.6426339999999999</v>
       </c>
       <c r="W11" s="85">
-        <v>0</v>
-      </c>
-      <c r="X11" s="85">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+        <v>0.1</v>
+      </c>
+      <c r="X11" s="94">
+        <v>0.66792358972713495</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" s="86" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="81">
         <v>500</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="81">
         <v>20</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="81">
         <v>1.5</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="81">
         <v>1.5</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="81">
         <v>0.7</v>
       </c>
-      <c r="H12" s="2">
-        <v>0</v>
-      </c>
-      <c r="I12" s="2">
-        <v>0</v>
-      </c>
-      <c r="J12" s="51">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K12" s="85">
-        <v>0</v>
-      </c>
-      <c r="L12" s="85">
-        <v>0</v>
-      </c>
-      <c r="M12" s="85">
-        <v>0</v>
-      </c>
-      <c r="N12" s="80">
+      <c r="H12" s="87">
+        <v>1.24794971393778E-2</v>
+      </c>
+      <c r="I12" s="81">
+        <f>3*60+43.91</f>
+        <v>223.91</v>
+      </c>
+      <c r="J12" s="82">
+        <f>I12/60</f>
+        <v>3.7318333333333333</v>
+      </c>
+      <c r="K12" s="83">
+        <v>5.0791991043726403</v>
+      </c>
+      <c r="L12" s="83">
+        <v>3.6404145364723002</v>
+      </c>
+      <c r="M12" s="83">
+        <v>5.9324971501398496</v>
+      </c>
+      <c r="N12" s="84">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="O12" s="80">
+      <c r="O12" s="84">
         <v>8.5518540000000005</v>
       </c>
-      <c r="P12" s="80">
+      <c r="P12" s="84">
         <v>7.1656500000000003</v>
       </c>
-      <c r="Q12" s="80">
+      <c r="Q12" s="84">
         <v>44.150669999999998</v>
       </c>
-      <c r="R12" s="80">
+      <c r="R12" s="84">
         <v>42.528283999999999</v>
       </c>
-      <c r="S12" s="80">
+      <c r="S12" s="84">
         <v>1E-4</v>
       </c>
-      <c r="T12" s="85">
-        <v>0</v>
-      </c>
-      <c r="U12" s="85">
-        <v>0</v>
-      </c>
-      <c r="V12" s="80">
+      <c r="T12" s="83">
+        <v>1.6798296474043799</v>
+      </c>
+      <c r="U12" s="83">
+        <v>3.95284452016142</v>
+      </c>
+      <c r="V12" s="84">
         <v>1.6426339999999999</v>
       </c>
       <c r="W12" s="85">
-        <v>0</v>
-      </c>
-      <c r="X12" s="85">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+        <v>1.48319268692199</v>
+      </c>
+      <c r="X12" s="94">
+        <v>0.10854293257686699</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" s="86" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="81">
         <v>500</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="81">
         <v>20</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="81">
         <v>1.5</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F13" s="81">
         <v>1.5</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="81">
         <v>0.7</v>
       </c>
-      <c r="H13" s="2">
-        <v>0</v>
-      </c>
-      <c r="I13" s="2">
-        <v>0</v>
-      </c>
-      <c r="J13" s="51">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K13" s="85">
-        <v>0</v>
-      </c>
-      <c r="L13" s="85">
-        <v>0</v>
-      </c>
-      <c r="M13" s="85">
-        <v>0</v>
-      </c>
-      <c r="N13" s="80">
+      <c r="H13" s="81">
+        <v>1.22828604596883E-3</v>
+      </c>
+      <c r="I13" s="81">
+        <f>20*60+26.29</f>
+        <v>1226.29</v>
+      </c>
+      <c r="J13" s="126">
+        <f>I13/60</f>
+        <v>20.438166666666667</v>
+      </c>
+      <c r="K13" s="83">
+        <v>1.10577438138983</v>
+      </c>
+      <c r="L13" s="83">
+        <v>7.8360003082510898</v>
+      </c>
+      <c r="M13" s="83">
+        <v>1.6052788739111301</v>
+      </c>
+      <c r="N13" s="84">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="O13" s="80">
+      <c r="O13" s="84">
         <v>8.5518540000000005</v>
       </c>
-      <c r="P13" s="80">
+      <c r="P13" s="84">
         <v>7.1656500000000003</v>
       </c>
-      <c r="Q13" s="80">
+      <c r="Q13" s="84">
         <v>44.150669999999998</v>
       </c>
-      <c r="R13" s="80">
+      <c r="R13" s="84">
         <v>42.528283999999999</v>
       </c>
-      <c r="S13" s="80">
+      <c r="S13" s="84">
         <v>1E-4</v>
       </c>
-      <c r="T13" s="85">
-        <v>0</v>
-      </c>
-      <c r="U13" s="85">
-        <v>0</v>
-      </c>
-      <c r="V13" s="80">
+      <c r="T13" s="83">
+        <v>1.2822673368615201</v>
+      </c>
+      <c r="U13" s="88">
+        <v>0.65248550329617405</v>
+      </c>
+      <c r="V13" s="84">
         <v>1.6426339999999999</v>
       </c>
       <c r="W13" s="85">
-        <v>0</v>
-      </c>
-      <c r="X13" s="85">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+        <v>0.51457518879894604</v>
+      </c>
+      <c r="X13" s="95">
+        <v>0.14428420432665601</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" s="86" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="81" t="s">
         <v>70</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="81">
         <v>500</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="81">
         <v>20</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="81">
         <v>1.5</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="81">
         <v>1.5</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="81">
         <v>0.7</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="54">
         <v>7.0311620720228901E-4</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="54">
         <f>4*60+9.5</f>
         <v>249.5</v>
       </c>
-      <c r="J14" s="51">
-        <f t="shared" si="0"/>
+      <c r="J14" s="111">
+        <f>I14/60</f>
         <v>4.1583333333333332</v>
       </c>
-      <c r="K14" s="83">
+      <c r="K14" s="112">
         <v>0.230277928812854</v>
       </c>
-      <c r="L14" s="84">
+      <c r="L14" s="113">
         <v>4.1471160732970196</v>
       </c>
-      <c r="M14" s="84">
+      <c r="M14" s="113">
         <v>6.0025562868090301</v>
       </c>
-      <c r="N14" s="80">
+      <c r="N14" s="115">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="O14" s="80">
+      <c r="O14" s="115">
         <v>8.5518540000000005</v>
       </c>
-      <c r="P14" s="80">
+      <c r="P14" s="115">
         <v>7.1656500000000003</v>
       </c>
-      <c r="Q14" s="80">
+      <c r="Q14" s="115">
         <v>44.150669999999998</v>
       </c>
-      <c r="R14" s="80">
+      <c r="R14" s="115">
         <v>42.528283999999999</v>
       </c>
-      <c r="S14" s="80">
+      <c r="S14" s="115">
         <v>1E-4</v>
       </c>
-      <c r="T14" s="84">
+      <c r="T14" s="113">
         <v>1.1015287199813399</v>
       </c>
-      <c r="U14" s="84">
+      <c r="U14" s="113">
         <v>2.49443328688508</v>
       </c>
-      <c r="V14" s="80">
+      <c r="V14" s="115">
         <v>1.6426339999999999</v>
       </c>
-      <c r="W14" s="83">
+      <c r="W14" s="112">
         <v>0.20757536882927899</v>
       </c>
-      <c r="X14" s="83">
+      <c r="X14" s="114">
         <v>0.59564622966884795</v>
       </c>
     </row>
+    <row r="15" spans="1:26" s="86" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="96" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="97" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" s="97">
+        <v>500</v>
+      </c>
+      <c r="D15" s="97">
+        <v>25</v>
+      </c>
+      <c r="E15" s="97">
+        <v>1.5</v>
+      </c>
+      <c r="F15" s="97">
+        <v>1.5</v>
+      </c>
+      <c r="G15" s="97">
+        <v>0.7</v>
+      </c>
+      <c r="H15" s="104">
+        <v>6.7861314633885098E-4</v>
+      </c>
+      <c r="I15" s="104">
+        <f>4*60+45.45</f>
+        <v>285.45</v>
+      </c>
+      <c r="J15" s="116">
+        <f>I15/60</f>
+        <v>4.7574999999999994</v>
+      </c>
+      <c r="K15" s="117">
+        <v>0.65584707161238898</v>
+      </c>
+      <c r="L15" s="118">
+        <v>1.6542627156257601</v>
+      </c>
+      <c r="M15" s="117">
+        <v>0.935993228967127</v>
+      </c>
+      <c r="N15" s="119">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O15" s="119">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P15" s="119">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q15" s="119">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R15" s="119">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S15" s="119">
+        <v>1E-4</v>
+      </c>
+      <c r="T15" s="118">
+        <v>6.3300111014726497</v>
+      </c>
+      <c r="U15" s="117">
+        <v>0.97696229125558598</v>
+      </c>
+      <c r="V15" s="119">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W15" s="117">
+        <v>0.351566393361611</v>
+      </c>
+      <c r="X15" s="120">
+        <v>0.40093322956893201</v>
+      </c>
+    </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="8" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A17" s="2"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" s="2"/>
-      <c r="H18" s="87"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
+      <c r="B16" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="9">
+        <v>150</v>
+      </c>
+      <c r="D16" s="9">
+        <v>20</v>
+      </c>
+      <c r="E16" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="F16" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="G16" s="9">
+        <v>0.7</v>
+      </c>
+      <c r="H16" s="9">
+        <v>1.11440624623557E-2</v>
+      </c>
+      <c r="I16" s="9">
+        <f>4*60+18.28</f>
+        <v>258.27999999999997</v>
+      </c>
+      <c r="J16" s="89">
+        <f>I16/60</f>
+        <v>4.304666666666666</v>
+      </c>
+      <c r="K16" s="105">
+        <v>2.3299381559274899</v>
+      </c>
+      <c r="L16" s="105">
+        <v>5.32287018685438</v>
+      </c>
+      <c r="M16" s="105">
+        <v>7.98243204684095</v>
+      </c>
+      <c r="N16" s="91">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O16" s="91">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P16" s="91">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q16" s="91">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R16" s="91">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S16" s="91">
+        <v>1E-4</v>
+      </c>
+      <c r="T16" s="90">
+        <v>0.17054697044964001</v>
+      </c>
+      <c r="U16" s="105">
+        <v>7.0897163559782097</v>
+      </c>
+      <c r="V16" s="91">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W16" s="106">
+        <v>0.47501878724573199</v>
+      </c>
+      <c r="X16" s="107">
+        <v>0.34154452509892902</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A17" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="81" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="81">
+        <v>150</v>
+      </c>
+      <c r="D17" s="81">
+        <v>20</v>
+      </c>
+      <c r="E17" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F17" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G17" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H17" s="2">
+        <v>3.3679725400876E-2</v>
+      </c>
+      <c r="I17" s="2">
+        <f>2*60+53.1</f>
+        <v>173.1</v>
+      </c>
+      <c r="J17" s="103">
+        <f t="shared" ref="J17:J25" si="1">I17/60</f>
+        <v>2.8849999999999998</v>
+      </c>
+      <c r="K17" s="60">
+        <v>3.8814631810598001</v>
+      </c>
+      <c r="L17" s="60">
+        <v>2.8667225940990999</v>
+      </c>
+      <c r="M17" s="60">
+        <v>6.8650101407296198</v>
+      </c>
+      <c r="N17" s="84">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O17" s="84">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P17" s="84">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q17" s="84">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R17" s="84">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S17" s="84">
+        <v>1E-4</v>
+      </c>
+      <c r="T17" s="60">
+        <v>1.16026489040905</v>
+      </c>
+      <c r="U17" s="60">
+        <v>5.8389022640940498</v>
+      </c>
+      <c r="V17" s="84">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W17" s="61">
+        <v>0.64665747418014496</v>
+      </c>
+      <c r="X17" s="108">
+        <v>0.204067557379424</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A18" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="81" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="81">
+        <v>150</v>
+      </c>
+      <c r="D18" s="81">
+        <v>20</v>
+      </c>
+      <c r="E18" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F18" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G18" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H18" s="109">
+        <v>1.15359229420309E-2</v>
+      </c>
+      <c r="I18" s="2">
+        <f>31*60+32.58</f>
+        <v>1892.58</v>
+      </c>
+      <c r="J18" s="110">
+        <f t="shared" si="1"/>
+        <v>31.542999999999999</v>
+      </c>
+      <c r="K18" s="60">
+        <v>4.66126484420837</v>
+      </c>
+      <c r="L18" s="60">
+        <v>7.6274459060809496</v>
+      </c>
+      <c r="M18" s="59">
+        <v>3.93887006942419</v>
+      </c>
+      <c r="N18" s="84">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O18" s="84">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P18" s="84">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q18" s="84">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R18" s="84">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S18" s="84">
+        <v>1E-4</v>
+      </c>
+      <c r="T18" s="61">
+        <v>0.17179967183183001</v>
+      </c>
+      <c r="U18" s="60">
+        <v>4.8454643039093703</v>
+      </c>
+      <c r="V18" s="84">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W18" s="61">
+        <v>0.71125671544458102</v>
+      </c>
+      <c r="X18" s="108">
+        <v>0.13681289788651901</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A19" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="81">
+        <v>150</v>
+      </c>
+      <c r="D19" s="81">
+        <v>20</v>
+      </c>
+      <c r="E19" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F19" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G19" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H19" s="57">
+        <v>1.1953798058781E-3</v>
+      </c>
+      <c r="I19" s="54">
+        <f>5*60+28.86</f>
+        <v>328.86</v>
+      </c>
+      <c r="J19" s="121">
+        <f t="shared" si="1"/>
+        <v>5.4809999999999999</v>
+      </c>
+      <c r="K19" s="112">
+        <v>8.6968657160830798E-2</v>
+      </c>
+      <c r="L19" s="112">
+        <v>0.37972652190723399</v>
+      </c>
+      <c r="M19" s="113">
+        <v>1.8859295434347501</v>
+      </c>
+      <c r="N19" s="115">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O19" s="115">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P19" s="115">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q19" s="115">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R19" s="115">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S19" s="115">
+        <v>1E-4</v>
+      </c>
+      <c r="T19" s="113">
+        <v>9.2643799195858598</v>
+      </c>
+      <c r="U19" s="113">
+        <v>9.9263324663812593</v>
+      </c>
+      <c r="V19" s="115">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W19" s="122">
+        <v>0.14259670949258901</v>
+      </c>
+      <c r="X19" s="123">
+        <v>0.67266227300008097</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A20" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="81" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="81">
+        <v>200</v>
+      </c>
+      <c r="D20" s="81">
+        <v>20</v>
+      </c>
+      <c r="E20" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F20" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G20" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H20" s="2">
+        <v>1.1136767684926699E-2</v>
+      </c>
+      <c r="I20" s="2">
+        <f>5*60+3.26</f>
+        <v>303.26</v>
+      </c>
+      <c r="J20" s="103">
+        <f t="shared" si="1"/>
+        <v>5.0543333333333331</v>
+      </c>
+      <c r="K20" s="60">
+        <v>2.40418844091263</v>
+      </c>
+      <c r="L20" s="60">
+        <v>5.3229813301373197</v>
+      </c>
+      <c r="M20" s="60">
+        <v>8.0155017949921401</v>
+      </c>
+      <c r="N20" s="84">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O20" s="84">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P20" s="84">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q20" s="84">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R20" s="84">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S20" s="84">
+        <v>1E-4</v>
+      </c>
+      <c r="T20" s="61">
+        <v>0.17047414015068499</v>
+      </c>
+      <c r="U20" s="60">
+        <v>7.0922970703933199</v>
+      </c>
+      <c r="V20" s="84">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W20" s="61">
+        <v>0.476047570705943</v>
+      </c>
+      <c r="X20" s="108">
+        <v>0.34404791544767399</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A21" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" s="81" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="81">
+        <v>200</v>
+      </c>
+      <c r="D21" s="81">
+        <v>20</v>
+      </c>
+      <c r="E21" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F21" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G21" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H21" s="2">
+        <v>3.3679725400876E-2</v>
+      </c>
+      <c r="I21" s="2">
+        <f>3*60+53.73</f>
+        <v>233.73</v>
+      </c>
+      <c r="J21" s="103">
+        <f t="shared" si="1"/>
+        <v>3.8954999999999997</v>
+      </c>
+      <c r="K21" s="60">
+        <v>3.8814631810598001</v>
+      </c>
+      <c r="L21" s="60">
+        <v>2.8667225940990999</v>
+      </c>
+      <c r="M21" s="60">
+        <v>6.8650101407296198</v>
+      </c>
+      <c r="N21" s="84">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O21" s="84">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P21" s="84">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q21" s="84">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R21" s="84">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S21" s="84">
+        <v>1E-4</v>
+      </c>
+      <c r="T21" s="60">
+        <v>1.16026489040905</v>
+      </c>
+      <c r="U21" s="60">
+        <v>5.8389022640940498</v>
+      </c>
+      <c r="V21" s="84">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W21" s="61">
+        <v>0.64665747418014496</v>
+      </c>
+      <c r="X21" s="108">
+        <v>0.204067557379424</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A22" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" s="81">
+        <v>200</v>
+      </c>
+      <c r="D22" s="81">
+        <v>20</v>
+      </c>
+      <c r="E22" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F22" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G22" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H22" s="54">
+        <v>1.1445614822087899E-3</v>
+      </c>
+      <c r="I22" s="54">
+        <f>11*60+48.17</f>
+        <v>708.17</v>
+      </c>
+      <c r="J22" s="121">
+        <f t="shared" si="1"/>
+        <v>11.802833333333332</v>
+      </c>
+      <c r="K22" s="112">
+        <v>9.7748777956490701E-2</v>
+      </c>
+      <c r="L22" s="112">
+        <v>0.33917373382219301</v>
+      </c>
+      <c r="M22" s="113">
+        <v>1.76771463748577</v>
+      </c>
+      <c r="N22" s="115">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O22" s="115">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P22" s="115">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q22" s="115">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R22" s="115">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S22" s="115">
+        <v>1E-4</v>
+      </c>
+      <c r="T22" s="113">
+        <v>9.9823011023231398</v>
+      </c>
+      <c r="U22" s="113">
+        <v>9.8388752079463302</v>
+      </c>
+      <c r="V22" s="115">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W22" s="122">
+        <v>0.144298087346836</v>
+      </c>
+      <c r="X22" s="123">
+        <v>0.67235045686653305</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A23" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="81" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" s="81">
+        <v>500</v>
+      </c>
+      <c r="D23" s="81">
+        <v>20</v>
+      </c>
+      <c r="E23" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F23" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G23" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H23" s="2">
+        <v>2.1153082388360899E-2</v>
+      </c>
+      <c r="I23" s="2">
+        <f>11*60+34.96</f>
+        <v>694.96</v>
+      </c>
+      <c r="J23" s="103">
+        <f t="shared" si="1"/>
+        <v>11.582666666666666</v>
+      </c>
+      <c r="K23" s="60">
+        <v>4.6003553841105704</v>
+      </c>
+      <c r="L23" s="60">
+        <v>2.9392767866460798</v>
+      </c>
+      <c r="M23" s="60">
+        <v>1.8114258287038001</v>
+      </c>
+      <c r="N23" s="84">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O23" s="84">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P23" s="84">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q23" s="84">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R23" s="84">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S23" s="84">
+        <v>1E-4</v>
+      </c>
+      <c r="T23" s="60">
+        <v>2.72866349573804</v>
+      </c>
+      <c r="U23" s="60">
+        <v>5.4387748973149801</v>
+      </c>
+      <c r="V23" s="84">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W23" s="61">
+        <v>0.52946081224504704</v>
+      </c>
+      <c r="X23" s="108">
+        <v>0.37852014574272003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A24" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="81">
+        <v>500</v>
+      </c>
+      <c r="D24" s="81">
+        <v>20</v>
+      </c>
+      <c r="E24" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F24" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G24" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H24" s="54">
+        <v>1.14236097186321E-3</v>
+      </c>
+      <c r="I24" s="54">
+        <f>19*60+15.09</f>
+        <v>1155.0899999999999</v>
+      </c>
+      <c r="J24" s="121">
+        <f t="shared" si="1"/>
+        <v>19.2515</v>
+      </c>
+      <c r="K24" s="112">
+        <v>9.7556289800075593E-2</v>
+      </c>
+      <c r="L24" s="112">
+        <v>0.33789906227527899</v>
+      </c>
+      <c r="M24" s="113">
+        <v>1.7766564066399899</v>
+      </c>
+      <c r="N24" s="115">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O24" s="115">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P24" s="115">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q24" s="115">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R24" s="115">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S24" s="115">
+        <v>1E-4</v>
+      </c>
+      <c r="T24" s="113">
+        <v>9.9987954209152292</v>
+      </c>
+      <c r="U24" s="113">
+        <v>9.9698073558070508</v>
+      </c>
+      <c r="V24" s="115">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W24" s="122">
+        <v>0.144349858891552</v>
+      </c>
+      <c r="X24" s="123">
+        <v>0.67196429289183002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="97" t="s">
+        <v>70</v>
+      </c>
+      <c r="C25" s="97">
+        <v>500</v>
+      </c>
+      <c r="D25" s="97">
+        <v>25</v>
+      </c>
+      <c r="E25" s="97">
+        <v>1.5</v>
+      </c>
+      <c r="F25" s="97">
+        <v>1.5</v>
+      </c>
+      <c r="G25" s="97">
+        <v>0.7</v>
+      </c>
+      <c r="H25" s="104">
+        <v>1.1658027202459599E-3</v>
+      </c>
+      <c r="I25" s="104">
+        <f>30*60+57.34</f>
+        <v>1857.34</v>
+      </c>
+      <c r="J25" s="124">
+        <f t="shared" si="1"/>
+        <v>30.955666666666666</v>
+      </c>
+      <c r="K25" s="117">
+        <v>9.7800415721008199E-2</v>
+      </c>
+      <c r="L25" s="117">
+        <v>0.71140617768074599</v>
+      </c>
+      <c r="M25" s="118">
+        <v>1.4257677322081099</v>
+      </c>
+      <c r="N25" s="119">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O25" s="119">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P25" s="119">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q25" s="119">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R25" s="119">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S25" s="119">
+        <v>1E-4</v>
+      </c>
+      <c r="T25" s="118">
+        <v>9.9977821280604804</v>
+      </c>
+      <c r="U25" s="118">
+        <v>6.5776873288542603</v>
+      </c>
+      <c r="V25" s="119">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W25" s="125">
+        <v>0.28729463418919698</v>
+      </c>
+      <c r="X25" s="127">
+        <v>0.52605879996048899</v>
+      </c>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A26" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="2"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" s="2"/>
+      <c r="B26" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="9">
+        <v>150</v>
+      </c>
+      <c r="D26" s="9">
+        <v>20</v>
+      </c>
+      <c r="E26" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="F26" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="G26" s="9">
+        <v>0.7</v>
+      </c>
+      <c r="H26" s="9">
+        <v>5.3784901232232596E-4</v>
+      </c>
+      <c r="I26" s="9">
+        <f>2*60+13.15</f>
+        <v>133.15</v>
+      </c>
+      <c r="J26" s="89">
+        <f>I26/60</f>
+        <v>2.2191666666666667</v>
+      </c>
+      <c r="K26" s="90">
+        <v>0.15796536035747399</v>
+      </c>
+      <c r="L26" s="105">
+        <v>4.0428520216839896</v>
+      </c>
+      <c r="M26" s="105">
+        <v>2.0987315453039099</v>
+      </c>
+      <c r="N26" s="91">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O26" s="91">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P26" s="91">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q26" s="91">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R26" s="91">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S26" s="91">
+        <v>1E-4</v>
+      </c>
+      <c r="T26" s="105">
+        <v>1.53299889476935</v>
+      </c>
+      <c r="U26" s="90">
+        <v>0.1</v>
+      </c>
+      <c r="V26" s="91">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W26" s="134">
+        <v>0.63770630487170998</v>
+      </c>
+      <c r="X26" s="107">
+        <v>0.257882208313367</v>
+      </c>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A27" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B27" s="81" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27" s="81">
+        <v>150</v>
+      </c>
+      <c r="D27" s="81">
+        <v>20</v>
+      </c>
+      <c r="E27" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F27" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G27" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H27" s="2">
+        <v>4.1148524856419004E-3</v>
+      </c>
+      <c r="I27" s="2">
+        <f>2*60+27.22</f>
+        <v>147.22</v>
+      </c>
+      <c r="J27" s="51">
+        <f>I27/60</f>
+        <v>2.4536666666666664</v>
+      </c>
+      <c r="K27" s="60">
+        <v>2.6203392577086202</v>
+      </c>
+      <c r="L27" s="60">
+        <v>1.1689487871134601</v>
+      </c>
+      <c r="M27" s="60">
+        <v>2.7977499112585198</v>
+      </c>
+      <c r="N27" s="84">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O27" s="84">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P27" s="84">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q27" s="84">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R27" s="84">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S27" s="84">
+        <v>1E-4</v>
+      </c>
+      <c r="T27" s="60">
+        <v>3.6733434323474299</v>
+      </c>
+      <c r="U27" s="60">
+        <v>1.39120350584148</v>
+      </c>
+      <c r="V27" s="84">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W27" s="135">
+        <v>1.00692090223985</v>
+      </c>
+      <c r="X27" s="108">
+        <v>0.30911593462982501</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A28" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B28" s="81" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="81">
+        <v>150</v>
+      </c>
+      <c r="D28" s="81">
+        <v>20</v>
+      </c>
+      <c r="E28" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F28" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G28" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H28" s="2">
+        <v>1.44192320669159E-3</v>
+      </c>
+      <c r="I28" s="2">
+        <f>29*60+9.65</f>
+        <v>1749.65</v>
+      </c>
+      <c r="J28" s="126">
+        <f t="shared" ref="J28:J35" si="2">I28/60</f>
+        <v>29.160833333333336</v>
+      </c>
+      <c r="K28" s="59">
+        <v>0.45522379527423301</v>
+      </c>
+      <c r="L28" s="60">
+        <v>2.1090735652864701</v>
+      </c>
+      <c r="M28" s="59">
+        <v>0.60134452548395001</v>
+      </c>
+      <c r="N28" s="84">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O28" s="84">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P28" s="84">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q28" s="84">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R28" s="84">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S28" s="84">
+        <v>1E-4</v>
+      </c>
+      <c r="T28" s="60">
+        <v>3.1990570598648702</v>
+      </c>
+      <c r="U28" s="60">
+        <v>9.3289686834751908</v>
+      </c>
+      <c r="V28" s="84">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W28" s="61">
+        <v>0.76147206598734196</v>
+      </c>
+      <c r="X28" s="108">
+        <v>0.14315943224626199</v>
+      </c>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A29" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B29" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="C29" s="81">
+        <v>150</v>
+      </c>
+      <c r="D29" s="81">
+        <v>20</v>
+      </c>
+      <c r="E29" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F29" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G29" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H29" s="54">
+        <v>5.5448295061802497E-4</v>
+      </c>
+      <c r="I29" s="54">
+        <f>60+50.06</f>
+        <v>110.06</v>
+      </c>
+      <c r="J29" s="111">
+        <f t="shared" si="2"/>
+        <v>1.8343333333333334</v>
+      </c>
+      <c r="K29" s="112">
+        <v>0.18277191334128001</v>
+      </c>
+      <c r="L29" s="112">
+        <v>0.93507902987293001</v>
+      </c>
+      <c r="M29" s="113">
+        <v>5.9846530300535496</v>
+      </c>
+      <c r="N29" s="115">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O29" s="115">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P29" s="115">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q29" s="115">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R29" s="115">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S29" s="115">
+        <v>1E-4</v>
+      </c>
+      <c r="T29" s="113">
+        <v>1.63578039188719</v>
+      </c>
+      <c r="U29" s="113">
+        <v>4.4317996594909204</v>
+      </c>
+      <c r="V29" s="115">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W29" s="122">
+        <v>0.169428071211535</v>
+      </c>
+      <c r="X29" s="123">
+        <v>0.79097187118017498</v>
+      </c>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A30" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30" s="81" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" s="81">
+        <v>200</v>
+      </c>
+      <c r="D30" s="81">
+        <v>20</v>
+      </c>
+      <c r="E30" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F30" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G30" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H30" s="2">
+        <v>5.3513470918326999E-4</v>
+      </c>
+      <c r="I30" s="2">
+        <f>2*60+28.82</f>
+        <v>148.82</v>
+      </c>
+      <c r="J30" s="51">
+        <f t="shared" si="2"/>
+        <v>2.4803333333333333</v>
+      </c>
+      <c r="K30" s="59">
+        <v>0.15787142809999999</v>
+      </c>
+      <c r="L30" s="59">
+        <v>4.0399279379999999</v>
+      </c>
+      <c r="M30" s="60">
+        <v>2.1032253427203802</v>
+      </c>
+      <c r="N30" s="84">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O30" s="84">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P30" s="84">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q30" s="84">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R30" s="84">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S30" s="84">
+        <v>1E-4</v>
+      </c>
+      <c r="T30" s="60">
+        <v>1.5308576470192199</v>
+      </c>
+      <c r="U30" s="59">
+        <v>0.1</v>
+      </c>
+      <c r="V30" s="84">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W30" s="61">
+        <v>0.63979153894325302</v>
+      </c>
+      <c r="X30" s="108">
+        <v>0.25571373554670501</v>
+      </c>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A31" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31" s="81" t="s">
+        <v>68</v>
+      </c>
+      <c r="C31" s="81">
+        <v>200</v>
+      </c>
+      <c r="D31" s="81">
+        <v>20</v>
+      </c>
+      <c r="E31" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F31" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G31" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H31" s="2">
+        <v>4.10590634113872E-3</v>
+      </c>
+      <c r="I31" s="2">
+        <f>2*60+58.02</f>
+        <v>178.02</v>
+      </c>
+      <c r="J31" s="51">
+        <f t="shared" si="2"/>
+        <v>2.9670000000000001</v>
+      </c>
+      <c r="K31" s="60">
+        <v>2.6203392075057299</v>
+      </c>
+      <c r="L31" s="60">
+        <v>1.1689507800277501</v>
+      </c>
+      <c r="M31" s="60">
+        <v>2.7976688751157401</v>
+      </c>
+      <c r="N31" s="84">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O31" s="84">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P31" s="84">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q31" s="84">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R31" s="84">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S31" s="84">
+        <v>1E-4</v>
+      </c>
+      <c r="T31" s="60">
+        <v>3.6733722842723902</v>
+      </c>
+      <c r="U31" s="60">
+        <v>1.3915161204550199</v>
+      </c>
+      <c r="V31" s="84">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W31" s="62">
+        <v>1.0069276057424901</v>
+      </c>
+      <c r="X31" s="136">
+        <v>0.30911590470633299</v>
+      </c>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A32" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="C32" s="81">
+        <v>200</v>
+      </c>
+      <c r="D32" s="81">
+        <v>20</v>
+      </c>
+      <c r="E32" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F32" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G32" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H32" s="54">
+        <v>5.3926815435973601E-4</v>
+      </c>
+      <c r="I32" s="54">
+        <f>2*60+31.79</f>
+        <v>151.79</v>
+      </c>
+      <c r="J32" s="111">
+        <f t="shared" si="2"/>
+        <v>2.5298333333333334</v>
+      </c>
+      <c r="K32" s="112">
+        <v>0.200090503125988</v>
+      </c>
+      <c r="L32" s="112">
+        <v>0.93334617005500298</v>
+      </c>
+      <c r="M32" s="113">
+        <v>6.05992631645519</v>
+      </c>
+      <c r="N32" s="115">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O32" s="115">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P32" s="115">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q32" s="115">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R32" s="115">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S32" s="115">
+        <v>1E-4</v>
+      </c>
+      <c r="T32" s="113">
+        <v>1.6315342260914001</v>
+      </c>
+      <c r="U32" s="113">
+        <v>3.8159681302494901</v>
+      </c>
+      <c r="V32" s="115">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W32" s="122">
+        <v>0.174710337054786</v>
+      </c>
+      <c r="X32" s="123">
+        <v>0.77567938513379198</v>
+      </c>
+    </row>
+    <row r="33" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A33" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33" s="81" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="81">
+        <v>500</v>
+      </c>
+      <c r="D33" s="81">
+        <v>20</v>
+      </c>
+      <c r="E33" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F33" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G33" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H33" s="2">
+        <v>5.2679333999513503E-4</v>
+      </c>
+      <c r="I33" s="2">
+        <f>6*60+43.62</f>
+        <v>403.62</v>
+      </c>
+      <c r="J33" s="51">
+        <f t="shared" si="2"/>
+        <v>6.7270000000000003</v>
+      </c>
+      <c r="K33" s="59">
+        <v>0.157463964667933</v>
+      </c>
+      <c r="L33" s="60">
+        <v>4.0531198810914901</v>
+      </c>
+      <c r="M33" s="60">
+        <v>2.0974792918972098</v>
+      </c>
+      <c r="N33" s="84">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O33" s="84">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P33" s="84">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q33" s="84">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R33" s="84">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S33" s="84">
+        <v>1E-4</v>
+      </c>
+      <c r="T33" s="60">
+        <v>1.52141408505271</v>
+      </c>
+      <c r="U33" s="59">
+        <v>0.1</v>
+      </c>
+      <c r="V33" s="84">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W33" s="61">
+        <v>0.64923804018372</v>
+      </c>
+      <c r="X33" s="108">
+        <v>0.24784531385410899</v>
+      </c>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A34" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34" s="81" t="s">
+        <v>68</v>
+      </c>
+      <c r="C34" s="81">
+        <v>500</v>
+      </c>
+      <c r="D34" s="81">
+        <v>20</v>
+      </c>
+      <c r="E34" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F34" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G34" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H34" s="2">
+        <v>4.0861062734903796E-3</v>
+      </c>
+      <c r="I34" s="2">
+        <f>60*7+58.57</f>
+        <v>478.57</v>
+      </c>
+      <c r="J34" s="51">
+        <f t="shared" si="2"/>
+        <v>7.9761666666666668</v>
+      </c>
+      <c r="K34" s="60">
+        <v>2.6203392068401099</v>
+      </c>
+      <c r="L34" s="60">
+        <v>1.1689507251606801</v>
+      </c>
+      <c r="M34" s="60">
+        <v>2.7976691013519499</v>
+      </c>
+      <c r="N34" s="84">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O34" s="84">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P34" s="84">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q34" s="84">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R34" s="84">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S34" s="84">
+        <v>1E-4</v>
+      </c>
+      <c r="T34" s="60">
+        <v>3.67337189781977</v>
+      </c>
+      <c r="U34" s="60">
+        <v>1.3915183032071201</v>
+      </c>
+      <c r="V34" s="84">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W34" s="62">
+        <v>1.0069275680676799</v>
+      </c>
+      <c r="X34" s="136">
+        <v>0.30911590444193399</v>
+      </c>
+    </row>
+    <row r="35" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A35" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B35" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="C35" s="81">
+        <v>500</v>
+      </c>
+      <c r="D35" s="81">
+        <v>20</v>
+      </c>
+      <c r="E35" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="F35" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="G35" s="81">
+        <v>0.7</v>
+      </c>
+      <c r="H35" s="54">
+        <v>5.33593973727646E-4</v>
+      </c>
+      <c r="I35" s="54">
+        <f>6*60+4.39</f>
+        <v>364.39</v>
+      </c>
+      <c r="J35" s="111">
+        <f t="shared" si="2"/>
+        <v>6.0731666666666664</v>
+      </c>
+      <c r="K35" s="112">
+        <v>0.200782865525586</v>
+      </c>
+      <c r="L35" s="112">
+        <v>0.93063361469372696</v>
+      </c>
+      <c r="M35" s="113">
+        <v>6.0938949101244804</v>
+      </c>
+      <c r="N35" s="115">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O35" s="115">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P35" s="115">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q35" s="115">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R35" s="115">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S35" s="115">
+        <v>1E-4</v>
+      </c>
+      <c r="T35" s="113">
+        <v>1.6305970614002501</v>
+      </c>
+      <c r="U35" s="113">
+        <v>3.9338297609874702</v>
+      </c>
+      <c r="V35" s="115">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W35" s="122">
+        <v>0.17573106357227899</v>
+      </c>
+      <c r="X35" s="123">
+        <v>0.76753466547034999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A36" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B36" s="97" t="s">
+        <v>70</v>
+      </c>
+      <c r="C36" s="97">
+        <v>500</v>
+      </c>
+      <c r="D36" s="97">
+        <v>25</v>
+      </c>
+      <c r="E36" s="97">
+        <v>1.5</v>
+      </c>
+      <c r="F36" s="97">
+        <v>1.5</v>
+      </c>
+      <c r="G36" s="97">
+        <v>0.7</v>
+      </c>
+      <c r="H36" s="104">
+        <v>4.9961670047101402E-4</v>
+      </c>
+      <c r="I36" s="104">
+        <f>10*60+4.18</f>
+        <v>604.17999999999995</v>
+      </c>
+      <c r="J36" s="116">
+        <f>I36/60</f>
+        <v>10.069666666666667</v>
+      </c>
+      <c r="K36" s="125">
+        <v>0.123108699728849</v>
+      </c>
+      <c r="L36" s="118">
+        <v>2.2809552057362699</v>
+      </c>
+      <c r="M36" s="118">
+        <v>9.1416504040918696</v>
+      </c>
+      <c r="N36" s="119">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="O36" s="119">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="P36" s="119">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="Q36" s="119">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="R36" s="119">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="S36" s="119">
+        <v>1E-4</v>
+      </c>
+      <c r="T36" s="117">
+        <v>0.91524577772073001</v>
+      </c>
+      <c r="U36" s="118">
+        <v>9.9941869830438801</v>
+      </c>
+      <c r="V36" s="119">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="W36" s="125">
+        <v>0.262348974530624</v>
+      </c>
+      <c r="X36" s="127">
+        <v>0.66041250315907096</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="C1:G1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:J2"/>
-    <mergeCell ref="K1:X1"/>
-  </mergeCells>
+  <autoFilter ref="A2:X36" xr:uid="{3F024A9F-720A-4384-9592-EDD81D7A1CFE}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Avances 30/03: Estimaciones de parámetros de sets de datos individuales para diferentes variedades (CS, SY, ME).
</commit_message>
<xml_diff>
--- a/Optimizacion/Resultados optimizadores.xlsx
+++ b/Optimizacion/Resultados optimizadores.xlsx
@@ -1,25 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://conchaytoro365-my.sharepoint.com/personal/p-maria_folch_conchaytoro_cl/Documents/Escritorio/Archivos/Proyecto_Tintos_CyT_P2/Optimizacion/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p-mfolch\Documents\Proyecto_Tintos_CyT\Optimizacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5334" documentId="11_AD4D2F04E46CFB4ACB3E20395551EF76693EDF1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{263C1EE3-9A70-4B48-987F-B05DF6177C16}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E43BD0-5E90-4E7E-8DBE-0825B8D1F991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
     <sheet name="Pruebas PSO" sheetId="3" r:id="rId3"/>
     <sheet name="Pruebas PSO termination" sheetId="4" r:id="rId4"/>
+    <sheet name="Pruebas variedades" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pruebas PSO'!$A$2:$X$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Pruebas variedades'!$A$1:$AA$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -105,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="126">
   <si>
     <t>Set de datos:</t>
   </si>
@@ -430,6 +432,60 @@
   <si>
     <t>Probé cambiando w=0.9 pero optimiza más lento</t>
   </si>
+  <si>
+    <t>Bien, mejorable</t>
+  </si>
+  <si>
+    <t>Variedad</t>
+  </si>
+  <si>
+    <t>Cabernet Sauvignon</t>
+  </si>
+  <si>
+    <t>Data CS 25 EL BOLDO estanque 55.xlsx</t>
+  </si>
+  <si>
+    <t>Data CS 24 EL BOLDO estanque 30.xlsx</t>
+  </si>
+  <si>
+    <t>Iteración de término</t>
+  </si>
+  <si>
+    <t>Alcanzó el final de las iteraciones</t>
+  </si>
+  <si>
+    <t>Data CS 25 LOU estanque 61.xlsx</t>
+  </si>
+  <si>
+    <t>Syrah</t>
+  </si>
+  <si>
+    <t>Data SY 24 LOU+VAL+FN estanque 36.xlsx</t>
+  </si>
+  <si>
+    <t>Data SY 24 VAL+STARAQ estanque 56.xlsx</t>
+  </si>
+  <si>
+    <t>Data SY 24 LOU estanque 62.xlsx</t>
+  </si>
+  <si>
+    <t>Data SY 25 LOU estanque 30.xlsx</t>
+  </si>
+  <si>
+    <t>Data ME 25 Q. AGUA estanque 85.xlsx</t>
+  </si>
+  <si>
+    <t>Merlot</t>
+  </si>
+  <si>
+    <t>Data ME 24 QAGUA estanque 54.xlsx</t>
+  </si>
+  <si>
+    <t>Data ME 25 AURORA + STA MARTA estanque 57.xlsx</t>
+  </si>
+  <si>
+    <t>Data ME 25 STA MARTA estanque 62.xlsx</t>
+  </si>
 </sst>
 </file>
 
@@ -506,10 +562,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="11">
@@ -970,7 +1028,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="227">
+  <cellXfs count="230">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1288,6 +1346,15 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1300,24 +1367,20 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3854,36 +3917,36 @@
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="B2" s="217" t="s">
+      <c r="B2" s="214" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="220" t="s">
+      <c r="C2" s="215" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="220"/>
-      <c r="E2" s="220"/>
-      <c r="F2" s="220"/>
-      <c r="G2" s="217" t="s">
+      <c r="D2" s="215"/>
+      <c r="E2" s="215"/>
+      <c r="F2" s="215"/>
+      <c r="G2" s="214" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="217" t="s">
+      <c r="H2" s="214" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="217" t="s">
+      <c r="I2" s="214" t="s">
         <v>34</v>
       </c>
-      <c r="N2" s="217" t="s">
+      <c r="N2" s="214" t="s">
         <v>40</v>
       </c>
-      <c r="O2" s="218" t="s">
+      <c r="O2" s="220" t="s">
         <v>1</v>
       </c>
-      <c r="P2" s="214" t="s">
+      <c r="P2" s="217" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="215"/>
-      <c r="R2" s="215"/>
-      <c r="S2" s="216"/>
+      <c r="Q2" s="218"/>
+      <c r="R2" s="218"/>
+      <c r="S2" s="219"/>
       <c r="T2" s="212" t="s">
         <v>9</v>
       </c>
@@ -3895,7 +3958,7 @@
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="B3" s="217"/>
+      <c r="B3" s="214"/>
       <c r="C3" s="50" t="s">
         <v>3</v>
       </c>
@@ -3908,11 +3971,11 @@
       <c r="F3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="217"/>
-      <c r="H3" s="217"/>
-      <c r="I3" s="217"/>
-      <c r="N3" s="217"/>
-      <c r="O3" s="218"/>
+      <c r="G3" s="214"/>
+      <c r="H3" s="214"/>
+      <c r="I3" s="214"/>
+      <c r="N3" s="214"/>
+      <c r="O3" s="220"/>
       <c r="P3" s="50" t="s">
         <v>3</v>
       </c>
@@ -3925,9 +3988,9 @@
       <c r="S3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="T3" s="213"/>
-      <c r="U3" s="213"/>
-      <c r="V3" s="213"/>
+      <c r="T3" s="216"/>
+      <c r="U3" s="216"/>
+      <c r="V3" s="216"/>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
@@ -4349,27 +4412,27 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B21" s="217" t="s">
+      <c r="B21" s="214" t="s">
         <v>1</v>
       </c>
-      <c r="C21" s="220" t="s">
+      <c r="C21" s="215" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="220"/>
-      <c r="E21" s="220"/>
-      <c r="F21" s="220"/>
-      <c r="G21" s="217" t="s">
+      <c r="D21" s="215"/>
+      <c r="E21" s="215"/>
+      <c r="F21" s="215"/>
+      <c r="G21" s="214" t="s">
         <v>9</v>
       </c>
-      <c r="H21" s="217" t="s">
+      <c r="H21" s="214" t="s">
         <v>6</v>
       </c>
-      <c r="I21" s="217" t="s">
+      <c r="I21" s="214" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B22" s="217"/>
+      <c r="B22" s="214"/>
       <c r="C22" s="50" t="s">
         <v>3</v>
       </c>
@@ -4382,9 +4445,9 @@
       <c r="F22" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G22" s="217"/>
-      <c r="H22" s="217"/>
-      <c r="I22" s="217"/>
+      <c r="G22" s="214"/>
+      <c r="H22" s="214"/>
+      <c r="I22" s="214"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B23" s="2" t="s">
@@ -4636,28 +4699,28 @@
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B40" s="217" t="s">
+      <c r="B40" s="214" t="s">
         <v>1</v>
       </c>
-      <c r="C40" s="220" t="s">
+      <c r="C40" s="215" t="s">
         <v>2</v>
       </c>
-      <c r="D40" s="220"/>
-      <c r="E40" s="220"/>
-      <c r="F40" s="220"/>
-      <c r="G40" s="217" t="s">
+      <c r="D40" s="215"/>
+      <c r="E40" s="215"/>
+      <c r="F40" s="215"/>
+      <c r="G40" s="214" t="s">
         <v>9</v>
       </c>
-      <c r="H40" s="217" t="s">
+      <c r="H40" s="214" t="s">
         <v>6</v>
       </c>
-      <c r="I40" s="217" t="s">
+      <c r="I40" s="214" t="s">
         <v>34</v>
       </c>
-      <c r="J40" s="219"/>
+      <c r="J40" s="213"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B41" s="217"/>
+      <c r="B41" s="214"/>
       <c r="C41" s="50" t="s">
         <v>3</v>
       </c>
@@ -4670,10 +4733,10 @@
       <c r="F41" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G41" s="217"/>
-      <c r="H41" s="217"/>
-      <c r="I41" s="217"/>
-      <c r="J41" s="219"/>
+      <c r="G41" s="214"/>
+      <c r="H41" s="214"/>
+      <c r="I41" s="214"/>
+      <c r="J41" s="213"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B42" s="2" t="s">
@@ -4759,6 +4822,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="T2:T3"/>
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
     <mergeCell ref="J40:J41"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="B21:B22"/>
@@ -4775,12 +4844,6 @@
     <mergeCell ref="G40:G41"/>
     <mergeCell ref="H40:H41"/>
     <mergeCell ref="I40:I41"/>
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="T2:T3"/>
-    <mergeCell ref="P2:S2"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10358,7 +10421,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BAAF89D-8B7A-4AB2-AE43-BA5F7D049F38}">
-  <dimension ref="A1:AE18"/>
+  <dimension ref="A1:AE20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40.33203125" bestFit="1" customWidth="1"/>
@@ -10474,7 +10537,7 @@
       <c r="A3" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B3" s="222" t="s">
+      <c r="B3" s="2" t="s">
         <v>70</v>
       </c>
       <c r="C3" s="2">
@@ -10548,7 +10611,7 @@
       <c r="A4" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="222" t="s">
+      <c r="B4" s="2" t="s">
         <v>70</v>
       </c>
       <c r="C4" s="2">
@@ -10622,7 +10685,7 @@
       <c r="A5" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B5" s="222" t="s">
+      <c r="B5" s="2" t="s">
         <v>70</v>
       </c>
       <c r="C5" s="2">
@@ -10696,7 +10759,7 @@
       <c r="A6" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="223" t="s">
+      <c r="B6" s="6" t="s">
         <v>70</v>
       </c>
       <c r="C6" s="6">
@@ -10770,7 +10833,7 @@
       <c r="A7" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="224" t="s">
+      <c r="B7" s="9" t="s">
         <v>70</v>
       </c>
       <c r="C7" s="9">
@@ -10846,7 +10909,7 @@
       <c r="A8" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="B8" s="225" t="s">
+      <c r="B8" s="23" t="s">
         <v>70</v>
       </c>
       <c r="C8" s="23">
@@ -10922,7 +10985,7 @@
       <c r="A9" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B9" s="224" t="s">
+      <c r="B9" s="9" t="s">
         <v>70</v>
       </c>
       <c r="C9" s="9">
@@ -10998,7 +11061,7 @@
       <c r="A10" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="B10" s="223" t="s">
+      <c r="B10" s="6" t="s">
         <v>70</v>
       </c>
       <c r="C10" s="6">
@@ -11075,165 +11138,165 @@
         <v>102</v>
       </c>
     </row>
-    <row r="14" spans="1:31" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="103" t="s">
+    <row r="14" spans="1:31" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="177" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="103" t="s">
+      <c r="B14" s="177" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="63" t="s">
+      <c r="C14" s="178" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="63" t="s">
+      <c r="D14" s="178" t="s">
         <v>46</v>
       </c>
-      <c r="E14" s="63" t="s">
+      <c r="E14" s="178" t="s">
         <v>48</v>
       </c>
-      <c r="F14" s="63" t="s">
+      <c r="F14" s="178" t="s">
         <v>49</v>
       </c>
-      <c r="G14" s="63" t="s">
+      <c r="G14" s="178" t="s">
         <v>50</v>
       </c>
-      <c r="H14" s="103" t="s">
+      <c r="H14" s="177" t="s">
         <v>104</v>
       </c>
-      <c r="I14" s="103" t="s">
+      <c r="I14" s="177" t="s">
         <v>9</v>
       </c>
-      <c r="J14" s="103" t="s">
+      <c r="J14" s="177" t="s">
         <v>6</v>
       </c>
-      <c r="K14" s="103" t="s">
+      <c r="K14" s="177" t="s">
         <v>34</v>
       </c>
-      <c r="L14" s="103" t="s">
+      <c r="L14" s="177" t="s">
         <v>103</v>
       </c>
-      <c r="M14" s="104" t="s">
+      <c r="M14" s="179" t="s">
         <v>52</v>
       </c>
-      <c r="N14" s="104" t="s">
+      <c r="N14" s="179" t="s">
         <v>53</v>
       </c>
-      <c r="O14" s="104" t="s">
+      <c r="O14" s="179" t="s">
         <v>54</v>
       </c>
-      <c r="P14" s="105" t="s">
+      <c r="P14" s="180" t="s">
         <v>55</v>
       </c>
-      <c r="Q14" s="105" t="s">
+      <c r="Q14" s="180" t="s">
         <v>56</v>
       </c>
-      <c r="R14" s="105" t="s">
+      <c r="R14" s="180" t="s">
         <v>57</v>
       </c>
-      <c r="S14" s="105" t="s">
+      <c r="S14" s="180" t="s">
         <v>58</v>
       </c>
-      <c r="T14" s="105" t="s">
+      <c r="T14" s="180" t="s">
         <v>59</v>
       </c>
-      <c r="U14" s="105" t="s">
+      <c r="U14" s="180" t="s">
         <v>60</v>
       </c>
-      <c r="V14" s="104" t="s">
+      <c r="V14" s="179" t="s">
         <v>61</v>
       </c>
-      <c r="W14" s="104" t="s">
+      <c r="W14" s="179" t="s">
         <v>65</v>
       </c>
-      <c r="X14" s="106" t="s">
+      <c r="X14" s="181" t="s">
         <v>62</v>
       </c>
-      <c r="Y14" s="104" t="s">
+      <c r="Y14" s="179" t="s">
         <v>63</v>
       </c>
-      <c r="Z14" s="104" t="s">
+      <c r="Z14" s="179" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B15" s="222" t="s">
+      <c r="B15" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="9">
         <v>1000</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="9">
         <v>25</v>
       </c>
-      <c r="E15" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="F15" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G15" s="2">
+      <c r="E15" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="F15" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="G15" s="9">
         <v>0.7</v>
       </c>
-      <c r="H15" s="226">
+      <c r="H15" s="221">
         <v>0.05</v>
       </c>
-      <c r="I15" s="101">
+      <c r="I15" s="126">
         <v>5.55195432457993E-4</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="9">
         <f>60*2+39.03</f>
         <v>159.03</v>
       </c>
-      <c r="K15" s="51">
+      <c r="K15" s="66">
         <f>J15/60</f>
         <v>2.6505000000000001</v>
       </c>
-      <c r="L15" s="2">
+      <c r="L15" s="9">
         <v>120</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="9">
         <v>0.17148699370661699</v>
       </c>
-      <c r="N15" s="101">
+      <c r="N15" s="126">
         <v>0.93707999896975003</v>
       </c>
-      <c r="O15" s="28">
+      <c r="O15" s="40">
         <v>6.80158187028744</v>
       </c>
-      <c r="P15" s="221">
+      <c r="P15" s="68">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="Q15" s="221">
+      <c r="Q15" s="68">
         <v>8.5518540000000005</v>
       </c>
-      <c r="R15" s="221">
+      <c r="R15" s="68">
         <v>7.1656500000000003</v>
       </c>
-      <c r="S15" s="221">
+      <c r="S15" s="68">
         <v>44.150669999999998</v>
       </c>
-      <c r="T15" s="221">
+      <c r="T15" s="68">
         <v>42.528283999999999</v>
       </c>
-      <c r="U15" s="221">
+      <c r="U15" s="68">
         <v>1E-4</v>
       </c>
-      <c r="V15" s="28">
+      <c r="V15" s="40">
         <v>1.4270934796395001</v>
       </c>
-      <c r="W15" s="28">
+      <c r="W15" s="40">
         <v>9.4254001304004191</v>
       </c>
-      <c r="X15" s="221">
+      <c r="X15" s="68">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Y15" s="2">
+      <c r="Y15" s="9">
         <v>0.14841027220081099</v>
       </c>
-      <c r="Z15" s="2">
+      <c r="Z15" s="11">
         <v>0.83068676382901196</v>
       </c>
       <c r="AA15" t="s">
@@ -11243,85 +11306,85 @@
         <v>107</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A16" s="23" t="s">
+    <row r="16" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="B16" s="222" t="s">
+      <c r="B16" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="6">
         <v>1000</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="6">
         <v>25</v>
       </c>
-      <c r="E16" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="F16" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G16" s="2">
+      <c r="E16" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="F16" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="G16" s="6">
         <v>0.7</v>
       </c>
-      <c r="H16" s="226">
+      <c r="H16" s="222">
         <v>0.01</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="6">
         <v>5.3728371690244599E-4</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="6">
         <f>3*60+57.5</f>
         <v>237.5</v>
       </c>
-      <c r="K16" s="51">
+      <c r="K16" s="172">
         <f>J16/60</f>
         <v>3.9583333333333335</v>
       </c>
-      <c r="L16" s="2">
+      <c r="L16" s="6">
         <v>187</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="6">
         <v>0.17572710819101101</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16" s="6">
         <v>0.92101837173550205</v>
       </c>
-      <c r="O16" s="28">
+      <c r="O16" s="131">
         <v>7.00299601712093</v>
       </c>
-      <c r="P16" s="221">
+      <c r="P16" s="130">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="Q16" s="221">
+      <c r="Q16" s="130">
         <v>8.5518540000000005</v>
       </c>
-      <c r="R16" s="221">
+      <c r="R16" s="130">
         <v>7.1656500000000003</v>
       </c>
-      <c r="S16" s="221">
+      <c r="S16" s="130">
         <v>44.150669999999998</v>
       </c>
-      <c r="T16" s="221">
+      <c r="T16" s="130">
         <v>42.528283999999999</v>
       </c>
-      <c r="U16" s="221">
+      <c r="U16" s="130">
         <v>1E-4</v>
       </c>
-      <c r="V16" s="28">
+      <c r="V16" s="131">
         <v>1.4245541826203501</v>
       </c>
-      <c r="W16" s="28">
+      <c r="W16" s="131">
         <v>8.4950237560708608</v>
       </c>
-      <c r="X16" s="221">
+      <c r="X16" s="130">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Y16" s="2">
+      <c r="Y16" s="6">
         <v>0.151063418330069</v>
       </c>
-      <c r="Z16" s="101">
+      <c r="Z16" s="150">
         <v>0.80636650349953598</v>
       </c>
       <c r="AA16" t="s">
@@ -11329,176 +11392,1477 @@
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B17" s="222" t="s">
+      <c r="B17" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17" s="9">
         <v>1000</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="9">
         <v>25</v>
       </c>
-      <c r="E17" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="F17" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G17" s="2">
+      <c r="E17" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="F17" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="G17" s="9">
         <v>0.7</v>
       </c>
-      <c r="H17" s="226">
+      <c r="H17" s="221">
         <v>0.05</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="9">
         <v>1.2027692073878901E-2</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="9">
         <v>25.73</v>
       </c>
-      <c r="K17" s="51">
+      <c r="K17" s="66">
         <f t="shared" ref="K17:K18" si="0">J17/60</f>
         <v>0.42883333333333334</v>
       </c>
-      <c r="L17" s="2">
+      <c r="L17" s="9">
         <v>54</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="9">
         <v>3.0258688925107802E-2</v>
       </c>
-      <c r="N17" s="28">
+      <c r="N17" s="40">
         <v>2.8780009556191799</v>
       </c>
-      <c r="O17" s="28">
+      <c r="O17" s="40">
         <v>2.3917163972983602</v>
       </c>
-      <c r="P17" s="221">
+      <c r="P17" s="68">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="Q17" s="221">
+      <c r="Q17" s="68">
         <v>8.5518540000000005</v>
       </c>
-      <c r="R17" s="221">
+      <c r="R17" s="68">
         <v>7.1656500000000003</v>
       </c>
-      <c r="S17" s="221">
+      <c r="S17" s="68">
         <v>44.150669999999998</v>
       </c>
-      <c r="T17" s="221">
+      <c r="T17" s="68">
         <v>42.528283999999999</v>
       </c>
-      <c r="U17" s="221">
+      <c r="U17" s="68">
         <v>1E-4</v>
       </c>
-      <c r="V17" s="28">
+      <c r="V17" s="40">
         <v>1.9838817605854999</v>
       </c>
-      <c r="W17" s="28">
+      <c r="W17" s="40">
         <v>8.1319685899103398</v>
       </c>
-      <c r="X17" s="221">
+      <c r="X17" s="68">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Y17" s="2">
+      <c r="Y17" s="9">
         <v>0.44018479275910699</v>
       </c>
-      <c r="Z17" s="101">
+      <c r="Z17" s="183">
         <v>2.0233553465868201</v>
       </c>
       <c r="AA17" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+    <row r="18" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="222" t="s">
+      <c r="B18" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="23">
         <v>1000</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="23">
         <v>25</v>
       </c>
-      <c r="E18" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="F18" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G18" s="2">
+      <c r="E18" s="23">
+        <v>1.5</v>
+      </c>
+      <c r="F18" s="23">
+        <v>1.5</v>
+      </c>
+      <c r="G18" s="23">
         <v>0.7</v>
       </c>
-      <c r="H18" s="226">
+      <c r="H18" s="223">
         <v>0.01</v>
       </c>
-      <c r="I18" s="2">
+      <c r="I18" s="23">
         <v>1.1976391588584099E-2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="23">
         <f>45.17</f>
         <v>45.17</v>
       </c>
-      <c r="K18" s="51">
+      <c r="K18" s="168">
         <f t="shared" si="0"/>
         <v>0.75283333333333335</v>
       </c>
-      <c r="L18" s="2">
+      <c r="L18" s="23">
         <v>97</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="23">
         <v>2.93395878836912E-2</v>
       </c>
-      <c r="N18" s="28">
+      <c r="N18" s="117">
         <v>2.77993378358271</v>
       </c>
-      <c r="O18" s="28">
+      <c r="O18" s="117">
         <v>2.3513550514641102</v>
       </c>
-      <c r="P18" s="221">
+      <c r="P18" s="118">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="Q18" s="221">
+      <c r="Q18" s="118">
         <v>8.5518540000000005</v>
       </c>
-      <c r="R18" s="221">
+      <c r="R18" s="118">
         <v>7.1656500000000003</v>
       </c>
-      <c r="S18" s="221">
+      <c r="S18" s="118">
         <v>44.150669999999998</v>
       </c>
-      <c r="T18" s="221">
+      <c r="T18" s="118">
         <v>42.528283999999999</v>
       </c>
-      <c r="U18" s="221">
+      <c r="U18" s="118">
         <v>1E-4</v>
       </c>
-      <c r="V18" s="28">
+      <c r="V18" s="117">
         <v>2.1385471670560201</v>
       </c>
-      <c r="W18" s="28">
+      <c r="W18" s="117">
         <v>8.4758062049886203</v>
       </c>
-      <c r="X18" s="221">
+      <c r="X18" s="118">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Y18" s="2">
+      <c r="Y18" s="23">
         <v>0.234028577704191</v>
       </c>
-      <c r="Z18" s="101">
+      <c r="Z18" s="159">
         <v>2.0751152127812298</v>
       </c>
       <c r="AA18" t="s">
         <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="9">
+        <v>1000</v>
+      </c>
+      <c r="D19" s="9">
+        <v>25</v>
+      </c>
+      <c r="E19" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="F19" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="G19" s="9">
+        <v>0.7</v>
+      </c>
+      <c r="H19" s="221">
+        <v>0.05</v>
+      </c>
+      <c r="I19" s="9">
+        <v>3.0301450294592802E-3</v>
+      </c>
+      <c r="J19" s="9">
+        <f>60+10.12</f>
+        <v>70.12</v>
+      </c>
+      <c r="K19" s="66">
+        <f>J19/60</f>
+        <v>1.1686666666666667</v>
+      </c>
+      <c r="L19" s="9">
+        <v>98</v>
+      </c>
+      <c r="M19" s="9">
+        <v>4.92734086261623E-2</v>
+      </c>
+      <c r="N19" s="40">
+        <v>2.72874389969224</v>
+      </c>
+      <c r="O19" s="40">
+        <v>1.62701115657096</v>
+      </c>
+      <c r="P19" s="68">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="Q19" s="68">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="R19" s="68">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="S19" s="68">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="T19" s="68">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="U19" s="68">
+        <v>1E-4</v>
+      </c>
+      <c r="V19" s="40">
+        <v>3.7377995511353301</v>
+      </c>
+      <c r="W19" s="40">
+        <v>6.2328719380524999</v>
+      </c>
+      <c r="X19" s="68">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Y19" s="40">
+        <v>0.435712826871338</v>
+      </c>
+      <c r="Z19" s="224">
+        <v>2.1271801326680002</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="6">
+        <v>1000</v>
+      </c>
+      <c r="D20" s="6">
+        <v>25</v>
+      </c>
+      <c r="E20" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="F20" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="G20" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="H20" s="222">
+        <v>0.01</v>
+      </c>
+      <c r="I20" s="132">
+        <v>2.13150469935204E-3</v>
+      </c>
+      <c r="J20" s="6">
+        <f>60*4+6.69</f>
+        <v>246.69</v>
+      </c>
+      <c r="K20" s="172">
+        <f>J20/60</f>
+        <v>4.1115000000000004</v>
+      </c>
+      <c r="L20" s="6">
+        <v>335</v>
+      </c>
+      <c r="M20" s="6">
+        <v>7.12607548997016E-2</v>
+      </c>
+      <c r="N20" s="131">
+        <v>1.40274742445062</v>
+      </c>
+      <c r="O20" s="6">
+        <v>0.65975582595110804</v>
+      </c>
+      <c r="P20" s="130">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="Q20" s="130">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="R20" s="130">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="S20" s="130">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="T20" s="130">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="U20" s="130">
+        <v>1E-4</v>
+      </c>
+      <c r="V20" s="131">
+        <v>9.9998221800693603</v>
+      </c>
+      <c r="W20" s="131">
+        <v>6.70277178666311</v>
+      </c>
+      <c r="X20" s="130">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Y20" s="6">
+        <v>0.42560517238199902</v>
+      </c>
+      <c r="Z20" s="225">
+        <v>2.7412487804322798</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{382E0A3D-09D8-49EB-98BB-1A19629C4812}">
+  <dimension ref="A1:AB22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="43.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="177" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="177" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="226" t="s">
+        <v>109</v>
+      </c>
+      <c r="D1" s="178" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="178" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="178" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" s="178" t="s">
+        <v>49</v>
+      </c>
+      <c r="H1" s="178" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1" s="177" t="s">
+        <v>104</v>
+      </c>
+      <c r="J1" s="177" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="177" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" s="177" t="s">
+        <v>34</v>
+      </c>
+      <c r="M1" s="177" t="s">
+        <v>113</v>
+      </c>
+      <c r="N1" s="179" t="s">
+        <v>52</v>
+      </c>
+      <c r="O1" s="179" t="s">
+        <v>53</v>
+      </c>
+      <c r="P1" s="179" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q1" s="180" t="s">
+        <v>55</v>
+      </c>
+      <c r="R1" s="180" t="s">
+        <v>56</v>
+      </c>
+      <c r="S1" s="180" t="s">
+        <v>57</v>
+      </c>
+      <c r="T1" s="180" t="s">
+        <v>58</v>
+      </c>
+      <c r="U1" s="180" t="s">
+        <v>59</v>
+      </c>
+      <c r="V1" s="180" t="s">
+        <v>60</v>
+      </c>
+      <c r="W1" s="179" t="s">
+        <v>61</v>
+      </c>
+      <c r="X1" s="179" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y1" s="181" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z1" s="179" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA1" s="179" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E2" s="2">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G2" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H2" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I2" s="227">
+        <v>0.01</v>
+      </c>
+      <c r="J2" s="2">
+        <v>9.1703383080884396E-4</v>
+      </c>
+      <c r="K2" s="2">
+        <f>12*60+42.48</f>
+        <v>762.48</v>
+      </c>
+      <c r="L2" s="51">
+        <f>K2/60</f>
+        <v>12.708</v>
+      </c>
+      <c r="M2" s="2">
+        <v>1001</v>
+      </c>
+      <c r="N2" s="2">
+        <v>4.94801127619185E-2</v>
+      </c>
+      <c r="O2" s="28">
+        <v>2.8123834061945798</v>
+      </c>
+      <c r="P2" s="2">
+        <v>0.99007892976186596</v>
+      </c>
+      <c r="Q2" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R2" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S2" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T2" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U2" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V2" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W2" s="28">
+        <v>6.5145360017396499</v>
+      </c>
+      <c r="X2" s="28">
+        <v>4.8258843066456301</v>
+      </c>
+      <c r="Y2" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z2" s="2">
+        <v>0.17887038422377</v>
+      </c>
+      <c r="AA2" s="2">
+        <v>0.96760882811171001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E3" s="2">
+        <v>25</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G3" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H3" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I3" s="227">
+        <v>0.01</v>
+      </c>
+      <c r="J3" s="2">
+        <v>5.3728371690244599E-4</v>
+      </c>
+      <c r="K3" s="2">
+        <f>3*60+57.5</f>
+        <v>237.5</v>
+      </c>
+      <c r="L3" s="51">
+        <f>K3/60</f>
+        <v>3.9583333333333335</v>
+      </c>
+      <c r="M3" s="2">
+        <v>187</v>
+      </c>
+      <c r="N3" s="2">
+        <v>0.17572710819101101</v>
+      </c>
+      <c r="O3" s="2">
+        <v>0.92101837173550205</v>
+      </c>
+      <c r="P3" s="28">
+        <v>7.00299601712093</v>
+      </c>
+      <c r="Q3" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R3" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S3" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T3" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U3" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V3" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W3" s="28">
+        <v>1.4245541826203501</v>
+      </c>
+      <c r="X3" s="28">
+        <v>8.4950237560708608</v>
+      </c>
+      <c r="Y3" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z3" s="2">
+        <v>0.151063418330069</v>
+      </c>
+      <c r="AA3" s="101">
+        <v>0.80636650349953598</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E4" s="2">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G4" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I4" s="227">
+        <v>0.01</v>
+      </c>
+      <c r="J4" s="2">
+        <v>2.5958116203005401E-3</v>
+      </c>
+      <c r="K4" s="2">
+        <f>60+20.57</f>
+        <v>80.569999999999993</v>
+      </c>
+      <c r="L4" s="51">
+        <f>K4/60</f>
+        <v>1.3428333333333333</v>
+      </c>
+      <c r="M4" s="2">
+        <v>160</v>
+      </c>
+      <c r="N4" s="2">
+        <v>7.1635567882672502E-2</v>
+      </c>
+      <c r="O4" s="2">
+        <v>0.336854386443387</v>
+      </c>
+      <c r="P4" s="28">
+        <v>9.9287094723392109</v>
+      </c>
+      <c r="Q4" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R4" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S4" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T4" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U4" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V4" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W4" s="28">
+        <v>2.53053621555713</v>
+      </c>
+      <c r="X4" s="28">
+        <v>5.1700245636405597</v>
+      </c>
+      <c r="Y4" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z4" s="2">
+        <v>0.10430418240273399</v>
+      </c>
+      <c r="AA4" s="2">
+        <v>0.57638438653270396</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E5" s="2">
+        <v>25</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G5" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I5" s="227">
+        <v>0.01</v>
+      </c>
+      <c r="J5" s="2">
+        <v>1.28824834718083E-3</v>
+      </c>
+      <c r="K5" s="2">
+        <f>60+59.04</f>
+        <v>119.03999999999999</v>
+      </c>
+      <c r="L5" s="51">
+        <f>K5/60</f>
+        <v>1.9839999999999998</v>
+      </c>
+      <c r="M5" s="2">
+        <v>212</v>
+      </c>
+      <c r="N5" s="2">
+        <v>7.2350665902395805E-2</v>
+      </c>
+      <c r="O5" s="2">
+        <v>1.661370709394</v>
+      </c>
+      <c r="P5" s="28">
+        <v>5.27666352393301</v>
+      </c>
+      <c r="Q5" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R5" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S5" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T5" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U5" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V5" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W5" s="28">
+        <v>3.56670862546062</v>
+      </c>
+      <c r="X5" s="28">
+        <v>7.4683228372815602</v>
+      </c>
+      <c r="Y5" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z5" s="2">
+        <v>0.99391512324229703</v>
+      </c>
+      <c r="AA5" s="2">
+        <v>0.25184995954331102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="228" t="s">
+        <v>116</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E6" s="2">
+        <v>25</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G6" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I6" s="227">
+        <v>0.01</v>
+      </c>
+      <c r="J6" s="2">
+        <v>5.45242703721959E-4</v>
+      </c>
+      <c r="K6" s="2">
+        <f>4*60+3.21</f>
+        <v>243.21</v>
+      </c>
+      <c r="L6" s="51">
+        <f>K6/60</f>
+        <v>4.0535000000000005</v>
+      </c>
+      <c r="M6" s="2">
+        <v>308</v>
+      </c>
+      <c r="N6" s="2">
+        <v>9.2688582178426501E-2</v>
+      </c>
+      <c r="O6" s="2">
+        <v>0.82698514617913099</v>
+      </c>
+      <c r="P6" s="28">
+        <v>3.3130029661054099</v>
+      </c>
+      <c r="Q6" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R6" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S6" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T6" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U6" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V6" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W6" s="28">
+        <v>3.1433656080569699</v>
+      </c>
+      <c r="X6" s="28">
+        <v>9.3510696982053094</v>
+      </c>
+      <c r="Y6" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z6" s="2">
+        <v>0.215128011883576</v>
+      </c>
+      <c r="AA6" s="2">
+        <v>0.58559062847041299</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="228" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E7" s="2">
+        <v>25</v>
+      </c>
+      <c r="F7" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G7" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I7" s="227">
+        <v>0.01</v>
+      </c>
+      <c r="J7" s="2">
+        <v>5.1794160110028799E-4</v>
+      </c>
+      <c r="K7" s="2">
+        <f>2*60+31.04</f>
+        <v>151.04</v>
+      </c>
+      <c r="L7" s="51">
+        <f>K7/60</f>
+        <v>2.5173333333333332</v>
+      </c>
+      <c r="M7" s="2">
+        <v>136</v>
+      </c>
+      <c r="N7" s="2">
+        <v>0.184225106052644</v>
+      </c>
+      <c r="O7" s="28">
+        <v>2.9503726109964701</v>
+      </c>
+      <c r="P7" s="28">
+        <v>2.0427886845833201</v>
+      </c>
+      <c r="Q7" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R7" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S7" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T7" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U7" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V7" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W7" s="28">
+        <v>4.4918699630599797</v>
+      </c>
+      <c r="X7" s="28">
+        <v>6.9729048484649603</v>
+      </c>
+      <c r="Y7" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z7" s="2">
+        <v>0.40447641067149598</v>
+      </c>
+      <c r="AA7" s="2">
+        <v>0.37700283178585597</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="228" t="s">
+        <v>116</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E8" s="2">
+        <v>25</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G8" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I8" s="227">
+        <v>0.01</v>
+      </c>
+      <c r="J8" s="2">
+        <v>2.6807562214175599E-3</v>
+      </c>
+      <c r="K8" s="2">
+        <f>14*60+48.75</f>
+        <v>888.75</v>
+      </c>
+      <c r="L8" s="51">
+        <f>K8/60</f>
+        <v>14.8125</v>
+      </c>
+      <c r="M8" s="2">
+        <v>82</v>
+      </c>
+      <c r="N8" s="2">
+        <v>9.2611654619837794E-2</v>
+      </c>
+      <c r="O8" s="28">
+        <v>2.3968675731176798</v>
+      </c>
+      <c r="P8" s="28">
+        <v>1.02819811558411</v>
+      </c>
+      <c r="Q8" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R8" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S8" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T8" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U8" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V8" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W8" s="28">
+        <v>5.9702543904673604</v>
+      </c>
+      <c r="X8" s="28">
+        <v>4.5947725392950103</v>
+      </c>
+      <c r="Y8" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z8" s="101">
+        <v>0.356330797947227</v>
+      </c>
+      <c r="AA8" s="2">
+        <v>0.64854762525253196</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="228" t="s">
+        <v>116</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E9" s="2">
+        <v>25</v>
+      </c>
+      <c r="F9" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G9" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I9" s="227">
+        <v>0.01</v>
+      </c>
+      <c r="J9" s="101">
+        <v>2.0583968975858001E-3</v>
+      </c>
+      <c r="K9" s="2">
+        <f>2*60+32.66</f>
+        <v>152.66</v>
+      </c>
+      <c r="L9" s="51">
+        <f>K9/60</f>
+        <v>2.5443333333333333</v>
+      </c>
+      <c r="M9" s="2">
+        <v>279</v>
+      </c>
+      <c r="N9" s="101">
+        <v>8.8806501677895E-2</v>
+      </c>
+      <c r="O9" s="28">
+        <v>3.3523979079684798</v>
+      </c>
+      <c r="P9" s="28">
+        <v>3.38237645491412</v>
+      </c>
+      <c r="Q9" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R9" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S9" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T9" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U9" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V9" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W9" s="28">
+        <v>4.6632521409408598</v>
+      </c>
+      <c r="X9" s="28">
+        <v>3.37161231449543</v>
+      </c>
+      <c r="Y9" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z9" s="2">
+        <v>0.93668432182181804</v>
+      </c>
+      <c r="AA9" s="2">
+        <v>0.22641692257075399</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="228" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E10" s="2">
+        <v>25</v>
+      </c>
+      <c r="F10" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G10" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I10" s="227">
+        <v>0.01</v>
+      </c>
+      <c r="J10" s="101">
+        <v>1.0803960696777501E-3</v>
+      </c>
+      <c r="K10" s="2">
+        <f>2*60+6.49</f>
+        <v>126.49</v>
+      </c>
+      <c r="L10" s="51">
+        <f>K10/60</f>
+        <v>2.1081666666666665</v>
+      </c>
+      <c r="M10" s="2">
+        <v>305</v>
+      </c>
+      <c r="N10" s="101">
+        <v>2.8278903668067599E-2</v>
+      </c>
+      <c r="O10" s="28">
+        <v>2.38404996610933</v>
+      </c>
+      <c r="P10" s="28">
+        <v>4.4014286023129197</v>
+      </c>
+      <c r="Q10" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R10" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S10" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T10" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U10" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V10" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W10" s="28">
+        <v>1.8014323415062901</v>
+      </c>
+      <c r="X10" s="28">
+        <v>4.5414411133846002</v>
+      </c>
+      <c r="Y10" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z10" s="2">
+        <v>0.51124238628788099</v>
+      </c>
+      <c r="AA10" s="2">
+        <v>0.29495795253380303</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="228" t="s">
+        <v>122</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E11" s="2">
+        <v>25</v>
+      </c>
+      <c r="F11" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G11" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I11" s="227">
+        <v>0.01</v>
+      </c>
+      <c r="J11" s="2">
+        <v>4.3972553486052698E-4</v>
+      </c>
+      <c r="K11" s="2">
+        <f>60+40.41</f>
+        <v>100.41</v>
+      </c>
+      <c r="L11" s="51">
+        <f t="shared" ref="L11:L13" si="0">K11/60</f>
+        <v>1.6735</v>
+      </c>
+      <c r="M11" s="2">
+        <v>128</v>
+      </c>
+      <c r="N11" s="2">
+        <v>9.22037845501157E-2</v>
+      </c>
+      <c r="O11" s="28">
+        <v>2.6433716459905501</v>
+      </c>
+      <c r="P11" s="101">
+        <v>0.66858669961273698</v>
+      </c>
+      <c r="Q11" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R11" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S11" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T11" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U11" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V11" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W11" s="28">
+        <v>4.1989298495253999</v>
+      </c>
+      <c r="X11" s="28">
+        <v>6.0398716017856096</v>
+      </c>
+      <c r="Y11" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z11" s="2">
+        <v>0.51999971548750701</v>
+      </c>
+      <c r="AA11" s="2">
+        <v>0.164395651736431</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="228" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E12" s="2">
+        <v>25</v>
+      </c>
+      <c r="F12" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G12" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I12" s="227">
+        <v>0.01</v>
+      </c>
+      <c r="J12" s="2">
+        <v>1.24854757679294E-3</v>
+      </c>
+      <c r="K12" s="2">
+        <f>60+2.87</f>
+        <v>62.87</v>
+      </c>
+      <c r="L12" s="51">
+        <f t="shared" si="0"/>
+        <v>1.0478333333333334</v>
+      </c>
+      <c r="M12" s="2">
+        <v>131</v>
+      </c>
+      <c r="N12" s="2">
+        <v>2.96311889904202E-2</v>
+      </c>
+      <c r="O12" s="28">
+        <v>1.14071996123754</v>
+      </c>
+      <c r="P12" s="28">
+        <v>9.9999999999877502</v>
+      </c>
+      <c r="Q12" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R12" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S12" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T12" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U12" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V12" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W12" s="2">
+        <v>0.96881493251810902</v>
+      </c>
+      <c r="X12" s="28">
+        <v>8.9496248051770806</v>
+      </c>
+      <c r="Y12" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z12" s="2">
+        <v>0.10000481200891199</v>
+      </c>
+      <c r="AA12" s="2">
+        <v>0.80615988242499903</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="228" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E13" s="2">
+        <v>25</v>
+      </c>
+      <c r="F13" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H13" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I13" s="227">
+        <v>0.01</v>
+      </c>
+      <c r="J13" s="2">
+        <v>3.2809640951366801E-3</v>
+      </c>
+      <c r="K13" s="2">
+        <v>42</v>
+      </c>
+      <c r="L13" s="51">
+        <f t="shared" si="0"/>
+        <v>0.7</v>
+      </c>
+      <c r="M13" s="2">
+        <v>75</v>
+      </c>
+      <c r="N13" s="101">
+        <v>4.0822695083438602E-2</v>
+      </c>
+      <c r="O13" s="28">
+        <v>3.9857931809526601</v>
+      </c>
+      <c r="P13" s="28">
+        <v>5.4224424779974996</v>
+      </c>
+      <c r="Q13" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R13" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S13" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T13" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U13" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V13" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W13" s="2">
+        <v>0.11828668451781101</v>
+      </c>
+      <c r="X13" s="28">
+        <v>6.1500927633445803</v>
+      </c>
+      <c r="Y13" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z13" s="101">
+        <v>0.24508389712613601</v>
+      </c>
+      <c r="AA13" s="2">
+        <v>0.71906850575006298</v>
+      </c>
+    </row>
+    <row r="22" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V22" s="229"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AA1" xr:uid="{382E0A3D-09D8-49EB-98BB-1A19629C4812}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AA5">
+      <sortCondition ref="A1"/>
+    </sortState>
+  </autoFilter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Avances 31/03 AM: más datos de variedades y volúmenes.
</commit_message>
<xml_diff>
--- a/Optimizacion/Resultados optimizadores.xlsx
+++ b/Optimizacion/Resultados optimizadores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p-mfolch\Documents\Proyecto_Tintos_CyT\Optimizacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1831DB2F-DA91-4EA7-82D7-22A097783AA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB1A6BB9-41FA-485D-A31C-B9C24F655343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="141">
   <si>
     <t>Set de datos:</t>
   </si>
@@ -505,13 +505,31 @@
     <t>Desv. Est. ME</t>
   </si>
   <si>
-    <t>MERLOT</t>
-  </si>
-  <si>
-    <t>SYRAH</t>
-  </si>
-  <si>
-    <t>CABERNET SAUVIGNON</t>
+    <t>Set de datos (100.000 L)</t>
+  </si>
+  <si>
+    <t>Set de datos (52.400 L)</t>
+  </si>
+  <si>
+    <t>Data CS 24 BOLDO estanque 159.xlsx</t>
+  </si>
+  <si>
+    <t>Ajuste no muy bueno</t>
+  </si>
+  <si>
+    <t>Data CS 25 EL BOLDO estanque 133.xlsx</t>
+  </si>
+  <si>
+    <t>Data CS 24 RH+BOLDO estanque 140.xlsx</t>
+  </si>
+  <si>
+    <t>Promedio</t>
+  </si>
+  <si>
+    <t>Desv. Est.</t>
+  </si>
+  <si>
+    <t>Data CS 24 CONQ+IVALDES estanque 144.xlsx</t>
   </si>
 </sst>
 </file>
@@ -659,7 +677,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -1050,12 +1068,68 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="235">
+  <cellXfs count="248">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1343,6 +1417,16 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1373,15 +1457,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1394,25 +1469,51 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2116,25 +2217,25 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B2" s="206" t="s">
+      <c r="B2" s="216" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="205" t="s">
+      <c r="C2" s="215" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="205"/>
-      <c r="E2" s="205"/>
-      <c r="F2" s="205"/>
-      <c r="G2" s="208" t="s">
+      <c r="D2" s="215"/>
+      <c r="E2" s="215"/>
+      <c r="F2" s="215"/>
+      <c r="G2" s="218" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="208" t="s">
+      <c r="H2" s="218" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="208" t="s">
+      <c r="I2" s="218" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="203" t="s">
+      <c r="J2" s="213" t="s">
         <v>6</v>
       </c>
       <c r="L2" t="s">
@@ -2142,7 +2243,7 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="207"/>
+      <c r="B3" s="217"/>
       <c r="C3" s="16" t="s">
         <v>3</v>
       </c>
@@ -2155,10 +2256,10 @@
       <c r="F3" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="209"/>
-      <c r="H3" s="209"/>
-      <c r="I3" s="209"/>
-      <c r="J3" s="210"/>
+      <c r="G3" s="219"/>
+      <c r="H3" s="219"/>
+      <c r="I3" s="219"/>
+      <c r="J3" s="220"/>
       <c r="L3" t="s">
         <v>15</v>
       </c>
@@ -3666,30 +3767,30 @@
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B71" s="206" t="s">
+      <c r="B71" s="216" t="s">
         <v>1</v>
       </c>
-      <c r="C71" s="205" t="s">
+      <c r="C71" s="215" t="s">
         <v>2</v>
       </c>
-      <c r="D71" s="205"/>
-      <c r="E71" s="205"/>
-      <c r="F71" s="205"/>
-      <c r="G71" s="208" t="s">
+      <c r="D71" s="215"/>
+      <c r="E71" s="215"/>
+      <c r="F71" s="215"/>
+      <c r="G71" s="218" t="s">
         <v>12</v>
       </c>
-      <c r="H71" s="208" t="s">
+      <c r="H71" s="218" t="s">
         <v>9</v>
       </c>
-      <c r="I71" s="208" t="s">
+      <c r="I71" s="218" t="s">
         <v>10</v>
       </c>
-      <c r="J71" s="203" t="s">
+      <c r="J71" s="213" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="72" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B72" s="211"/>
+      <c r="B72" s="221"/>
       <c r="C72" s="7" t="s">
         <v>3</v>
       </c>
@@ -3702,10 +3803,10 @@
       <c r="F72" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G72" s="212"/>
-      <c r="H72" s="212"/>
-      <c r="I72" s="212"/>
-      <c r="J72" s="204"/>
+      <c r="G72" s="222"/>
+      <c r="H72" s="222"/>
+      <c r="I72" s="222"/>
+      <c r="J72" s="214"/>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B73" s="8" t="s">
@@ -3949,48 +4050,48 @@
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="B2" s="214" t="s">
+      <c r="B2" s="227" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="215" t="s">
+      <c r="C2" s="230" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="215"/>
-      <c r="E2" s="215"/>
-      <c r="F2" s="215"/>
-      <c r="G2" s="214" t="s">
+      <c r="D2" s="230"/>
+      <c r="E2" s="230"/>
+      <c r="F2" s="230"/>
+      <c r="G2" s="227" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="214" t="s">
+      <c r="H2" s="227" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="214" t="s">
+      <c r="I2" s="227" t="s">
         <v>34</v>
       </c>
-      <c r="N2" s="214" t="s">
+      <c r="N2" s="227" t="s">
         <v>40</v>
       </c>
-      <c r="O2" s="220" t="s">
+      <c r="O2" s="228" t="s">
         <v>1</v>
       </c>
-      <c r="P2" s="217" t="s">
+      <c r="P2" s="224" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="218"/>
-      <c r="R2" s="218"/>
-      <c r="S2" s="219"/>
-      <c r="T2" s="212" t="s">
+      <c r="Q2" s="225"/>
+      <c r="R2" s="225"/>
+      <c r="S2" s="226"/>
+      <c r="T2" s="222" t="s">
         <v>9</v>
       </c>
-      <c r="U2" s="212" t="s">
+      <c r="U2" s="222" t="s">
         <v>6</v>
       </c>
-      <c r="V2" s="212" t="s">
+      <c r="V2" s="222" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="B3" s="214"/>
+      <c r="B3" s="227"/>
       <c r="C3" s="50" t="s">
         <v>3</v>
       </c>
@@ -4003,11 +4104,11 @@
       <c r="F3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="214"/>
-      <c r="H3" s="214"/>
-      <c r="I3" s="214"/>
-      <c r="N3" s="214"/>
-      <c r="O3" s="220"/>
+      <c r="G3" s="227"/>
+      <c r="H3" s="227"/>
+      <c r="I3" s="227"/>
+      <c r="N3" s="227"/>
+      <c r="O3" s="228"/>
       <c r="P3" s="50" t="s">
         <v>3</v>
       </c>
@@ -4020,9 +4121,9 @@
       <c r="S3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="T3" s="216"/>
-      <c r="U3" s="216"/>
-      <c r="V3" s="216"/>
+      <c r="T3" s="223"/>
+      <c r="U3" s="223"/>
+      <c r="V3" s="223"/>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
@@ -4444,27 +4545,27 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B21" s="214" t="s">
+      <c r="B21" s="227" t="s">
         <v>1</v>
       </c>
-      <c r="C21" s="215" t="s">
+      <c r="C21" s="230" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="215"/>
-      <c r="E21" s="215"/>
-      <c r="F21" s="215"/>
-      <c r="G21" s="214" t="s">
+      <c r="D21" s="230"/>
+      <c r="E21" s="230"/>
+      <c r="F21" s="230"/>
+      <c r="G21" s="227" t="s">
         <v>9</v>
       </c>
-      <c r="H21" s="214" t="s">
+      <c r="H21" s="227" t="s">
         <v>6</v>
       </c>
-      <c r="I21" s="214" t="s">
+      <c r="I21" s="227" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B22" s="214"/>
+      <c r="B22" s="227"/>
       <c r="C22" s="50" t="s">
         <v>3</v>
       </c>
@@ -4477,9 +4578,9 @@
       <c r="F22" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G22" s="214"/>
-      <c r="H22" s="214"/>
-      <c r="I22" s="214"/>
+      <c r="G22" s="227"/>
+      <c r="H22" s="227"/>
+      <c r="I22" s="227"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B23" s="2" t="s">
@@ -4731,28 +4832,28 @@
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B40" s="214" t="s">
+      <c r="B40" s="227" t="s">
         <v>1</v>
       </c>
-      <c r="C40" s="215" t="s">
+      <c r="C40" s="230" t="s">
         <v>2</v>
       </c>
-      <c r="D40" s="215"/>
-      <c r="E40" s="215"/>
-      <c r="F40" s="215"/>
-      <c r="G40" s="214" t="s">
+      <c r="D40" s="230"/>
+      <c r="E40" s="230"/>
+      <c r="F40" s="230"/>
+      <c r="G40" s="227" t="s">
         <v>9</v>
       </c>
-      <c r="H40" s="214" t="s">
+      <c r="H40" s="227" t="s">
         <v>6</v>
       </c>
-      <c r="I40" s="214" t="s">
+      <c r="I40" s="227" t="s">
         <v>34</v>
       </c>
-      <c r="J40" s="213"/>
+      <c r="J40" s="229"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B41" s="214"/>
+      <c r="B41" s="227"/>
       <c r="C41" s="50" t="s">
         <v>3</v>
       </c>
@@ -4765,10 +4866,10 @@
       <c r="F41" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G41" s="214"/>
-      <c r="H41" s="214"/>
-      <c r="I41" s="214"/>
-      <c r="J41" s="213"/>
+      <c r="G41" s="227"/>
+      <c r="H41" s="227"/>
+      <c r="I41" s="227"/>
+      <c r="J41" s="229"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B42" s="2" t="s">
@@ -4854,12 +4955,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="T2:T3"/>
-    <mergeCell ref="P2:S2"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
     <mergeCell ref="J40:J41"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="B21:B22"/>
@@ -4876,6 +4971,12 @@
     <mergeCell ref="G40:G41"/>
     <mergeCell ref="H40:H41"/>
     <mergeCell ref="I40:I41"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="T2:T3"/>
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11272,7 +11373,7 @@
       <c r="G15" s="9">
         <v>0.7</v>
       </c>
-      <c r="H15" s="221">
+      <c r="H15" s="203">
         <v>0.05</v>
       </c>
       <c r="I15" s="126">
@@ -11360,7 +11461,7 @@
       <c r="G16" s="6">
         <v>0.7</v>
       </c>
-      <c r="H16" s="222">
+      <c r="H16" s="204">
         <v>0.01</v>
       </c>
       <c r="I16" s="6">
@@ -11445,7 +11546,7 @@
       <c r="G17" s="9">
         <v>0.7</v>
       </c>
-      <c r="H17" s="221">
+      <c r="H17" s="203">
         <v>0.05</v>
       </c>
       <c r="I17" s="9">
@@ -11529,7 +11630,7 @@
       <c r="G18" s="23">
         <v>0.7</v>
       </c>
-      <c r="H18" s="223">
+      <c r="H18" s="205">
         <v>0.01</v>
       </c>
       <c r="I18" s="23">
@@ -11614,7 +11715,7 @@
       <c r="G19" s="9">
         <v>0.7</v>
       </c>
-      <c r="H19" s="221">
+      <c r="H19" s="203">
         <v>0.05</v>
       </c>
       <c r="I19" s="9">
@@ -11670,7 +11771,7 @@
       <c r="Y19" s="40">
         <v>0.435712826871338</v>
       </c>
-      <c r="Z19" s="224">
+      <c r="Z19" s="206">
         <v>2.1271801326680002</v>
       </c>
       <c r="AA19" t="s">
@@ -11699,7 +11800,7 @@
       <c r="G20" s="6">
         <v>0.7</v>
       </c>
-      <c r="H20" s="222">
+      <c r="H20" s="204">
         <v>0.01</v>
       </c>
       <c r="I20" s="132">
@@ -11755,7 +11856,7 @@
       <c r="Y20" s="6">
         <v>0.42560517238199902</v>
       </c>
-      <c r="Z20" s="225">
+      <c r="Z20" s="207">
         <v>2.7412487804322798</v>
       </c>
       <c r="AA20" t="s">
@@ -11770,183 +11871,184 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{382E0A3D-09D8-49EB-98BB-1A19629C4812}">
-  <dimension ref="A1:AB26"/>
+  <dimension ref="A1:AB34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="43.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="177" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" s="177" t="s">
+    <row r="1" spans="1:28" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="233" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" s="234" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="226" t="s">
+      <c r="C1" s="235" t="s">
         <v>109</v>
       </c>
-      <c r="D1" s="178" t="s">
+      <c r="D1" s="236" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="178" t="s">
+      <c r="E1" s="236" t="s">
         <v>46</v>
       </c>
-      <c r="F1" s="178" t="s">
+      <c r="F1" s="236" t="s">
         <v>48</v>
       </c>
-      <c r="G1" s="178" t="s">
+      <c r="G1" s="236" t="s">
         <v>49</v>
       </c>
-      <c r="H1" s="178" t="s">
+      <c r="H1" s="236" t="s">
         <v>50</v>
       </c>
-      <c r="I1" s="177" t="s">
+      <c r="I1" s="234" t="s">
         <v>104</v>
       </c>
-      <c r="J1" s="177" t="s">
+      <c r="J1" s="234" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="177" t="s">
+      <c r="K1" s="234" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="177" t="s">
+      <c r="L1" s="234" t="s">
         <v>34</v>
       </c>
-      <c r="M1" s="177" t="s">
+      <c r="M1" s="234" t="s">
         <v>113</v>
       </c>
-      <c r="N1" s="179" t="s">
+      <c r="N1" s="237" t="s">
         <v>52</v>
       </c>
-      <c r="O1" s="179" t="s">
+      <c r="O1" s="237" t="s">
         <v>53</v>
       </c>
-      <c r="P1" s="179" t="s">
+      <c r="P1" s="237" t="s">
         <v>54</v>
       </c>
-      <c r="Q1" s="180" t="s">
+      <c r="Q1" s="238" t="s">
         <v>55</v>
       </c>
-      <c r="R1" s="180" t="s">
+      <c r="R1" s="238" t="s">
         <v>56</v>
       </c>
-      <c r="S1" s="180" t="s">
+      <c r="S1" s="238" t="s">
         <v>57</v>
       </c>
-      <c r="T1" s="180" t="s">
+      <c r="T1" s="238" t="s">
         <v>58</v>
       </c>
-      <c r="U1" s="180" t="s">
+      <c r="U1" s="238" t="s">
         <v>59</v>
       </c>
-      <c r="V1" s="180" t="s">
+      <c r="V1" s="238" t="s">
         <v>60</v>
       </c>
-      <c r="W1" s="179" t="s">
+      <c r="W1" s="237" t="s">
         <v>61</v>
       </c>
-      <c r="X1" s="179" t="s">
+      <c r="X1" s="237" t="s">
         <v>65</v>
       </c>
-      <c r="Y1" s="181" t="s">
+      <c r="Y1" s="239" t="s">
         <v>62</v>
       </c>
-      <c r="Z1" s="179" t="s">
+      <c r="Z1" s="237" t="s">
         <v>63</v>
       </c>
-      <c r="AA1" s="179" t="s">
+      <c r="AA1" s="240" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="9">
         <v>1000</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="9">
         <v>25</v>
       </c>
-      <c r="F2" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G2" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="H2" s="2">
+      <c r="F2" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="G2" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="H2" s="9">
         <v>0.7</v>
       </c>
-      <c r="I2" s="228">
+      <c r="I2" s="231">
         <v>0.01</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="9">
         <v>9.1703383080884396E-4</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="9">
         <f>12*60+42.48</f>
         <v>762.48</v>
       </c>
-      <c r="L2" s="51">
-        <f>K2/60</f>
+      <c r="L2" s="66">
+        <f t="shared" ref="L2:L10" si="0">K2/60</f>
         <v>12.708</v>
       </c>
-      <c r="M2" s="2">
+      <c r="M2" s="9">
         <v>1001</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="9">
         <v>4.94801127619185E-2</v>
       </c>
-      <c r="O2" s="28">
+      <c r="O2" s="40">
         <v>2.8123834061945798</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="9">
         <v>0.99007892976186596</v>
       </c>
-      <c r="Q2" s="64">
+      <c r="Q2" s="68">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="R2" s="64">
+      <c r="R2" s="68">
         <v>8.5518540000000005</v>
       </c>
-      <c r="S2" s="64">
+      <c r="S2" s="68">
         <v>7.1656500000000003</v>
       </c>
-      <c r="T2" s="64">
+      <c r="T2" s="68">
         <v>44.150669999999998</v>
       </c>
-      <c r="U2" s="64">
+      <c r="U2" s="68">
         <v>42.528283999999999</v>
       </c>
-      <c r="V2" s="64">
+      <c r="V2" s="68">
         <v>1E-4</v>
       </c>
-      <c r="W2" s="28">
+      <c r="W2" s="40">
         <v>6.5145360017396499</v>
       </c>
-      <c r="X2" s="28">
+      <c r="X2" s="40">
         <v>4.8258843066456301</v>
       </c>
-      <c r="Y2" s="64">
+      <c r="Y2" s="68">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Z2" s="2">
+      <c r="Z2" s="9">
         <v>0.17887038422377</v>
       </c>
-      <c r="AA2" s="2">
+      <c r="AA2" s="11">
         <v>0.96760882811171001</v>
       </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="12" t="s">
         <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -11970,7 +12072,7 @@
       <c r="H3" s="2">
         <v>0.7</v>
       </c>
-      <c r="I3" s="228">
+      <c r="I3" s="208">
         <v>0.01</v>
       </c>
       <c r="J3" s="2">
@@ -11981,7 +12083,7 @@
         <v>237.5</v>
       </c>
       <c r="L3" s="51">
-        <f>K3/60</f>
+        <f t="shared" si="0"/>
         <v>3.9583333333333335</v>
       </c>
       <c r="M3" s="2">
@@ -12026,12 +12128,12 @@
       <c r="Z3" s="2">
         <v>0.151063418330069</v>
       </c>
-      <c r="AA3" s="101">
+      <c r="AA3" s="146">
         <v>0.80636650349953598</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="12" t="s">
         <v>111</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -12055,7 +12157,7 @@
       <c r="H4" s="2">
         <v>0.7</v>
       </c>
-      <c r="I4" s="228">
+      <c r="I4" s="208">
         <v>0.01</v>
       </c>
       <c r="J4" s="2">
@@ -12066,7 +12168,7 @@
         <v>80.569999999999993</v>
       </c>
       <c r="L4" s="51">
-        <f>K4/60</f>
+        <f t="shared" si="0"/>
         <v>1.3428333333333333</v>
       </c>
       <c r="M4" s="2">
@@ -12111,180 +12213,180 @@
       <c r="Z4" s="2">
         <v>0.10430418240273399</v>
       </c>
-      <c r="AA4" s="2">
+      <c r="AA4" s="13">
         <v>0.57638438653270396</v>
       </c>
       <c r="AB4" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="6">
         <v>1000</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="6">
         <v>25</v>
       </c>
-      <c r="F5" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G5" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="H5" s="2">
+      <c r="F5" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="G5" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="H5" s="6">
         <v>0.7</v>
       </c>
-      <c r="I5" s="228">
+      <c r="I5" s="232">
         <v>0.01</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="6">
         <v>1.28824834718083E-3</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="6">
         <f>60+59.04</f>
         <v>119.03999999999999</v>
       </c>
-      <c r="L5" s="51">
-        <f>K5/60</f>
+      <c r="L5" s="172">
+        <f t="shared" si="0"/>
         <v>1.9839999999999998</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="6">
         <v>212</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="6">
         <v>7.2350665902395805E-2</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="6">
         <v>1.661370709394</v>
       </c>
-      <c r="P5" s="28">
+      <c r="P5" s="131">
         <v>5.27666352393301</v>
       </c>
-      <c r="Q5" s="64">
+      <c r="Q5" s="130">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="R5" s="64">
+      <c r="R5" s="130">
         <v>8.5518540000000005</v>
       </c>
-      <c r="S5" s="64">
+      <c r="S5" s="130">
         <v>7.1656500000000003</v>
       </c>
-      <c r="T5" s="64">
+      <c r="T5" s="130">
         <v>44.150669999999998</v>
       </c>
-      <c r="U5" s="64">
+      <c r="U5" s="130">
         <v>42.528283999999999</v>
       </c>
-      <c r="V5" s="64">
+      <c r="V5" s="130">
         <v>1E-4</v>
       </c>
-      <c r="W5" s="28">
+      <c r="W5" s="131">
         <v>3.56670862546062</v>
       </c>
-      <c r="X5" s="28">
+      <c r="X5" s="131">
         <v>7.4683228372815602</v>
       </c>
-      <c r="Y5" s="64">
+      <c r="Y5" s="130">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Z5" s="2">
+      <c r="Z5" s="6">
         <v>0.99391512324229703</v>
       </c>
-      <c r="AA5" s="2">
+      <c r="AA5" s="27">
         <v>0.25184995954331102</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="229" t="s">
+      <c r="C6" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="9">
         <v>1000</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="9">
         <v>25</v>
       </c>
-      <c r="F6" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G6" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="H6" s="2">
+      <c r="F6" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="G6" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="H6" s="9">
         <v>0.7</v>
       </c>
-      <c r="I6" s="228">
+      <c r="I6" s="231">
         <v>0.01</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="9">
         <v>5.45242703721959E-4</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="9">
         <f>4*60+3.21</f>
         <v>243.21</v>
       </c>
-      <c r="L6" s="51">
-        <f>K6/60</f>
+      <c r="L6" s="66">
+        <f t="shared" si="0"/>
         <v>4.0535000000000005</v>
       </c>
-      <c r="M6" s="2">
+      <c r="M6" s="9">
         <v>308</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="9">
         <v>9.2688582178426501E-2</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="9">
         <v>0.82698514617913099</v>
       </c>
-      <c r="P6" s="28">
+      <c r="P6" s="40">
         <v>3.3130029661054099</v>
       </c>
-      <c r="Q6" s="64">
+      <c r="Q6" s="68">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="R6" s="64">
+      <c r="R6" s="68">
         <v>8.5518540000000005</v>
       </c>
-      <c r="S6" s="64">
+      <c r="S6" s="68">
         <v>7.1656500000000003</v>
       </c>
-      <c r="T6" s="64">
+      <c r="T6" s="68">
         <v>44.150669999999998</v>
       </c>
-      <c r="U6" s="64">
+      <c r="U6" s="68">
         <v>42.528283999999999</v>
       </c>
-      <c r="V6" s="64">
+      <c r="V6" s="68">
         <v>1E-4</v>
       </c>
-      <c r="W6" s="28">
+      <c r="W6" s="40">
         <v>3.1433656080569699</v>
       </c>
-      <c r="X6" s="28">
+      <c r="X6" s="40">
         <v>9.3510696982053094</v>
       </c>
-      <c r="Y6" s="64">
+      <c r="Y6" s="68">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Z6" s="2">
+      <c r="Z6" s="9">
         <v>0.215128011883576</v>
       </c>
-      <c r="AA6" s="2">
+      <c r="AA6" s="11">
         <v>0.58559062847041299</v>
       </c>
       <c r="AB6" t="s">
@@ -12292,13 +12394,13 @@
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="12" t="s">
         <v>118</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C7" s="229" t="s">
+      <c r="C7" s="2" t="s">
         <v>116</v>
       </c>
       <c r="D7" s="2">
@@ -12316,7 +12418,7 @@
       <c r="H7" s="2">
         <v>0.7</v>
       </c>
-      <c r="I7" s="228">
+      <c r="I7" s="208">
         <v>0.01</v>
       </c>
       <c r="J7" s="2">
@@ -12327,7 +12429,7 @@
         <v>151.04</v>
       </c>
       <c r="L7" s="51">
-        <f>K7/60</f>
+        <f t="shared" si="0"/>
         <v>2.5173333333333332</v>
       </c>
       <c r="M7" s="2">
@@ -12372,18 +12474,18 @@
       <c r="Z7" s="2">
         <v>0.40447641067149598</v>
       </c>
-      <c r="AA7" s="2">
+      <c r="AA7" s="13">
         <v>0.37700283178585597</v>
       </c>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="12" t="s">
         <v>119</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C8" s="229" t="s">
+      <c r="C8" s="2" t="s">
         <v>116</v>
       </c>
       <c r="D8" s="2">
@@ -12401,7 +12503,7 @@
       <c r="H8" s="2">
         <v>0.7</v>
       </c>
-      <c r="I8" s="228">
+      <c r="I8" s="208">
         <v>0.01</v>
       </c>
       <c r="J8" s="2">
@@ -12412,7 +12514,7 @@
         <v>888.75</v>
       </c>
       <c r="L8" s="51">
-        <f>K8/60</f>
+        <f t="shared" si="0"/>
         <v>14.8125</v>
       </c>
       <c r="M8" s="2">
@@ -12457,188 +12559,188 @@
       <c r="Z8" s="101">
         <v>0.356330797947227</v>
       </c>
-      <c r="AA8" s="2">
+      <c r="AA8" s="13">
         <v>0.64854762525253196</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="C9" s="229" t="s">
+      <c r="C9" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="23">
         <v>1000</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="23">
         <v>25</v>
       </c>
-      <c r="F9" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G9" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="H9" s="2">
+      <c r="F9" s="23">
+        <v>1.5</v>
+      </c>
+      <c r="G9" s="23">
+        <v>1.5</v>
+      </c>
+      <c r="H9" s="23">
         <v>0.7</v>
       </c>
-      <c r="I9" s="228">
+      <c r="I9" s="241">
         <v>0.01</v>
       </c>
-      <c r="J9" s="101">
+      <c r="J9" s="242">
         <v>2.0583968975858001E-3</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="23">
         <f>2*60+32.66</f>
         <v>152.66</v>
       </c>
-      <c r="L9" s="51">
-        <f>K9/60</f>
+      <c r="L9" s="168">
+        <f t="shared" si="0"/>
         <v>2.5443333333333333</v>
       </c>
-      <c r="M9" s="2">
+      <c r="M9" s="23">
         <v>279</v>
       </c>
-      <c r="N9" s="101">
+      <c r="N9" s="242">
         <v>8.8806501677895E-2</v>
       </c>
-      <c r="O9" s="28">
+      <c r="O9" s="117">
         <v>3.3523979079684798</v>
       </c>
-      <c r="P9" s="28">
+      <c r="P9" s="117">
         <v>3.38237645491412</v>
       </c>
-      <c r="Q9" s="64">
+      <c r="Q9" s="118">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="R9" s="64">
+      <c r="R9" s="118">
         <v>8.5518540000000005</v>
       </c>
-      <c r="S9" s="64">
+      <c r="S9" s="118">
         <v>7.1656500000000003</v>
       </c>
-      <c r="T9" s="64">
+      <c r="T9" s="118">
         <v>44.150669999999998</v>
       </c>
-      <c r="U9" s="64">
+      <c r="U9" s="118">
         <v>42.528283999999999</v>
       </c>
-      <c r="V9" s="64">
+      <c r="V9" s="118">
         <v>1E-4</v>
       </c>
-      <c r="W9" s="28">
+      <c r="W9" s="117">
         <v>4.6632521409408598</v>
       </c>
-      <c r="X9" s="28">
+      <c r="X9" s="117">
         <v>3.37161231449543</v>
       </c>
-      <c r="Y9" s="64">
+      <c r="Y9" s="118">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Z9" s="2">
+      <c r="Z9" s="23">
         <v>0.93668432182181804</v>
       </c>
-      <c r="AA9" s="2">
+      <c r="AA9" s="24">
         <v>0.22641692257075399</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="229" t="s">
+      <c r="C10" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="9">
         <v>1000</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="9">
         <v>25</v>
       </c>
-      <c r="F10" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G10" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="H10" s="2">
+      <c r="F10" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="G10" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="H10" s="9">
         <v>0.7</v>
       </c>
-      <c r="I10" s="228">
+      <c r="I10" s="231">
         <v>0.01</v>
       </c>
-      <c r="J10" s="101">
+      <c r="J10" s="126">
         <v>1.0803960696777501E-3</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="9">
         <f>2*60+6.49</f>
         <v>126.49</v>
       </c>
-      <c r="L10" s="51">
-        <f>K10/60</f>
+      <c r="L10" s="66">
+        <f t="shared" si="0"/>
         <v>2.1081666666666665</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="9">
         <v>305</v>
       </c>
-      <c r="N10" s="101">
+      <c r="N10" s="126">
         <v>2.8278903668067599E-2</v>
       </c>
-      <c r="O10" s="28">
+      <c r="O10" s="40">
         <v>2.38404996610933</v>
       </c>
-      <c r="P10" s="28">
+      <c r="P10" s="40">
         <v>4.4014286023129197</v>
       </c>
-      <c r="Q10" s="64">
+      <c r="Q10" s="68">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="R10" s="64">
+      <c r="R10" s="68">
         <v>8.5518540000000005</v>
       </c>
-      <c r="S10" s="64">
+      <c r="S10" s="68">
         <v>7.1656500000000003</v>
       </c>
-      <c r="T10" s="64">
+      <c r="T10" s="68">
         <v>44.150669999999998</v>
       </c>
-      <c r="U10" s="64">
+      <c r="U10" s="68">
         <v>42.528283999999999</v>
       </c>
-      <c r="V10" s="64">
+      <c r="V10" s="68">
         <v>1E-4</v>
       </c>
-      <c r="W10" s="28">
+      <c r="W10" s="40">
         <v>1.8014323415062901</v>
       </c>
-      <c r="X10" s="28">
+      <c r="X10" s="40">
         <v>4.5414411133846002</v>
       </c>
-      <c r="Y10" s="64">
+      <c r="Y10" s="68">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Z10" s="2">
+      <c r="Z10" s="9">
         <v>0.51124238628788099</v>
       </c>
-      <c r="AA10" s="2">
+      <c r="AA10" s="11">
         <v>0.29495795253380303</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="12" t="s">
         <v>123</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="229" t="s">
+      <c r="C11" s="2" t="s">
         <v>122</v>
       </c>
       <c r="D11" s="2">
@@ -12656,7 +12758,7 @@
       <c r="H11" s="2">
         <v>0.7</v>
       </c>
-      <c r="I11" s="228">
+      <c r="I11" s="208">
         <v>0.01</v>
       </c>
       <c r="J11" s="2">
@@ -12667,7 +12769,7 @@
         <v>100.41</v>
       </c>
       <c r="L11" s="51">
-        <f t="shared" ref="L11:L13" si="0">K11/60</f>
+        <f t="shared" ref="L11:L13" si="1">K11/60</f>
         <v>1.6735</v>
       </c>
       <c r="M11" s="2">
@@ -12712,18 +12814,18 @@
       <c r="Z11" s="2">
         <v>0.51999971548750701</v>
       </c>
-      <c r="AA11" s="2">
+      <c r="AA11" s="13">
         <v>0.164395651736431</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="12" t="s">
         <v>124</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C12" s="229" t="s">
+      <c r="C12" s="2" t="s">
         <v>122</v>
       </c>
       <c r="D12" s="2">
@@ -12741,7 +12843,7 @@
       <c r="H12" s="2">
         <v>0.7</v>
       </c>
-      <c r="I12" s="228">
+      <c r="I12" s="208">
         <v>0.01</v>
       </c>
       <c r="J12" s="2">
@@ -12752,7 +12854,7 @@
         <v>62.87</v>
       </c>
       <c r="L12" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.0478333333333334</v>
       </c>
       <c r="M12" s="2">
@@ -12764,7 +12866,7 @@
       <c r="O12" s="28">
         <v>1.14071996123754</v>
       </c>
-      <c r="P12" s="28">
+      <c r="P12" s="3">
         <v>9.9999999999877502</v>
       </c>
       <c r="Q12" s="64">
@@ -12797,139 +12899,218 @@
       <c r="Z12" s="2">
         <v>0.10000481200891199</v>
       </c>
-      <c r="AA12" s="2">
+      <c r="AA12" s="13">
         <v>0.80615988242499903</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="229" t="s">
+      <c r="C13" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="6">
         <v>1000</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="6">
         <v>25</v>
       </c>
-      <c r="F13" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G13" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="H13" s="2">
+      <c r="F13" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="G13" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="H13" s="6">
         <v>0.7</v>
       </c>
-      <c r="I13" s="228">
+      <c r="I13" s="232">
         <v>0.01</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="6">
         <v>3.2809640951366801E-3</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="6">
         <v>42</v>
       </c>
-      <c r="L13" s="51">
-        <f t="shared" si="0"/>
+      <c r="L13" s="172">
+        <f t="shared" si="1"/>
         <v>0.7</v>
       </c>
-      <c r="M13" s="2">
+      <c r="M13" s="6">
         <v>75</v>
       </c>
-      <c r="N13" s="101">
+      <c r="N13" s="132">
         <v>4.0822695083438602E-2</v>
       </c>
-      <c r="O13" s="28">
+      <c r="O13" s="131">
         <v>3.9857931809526601</v>
       </c>
-      <c r="P13" s="28">
+      <c r="P13" s="131">
         <v>5.4224424779974996</v>
       </c>
-      <c r="Q13" s="64">
+      <c r="Q13" s="130">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="R13" s="64">
+      <c r="R13" s="130">
         <v>8.5518540000000005</v>
       </c>
-      <c r="S13" s="64">
+      <c r="S13" s="130">
         <v>7.1656500000000003</v>
       </c>
-      <c r="T13" s="64">
+      <c r="T13" s="130">
         <v>44.150669999999998</v>
       </c>
-      <c r="U13" s="64">
+      <c r="U13" s="130">
         <v>42.528283999999999</v>
       </c>
-      <c r="V13" s="64">
+      <c r="V13" s="130">
         <v>1E-4</v>
       </c>
-      <c r="W13" s="2">
+      <c r="W13" s="6">
         <v>0.11828668451781101</v>
       </c>
-      <c r="X13" s="28">
+      <c r="X13" s="131">
         <v>6.1500927633445803</v>
       </c>
-      <c r="Y13" s="64">
+      <c r="Y13" s="130">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Z13" s="101">
+      <c r="Z13" s="132">
         <v>0.24508389712613601</v>
       </c>
-      <c r="AA13" s="2">
+      <c r="AA13" s="27">
         <v>0.71906850575006298</v>
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A14" s="227"/>
+      <c r="A14" s="243"/>
+      <c r="B14" s="243"/>
+      <c r="C14" s="243"/>
+      <c r="D14" s="243"/>
+      <c r="E14" s="243"/>
+      <c r="F14" s="243"/>
+      <c r="G14" s="243"/>
+      <c r="H14" s="243"/>
+      <c r="I14" s="244"/>
+      <c r="J14" s="243"/>
+      <c r="K14" s="243"/>
+      <c r="L14" s="243"/>
+      <c r="M14" s="243"/>
+      <c r="N14" s="243"/>
+      <c r="O14" s="243"/>
+      <c r="P14" s="243"/>
+      <c r="Q14" s="245"/>
+      <c r="R14" s="245"/>
+      <c r="S14" s="245"/>
+      <c r="T14" s="245"/>
+      <c r="U14" s="245"/>
+      <c r="V14" s="245"/>
+      <c r="W14" s="243"/>
+      <c r="X14" s="243"/>
+      <c r="Y14" s="245"/>
+      <c r="Z14" s="243"/>
+      <c r="AA14" s="243"/>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A15" s="243"/>
+      <c r="B15" s="243"/>
+      <c r="C15" s="243"/>
+      <c r="D15" s="243"/>
+      <c r="E15" s="243"/>
+      <c r="F15" s="243"/>
+      <c r="G15" s="243"/>
+      <c r="H15" s="243"/>
+      <c r="I15" s="244"/>
+      <c r="J15" s="243"/>
+      <c r="K15" s="243"/>
+      <c r="L15" s="243"/>
+      <c r="M15" s="243"/>
+      <c r="N15" s="243"/>
+      <c r="O15" s="243"/>
+      <c r="P15" s="243"/>
+      <c r="Q15" s="245"/>
+      <c r="R15" s="245"/>
+      <c r="S15" s="245"/>
+      <c r="T15" s="245"/>
+      <c r="U15" s="245"/>
+      <c r="V15" s="245"/>
+      <c r="W15" s="243"/>
+      <c r="X15" s="243"/>
+      <c r="Y15" s="245"/>
+      <c r="Z15" s="243"/>
+      <c r="AA15" s="243"/>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="M16" s="231" t="s">
+      <c r="A16" s="243"/>
+      <c r="B16" s="243"/>
+      <c r="C16" s="243"/>
+      <c r="D16" s="243"/>
+      <c r="E16" s="243"/>
+      <c r="F16" s="243"/>
+      <c r="G16" s="243"/>
+      <c r="H16" s="243"/>
+      <c r="I16" s="244"/>
+      <c r="J16" s="243"/>
+      <c r="K16" s="243"/>
+      <c r="L16" s="243"/>
+      <c r="M16" s="210" t="s">
         <v>127</v>
       </c>
-      <c r="N16" s="231">
+      <c r="N16" s="210">
         <f>AVERAGE(N2:N5)</f>
         <v>9.2298363684499451E-2</v>
       </c>
-      <c r="O16" s="232">
+      <c r="O16" s="211">
         <f>AVERAGE(O2:O5)</f>
         <v>1.4329067184418673</v>
       </c>
-      <c r="P16" s="231">
+      <c r="P16" s="210">
         <f>AVERAGE(P2:P5)</f>
         <v>5.7996119857887543</v>
       </c>
-      <c r="Q16" s="231"/>
-      <c r="R16" s="231"/>
-      <c r="S16" s="231"/>
-      <c r="T16" s="231"/>
-      <c r="U16" s="231"/>
-      <c r="V16" s="231"/>
-      <c r="W16" s="231">
-        <f t="shared" ref="O16:AA16" si="1">AVERAGE(W2:W5)</f>
+      <c r="Q16" s="210"/>
+      <c r="R16" s="210"/>
+      <c r="S16" s="210"/>
+      <c r="T16" s="210"/>
+      <c r="U16" s="210"/>
+      <c r="V16" s="210"/>
+      <c r="W16" s="210">
+        <f>AVERAGE(W2:W5)</f>
         <v>3.5090837563444373</v>
       </c>
-      <c r="X16" s="231">
-        <f t="shared" si="1"/>
+      <c r="X16" s="210">
+        <f>AVERAGE(X2:X5)</f>
         <v>6.4898138659096531</v>
       </c>
-      <c r="Y16" s="231"/>
-      <c r="Z16" s="231">
-        <f t="shared" si="1"/>
+      <c r="Y16" s="210"/>
+      <c r="Z16" s="210">
+        <f>AVERAGE(Z2:Z5)</f>
         <v>0.35703827704971747</v>
       </c>
-      <c r="AA16" s="231">
-        <f t="shared" si="1"/>
+      <c r="AA16" s="210">
+        <f>AVERAGE(AA2:AA5)</f>
         <v>0.6505524194218153</v>
       </c>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M17" s="234" t="s">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A17" s="243"/>
+      <c r="B17" s="243"/>
+      <c r="C17" s="243"/>
+      <c r="D17" s="243"/>
+      <c r="E17" s="243"/>
+      <c r="F17" s="243"/>
+      <c r="G17" s="243"/>
+      <c r="H17" s="243"/>
+      <c r="I17" s="244"/>
+      <c r="J17" s="243"/>
+      <c r="K17" s="243"/>
+      <c r="L17" s="243"/>
+      <c r="M17" s="52" t="s">
         <v>126</v>
       </c>
       <c r="N17" s="2">
@@ -12941,7 +13122,7 @@
         <v>1.0674755455728331</v>
       </c>
       <c r="P17" s="2">
-        <f t="shared" ref="O17:AA17" si="2">_xlfn.STDEV.S(P2:P5)</f>
+        <f>_xlfn.STDEV.S(P2:P5)</f>
         <v>3.7373191145113278</v>
       </c>
       <c r="Q17" s="2"/>
@@ -12951,65 +13132,65 @@
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
       <c r="W17" s="2">
-        <f t="shared" si="2"/>
+        <f>_xlfn.STDEV.S(W2:W5)</f>
         <v>2.1862359325412095</v>
       </c>
       <c r="X17" s="2">
-        <f t="shared" si="2"/>
+        <f>_xlfn.STDEV.S(X2:X5)</f>
         <v>1.7784686194618968</v>
       </c>
       <c r="Y17" s="2"/>
       <c r="Z17" s="2">
-        <f t="shared" si="2"/>
+        <f>_xlfn.STDEV.S(Z2:Z5)</f>
         <v>0.42569788985141976</v>
       </c>
       <c r="AA17" s="2">
-        <f t="shared" si="2"/>
+        <f>_xlfn.STDEV.S(AA2:AA5)</f>
         <v>0.31051964173200736</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M18" s="231" t="s">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="M18" s="210" t="s">
         <v>128</v>
       </c>
-      <c r="N18" s="231">
+      <c r="N18" s="210">
         <f>AVERAGE(N6:N9)</f>
         <v>0.11458296113220082</v>
       </c>
-      <c r="O18" s="231">
-        <f t="shared" ref="O18:AA18" si="3">AVERAGE(O6:O9)</f>
+      <c r="O18" s="210">
+        <f>AVERAGE(O6:O9)</f>
         <v>2.3816558095654399</v>
       </c>
-      <c r="P18" s="231">
-        <f t="shared" si="3"/>
+      <c r="P18" s="210">
+        <f>AVERAGE(P6:P9)</f>
         <v>2.44159155529674</v>
       </c>
-      <c r="Q18" s="231"/>
-      <c r="R18" s="231"/>
-      <c r="S18" s="231"/>
-      <c r="T18" s="231"/>
-      <c r="U18" s="231"/>
-      <c r="V18" s="231"/>
-      <c r="W18" s="231">
-        <f t="shared" si="3"/>
+      <c r="Q18" s="210"/>
+      <c r="R18" s="210"/>
+      <c r="S18" s="210"/>
+      <c r="T18" s="210"/>
+      <c r="U18" s="210"/>
+      <c r="V18" s="210"/>
+      <c r="W18" s="210">
+        <f>AVERAGE(W6:W9)</f>
         <v>4.5671855256312925</v>
       </c>
-      <c r="X18" s="231">
-        <f t="shared" si="3"/>
+      <c r="X18" s="210">
+        <f>AVERAGE(X6:X9)</f>
         <v>6.072589850115178</v>
       </c>
-      <c r="Y18" s="231"/>
-      <c r="Z18" s="231">
-        <f t="shared" si="3"/>
+      <c r="Y18" s="210"/>
+      <c r="Z18" s="210">
+        <f>AVERAGE(Z6:Z9)</f>
         <v>0.47815488558102925</v>
       </c>
-      <c r="AA18" s="231">
-        <f t="shared" si="3"/>
+      <c r="AA18" s="210">
+        <f>AVERAGE(AA6:AA9)</f>
         <v>0.45938950201988871</v>
       </c>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M19" s="229" t="s">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="M19" s="2" t="s">
         <v>129</v>
       </c>
       <c r="N19" s="2">
@@ -13031,65 +13212,65 @@
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
       <c r="W19" s="2">
-        <f t="shared" ref="O19:AA19" si="4">_xlfn.STDEV.S(W6:W9)</f>
+        <f>_xlfn.STDEV.S(W6:W9)</f>
         <v>1.1562535226175066</v>
       </c>
       <c r="X19" s="2">
-        <f t="shared" si="4"/>
+        <f>_xlfn.STDEV.S(X6:X9)</f>
         <v>2.6481579045737234</v>
       </c>
       <c r="Y19" s="2"/>
       <c r="Z19" s="2">
-        <f t="shared" si="4"/>
+        <f>_xlfn.STDEV.S(Z6:Z9)</f>
         <v>0.3160706704621371</v>
       </c>
       <c r="AA19" s="2">
-        <f t="shared" si="4"/>
+        <f>_xlfn.STDEV.S(AA6:AA9)</f>
         <v>0.19388252982129142</v>
       </c>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M20" s="231" t="s">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="M20" s="210" t="s">
         <v>130</v>
       </c>
-      <c r="N20" s="233">
+      <c r="N20" s="212">
         <f>AVERAGE(N10:N13)</f>
         <v>4.7734143073010528E-2</v>
       </c>
-      <c r="O20" s="233">
-        <f t="shared" ref="O20:AA20" si="5">AVERAGE(O10:O13)</f>
+      <c r="O20" s="212">
+        <f>AVERAGE(O10:O13)</f>
         <v>2.5384836885725202</v>
       </c>
-      <c r="P20" s="233">
+      <c r="P20" s="212">
         <f>AVERAGE(P10:P13)</f>
         <v>5.1231144449777268</v>
       </c>
-      <c r="Q20" s="233"/>
-      <c r="R20" s="233"/>
-      <c r="S20" s="233"/>
-      <c r="T20" s="233"/>
-      <c r="U20" s="233"/>
-      <c r="V20" s="233"/>
-      <c r="W20" s="233">
-        <f t="shared" si="5"/>
+      <c r="Q20" s="212"/>
+      <c r="R20" s="212"/>
+      <c r="S20" s="212"/>
+      <c r="T20" s="212"/>
+      <c r="U20" s="212"/>
+      <c r="V20" s="212"/>
+      <c r="W20" s="212">
+        <f>AVERAGE(W10:W13)</f>
         <v>1.7718659520169024</v>
       </c>
-      <c r="X20" s="233">
-        <f t="shared" si="5"/>
+      <c r="X20" s="212">
+        <f>AVERAGE(X10:X13)</f>
         <v>6.4202575709229679</v>
       </c>
-      <c r="Y20" s="233"/>
-      <c r="Z20" s="233">
-        <f t="shared" si="5"/>
+      <c r="Y20" s="212"/>
+      <c r="Z20" s="212">
+        <f>AVERAGE(Z10:Z13)</f>
         <v>0.34408270272760899</v>
       </c>
-      <c r="AA20" s="233">
-        <f t="shared" si="5"/>
+      <c r="AA20" s="212">
+        <f>AVERAGE(AA10:AA13)</f>
         <v>0.49614549811132402</v>
       </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M21" s="229" t="s">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="M21" s="2" t="s">
         <v>131</v>
       </c>
       <c r="N21" s="2">
@@ -13097,7 +13278,7 @@
         <v>3.0174715758036277E-2</v>
       </c>
       <c r="O21" s="2">
-        <f t="shared" ref="O21:AA21" si="6">_xlfn.STDEV.S(O10:O13)</f>
+        <f>_xlfn.STDEV.S(O10:O13)</f>
         <v>1.1666618279564698</v>
       </c>
       <c r="P21" s="2">
@@ -13111,230 +13292,532 @@
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
       <c r="W21" s="2">
-        <f t="shared" si="6"/>
+        <f>_xlfn.STDEV.S(W10:W13)</f>
         <v>1.7579086692049222</v>
       </c>
       <c r="X21" s="2">
-        <f t="shared" si="6"/>
+        <f>_xlfn.STDEV.S(X10:X13)</f>
         <v>1.838960974355333</v>
       </c>
       <c r="Y21" s="2"/>
       <c r="Z21" s="2">
-        <f t="shared" si="6"/>
+        <f>_xlfn.STDEV.S(Z10:Z13)</f>
         <v>0.20677196411711046</v>
       </c>
       <c r="AA21" s="2">
-        <f t="shared" si="6"/>
+        <f>_xlfn.STDEV.S(AA10:AA13)</f>
         <v>0.31429178315771072</v>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="V22" s="230"/>
-    </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
+    <row r="24" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="25" spans="1:28" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="233" t="s">
+        <v>133</v>
+      </c>
+      <c r="B25" s="234" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="235" t="s">
+        <v>109</v>
+      </c>
+      <c r="D25" s="236" t="s">
+        <v>47</v>
+      </c>
+      <c r="E25" s="236" t="s">
+        <v>46</v>
+      </c>
+      <c r="F25" s="236" t="s">
+        <v>48</v>
+      </c>
+      <c r="G25" s="236" t="s">
+        <v>49</v>
+      </c>
+      <c r="H25" s="236" t="s">
+        <v>50</v>
+      </c>
+      <c r="I25" s="234" t="s">
+        <v>104</v>
+      </c>
+      <c r="J25" s="234" t="s">
+        <v>9</v>
+      </c>
+      <c r="K25" s="234" t="s">
+        <v>6</v>
+      </c>
+      <c r="L25" s="234" t="s">
+        <v>34</v>
+      </c>
+      <c r="M25" s="234" t="s">
+        <v>113</v>
+      </c>
+      <c r="N25" s="237" t="s">
+        <v>52</v>
+      </c>
+      <c r="O25" s="237" t="s">
+        <v>53</v>
+      </c>
+      <c r="P25" s="237" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q25" s="238" t="s">
+        <v>55</v>
+      </c>
+      <c r="R25" s="238" t="s">
+        <v>56</v>
+      </c>
+      <c r="S25" s="238" t="s">
+        <v>57</v>
+      </c>
+      <c r="T25" s="238" t="s">
+        <v>58</v>
+      </c>
+      <c r="U25" s="238" t="s">
+        <v>59</v>
+      </c>
+      <c r="V25" s="238" t="s">
+        <v>60</v>
+      </c>
+      <c r="W25" s="237" t="s">
+        <v>61</v>
+      </c>
+      <c r="X25" s="237" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y25" s="239" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z25" s="237" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA25" s="240" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A26" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B26" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C26" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D26" s="9">
         <v>1000</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E26" s="9">
         <v>25</v>
       </c>
-      <c r="F24" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G24" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="H24" s="2">
+      <c r="F26" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="G26" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="H26" s="9">
         <v>0.7</v>
       </c>
-      <c r="I24" s="228">
+      <c r="I26" s="231">
         <v>0.01</v>
       </c>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="64">
+      <c r="J26" s="9">
+        <v>2.4504995388063698E-3</v>
+      </c>
+      <c r="K26" s="9">
+        <f>6*60+45.13</f>
+        <v>405.13</v>
+      </c>
+      <c r="L26" s="66">
+        <f>K26/60</f>
+        <v>6.7521666666666667</v>
+      </c>
+      <c r="M26" s="9">
+        <v>406</v>
+      </c>
+      <c r="N26" s="9">
+        <v>0.68517564480621196</v>
+      </c>
+      <c r="O26" s="40">
+        <v>5.3129944719811304</v>
+      </c>
+      <c r="P26" s="40">
+        <v>2.7984381878306301</v>
+      </c>
+      <c r="Q26" s="68">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="R24" s="64">
+      <c r="R26" s="68">
         <v>8.5518540000000005</v>
       </c>
-      <c r="S24" s="64">
+      <c r="S26" s="68">
         <v>7.1656500000000003</v>
       </c>
-      <c r="T24" s="64">
+      <c r="T26" s="68">
         <v>44.150669999999998</v>
       </c>
-      <c r="U24" s="64">
+      <c r="U26" s="68">
         <v>42.528283999999999</v>
       </c>
-      <c r="V24" s="64">
+      <c r="V26" s="68">
         <v>1E-4</v>
       </c>
-      <c r="W24" s="2"/>
-      <c r="X24" s="2"/>
-      <c r="Y24" s="64">
+      <c r="W26" s="40">
+        <v>1.17434087379236</v>
+      </c>
+      <c r="X26" s="40">
+        <v>0.100002351778943</v>
+      </c>
+      <c r="Y26" s="68">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Z24" s="2"/>
-      <c r="AA24" s="2"/>
-    </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="B25" s="2" t="s">
+      <c r="Z26" s="9">
+        <v>0.396474674349798</v>
+      </c>
+      <c r="AA26" s="11">
+        <v>0.50836771896878297</v>
+      </c>
+      <c r="AB26" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="27" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A27" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="D25" s="2">
+      <c r="C27" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D27" s="2">
         <v>1000</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E27" s="2">
         <v>25</v>
       </c>
-      <c r="F25" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G25" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="H25" s="2">
+      <c r="F27" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G27" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H27" s="2">
         <v>0.7</v>
       </c>
-      <c r="I25" s="228">
+      <c r="I27" s="208">
         <v>0.01</v>
       </c>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
-      <c r="P25" s="2"/>
-      <c r="Q25" s="64">
+      <c r="J27" s="246">
+        <v>1.05437471085419E-3</v>
+      </c>
+      <c r="K27" s="2">
+        <f>5*60+31.28</f>
+        <v>331.28</v>
+      </c>
+      <c r="L27" s="51">
+        <f>K27/60</f>
+        <v>5.5213333333333328</v>
+      </c>
+      <c r="M27" s="2">
+        <v>491</v>
+      </c>
+      <c r="N27" s="2">
+        <v>6.0474330476258199E-2</v>
+      </c>
+      <c r="O27" s="2">
+        <v>0.80628107870271104</v>
+      </c>
+      <c r="P27" s="28">
+        <v>0.917299244931577</v>
+      </c>
+      <c r="Q27" s="64">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="R25" s="64">
+      <c r="R27" s="64">
         <v>8.5518540000000005</v>
       </c>
-      <c r="S25" s="64">
+      <c r="S27" s="64">
         <v>7.1656500000000003</v>
       </c>
-      <c r="T25" s="64">
+      <c r="T27" s="64">
         <v>44.150669999999998</v>
       </c>
-      <c r="U25" s="64">
+      <c r="U27" s="64">
         <v>42.528283999999999</v>
       </c>
-      <c r="V25" s="64">
+      <c r="V27" s="64">
         <v>1E-4</v>
       </c>
-      <c r="W25" s="2"/>
-      <c r="X25" s="2"/>
-      <c r="Y25" s="64">
+      <c r="W27" s="28">
+        <v>3.91745413934524</v>
+      </c>
+      <c r="X27" s="28">
+        <v>3.4102711653503799</v>
+      </c>
+      <c r="Y27" s="64">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Z25" s="2"/>
-      <c r="AA25" s="2"/>
-    </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="B26" s="2" t="s">
+      <c r="Z27" s="2">
+        <v>0.27767596716205301</v>
+      </c>
+      <c r="AA27" s="146">
+        <v>0.62829096093755399</v>
+      </c>
+    </row>
+    <row r="28" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A28" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="D26" s="2">
+      <c r="C28" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D28" s="2">
         <v>1000</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E28" s="2">
         <v>25</v>
       </c>
-      <c r="F26" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="G26" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="H26" s="2">
+      <c r="F28" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G28" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H28" s="2">
         <v>0.7</v>
       </c>
-      <c r="I26" s="228">
+      <c r="I28" s="208">
         <v>0.01</v>
       </c>
-      <c r="J26" s="2">
-        <v>5.2039279251215001E-2</v>
-      </c>
-      <c r="K26" s="2">
-        <f>10*60+16.29</f>
-        <v>616.29</v>
-      </c>
-      <c r="L26" s="51">
-        <f>K26/60</f>
-        <v>10.2715</v>
-      </c>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2">
-        <v>9.3049520694203094E-2</v>
-      </c>
-      <c r="O26" s="28">
-        <v>2.0666549393433198</v>
-      </c>
-      <c r="P26" s="2">
-        <v>0.97768887548474503</v>
-      </c>
-      <c r="Q26" s="64">
+      <c r="J28" s="246">
+        <v>7.5686483089474103E-4</v>
+      </c>
+      <c r="K28" s="2">
+        <f>5*60+55.08</f>
+        <v>355.08</v>
+      </c>
+      <c r="L28" s="51">
+        <f>K28/60</f>
+        <v>5.9180000000000001</v>
+      </c>
+      <c r="M28" s="2">
+        <v>168</v>
+      </c>
+      <c r="N28" s="2">
+        <v>0.110272721924296</v>
+      </c>
+      <c r="O28" s="28">
+        <v>1.17076295572537</v>
+      </c>
+      <c r="P28" s="28">
+        <v>2.25578090010531</v>
+      </c>
+      <c r="Q28" s="64">
         <v>9.6469999999999993E-3</v>
       </c>
-      <c r="R26" s="64">
+      <c r="R28" s="64">
         <v>8.5518540000000005</v>
       </c>
-      <c r="S26" s="64">
+      <c r="S28" s="64">
         <v>7.1656500000000003</v>
       </c>
-      <c r="T26" s="64">
+      <c r="T28" s="64">
         <v>44.150669999999998</v>
       </c>
-      <c r="U26" s="64">
+      <c r="U28" s="64">
         <v>42.528283999999999</v>
       </c>
-      <c r="V26" s="64">
+      <c r="V28" s="64">
         <v>1E-4</v>
       </c>
-      <c r="W26" s="28">
-        <v>4.2720680669276803</v>
-      </c>
-      <c r="X26" s="28">
-        <v>3.5218612712384498</v>
-      </c>
-      <c r="Y26" s="64">
+      <c r="W28" s="28">
+        <v>5.3631699111812496</v>
+      </c>
+      <c r="X28" s="28">
+        <v>9.2128024788256297</v>
+      </c>
+      <c r="Y28" s="64">
         <v>1.6426339999999999</v>
       </c>
-      <c r="Z26" s="2">
-        <v>0.42123755378781103</v>
-      </c>
-      <c r="AA26" s="2">
-        <v>0.415775288041493</v>
-      </c>
+      <c r="Z28" s="28">
+        <v>1.01837154620533</v>
+      </c>
+      <c r="AA28" s="13">
+        <v>0.15050491430758201</v>
+      </c>
+    </row>
+    <row r="29" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D29" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E29" s="6">
+        <v>25</v>
+      </c>
+      <c r="F29" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="G29" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="H29" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="I29" s="232">
+        <v>0.01</v>
+      </c>
+      <c r="J29" s="247">
+        <v>6.4367444323311796E-4</v>
+      </c>
+      <c r="K29" s="6">
+        <f>15*60+22.24</f>
+        <v>922.24</v>
+      </c>
+      <c r="L29" s="172">
+        <f>K29/60</f>
+        <v>15.370666666666667</v>
+      </c>
+      <c r="M29" s="6">
+        <v>1001</v>
+      </c>
+      <c r="N29" s="6">
+        <v>8.6457123240578596E-2</v>
+      </c>
+      <c r="O29" s="6">
+        <v>0.60511754362607695</v>
+      </c>
+      <c r="P29" s="131">
+        <v>1.4096919303894699</v>
+      </c>
+      <c r="Q29" s="130">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R29" s="130">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S29" s="130">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T29" s="130">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U29" s="130">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V29" s="130">
+        <v>1E-4</v>
+      </c>
+      <c r="W29" s="131">
+        <v>5.54125213678254</v>
+      </c>
+      <c r="X29" s="131">
+        <v>0.49724142545709898</v>
+      </c>
+      <c r="Y29" s="130">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z29" s="6">
+        <v>0.117665351146806</v>
+      </c>
+      <c r="AA29" s="27">
+        <v>0.71892168022052105</v>
+      </c>
+    </row>
+    <row r="31" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="M31" s="210" t="s">
+        <v>138</v>
+      </c>
+      <c r="N31" s="210">
+        <f>AVERAGE(N26:N29)</f>
+        <v>0.2355949551118362</v>
+      </c>
+      <c r="O31" s="210">
+        <f t="shared" ref="O31:AA31" si="2">AVERAGE(O26:O29)</f>
+        <v>1.973789012508822</v>
+      </c>
+      <c r="P31" s="210">
+        <f t="shared" si="2"/>
+        <v>1.8453025658142468</v>
+      </c>
+      <c r="Q31" s="210"/>
+      <c r="R31" s="210"/>
+      <c r="S31" s="210"/>
+      <c r="T31" s="210"/>
+      <c r="U31" s="210"/>
+      <c r="V31" s="210"/>
+      <c r="W31" s="210">
+        <f t="shared" si="2"/>
+        <v>3.9990542652753476</v>
+      </c>
+      <c r="X31" s="210">
+        <f t="shared" si="2"/>
+        <v>3.3050793553530129</v>
+      </c>
+      <c r="Y31" s="210"/>
+      <c r="Z31" s="210">
+        <f t="shared" si="2"/>
+        <v>0.45254688471599674</v>
+      </c>
+      <c r="AA31" s="210">
+        <f t="shared" si="2"/>
+        <v>0.50152131860861004</v>
+      </c>
+    </row>
+    <row r="32" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="M32" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="N32" s="2">
+        <f>_xlfn.STDEV.S(N26:N29)</f>
+        <v>0.30040960079264961</v>
+      </c>
+      <c r="O32" s="2">
+        <f t="shared" ref="O32:AA32" si="3">_xlfn.STDEV.S(O26:O29)</f>
+        <v>2.2384131517421531</v>
+      </c>
+      <c r="P32" s="2">
+        <f t="shared" si="3"/>
+        <v>0.84220084028758913</v>
+      </c>
+      <c r="Q32" s="2"/>
+      <c r="R32" s="2"/>
+      <c r="S32" s="2"/>
+      <c r="T32" s="2"/>
+      <c r="U32" s="2"/>
+      <c r="V32" s="2"/>
+      <c r="W32" s="2">
+        <f t="shared" si="3"/>
+        <v>2.0186505471776366</v>
+      </c>
+      <c r="X32" s="2">
+        <f t="shared" si="3"/>
+        <v>4.2058978534079605</v>
+      </c>
+      <c r="Y32" s="2"/>
+      <c r="Z32" s="2">
+        <f t="shared" si="3"/>
+        <v>0.39413496827723071</v>
+      </c>
+      <c r="AA32" s="2">
+        <f t="shared" si="3"/>
+        <v>0.24939449922529852</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C34" s="209"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AA1" xr:uid="{382E0A3D-09D8-49EB-98BB-1A19629C4812}">

</xml_diff>

<commit_message>
Avances 06/04: agregué carmenere de 100.000 L
</commit_message>
<xml_diff>
--- a/Optimizacion/Resultados optimizadores.xlsx
+++ b/Optimizacion/Resultados optimizadores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p-mfolch\Documents\Proyecto_Tintos_CyT\Optimizacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB1A6BB9-41FA-485D-A31C-B9C24F655343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB7B6917-2268-47DB-B444-E91BC8AB1CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="147">
   <si>
     <t>Set de datos:</t>
   </si>
@@ -530,6 +530,24 @@
   </si>
   <si>
     <t>Data CS 24 CONQ+IVALDES estanque 144.xlsx</t>
+  </si>
+  <si>
+    <t>Set de datos (29.000 L)</t>
+  </si>
+  <si>
+    <t>Data CS 24 ARE estanque 210.xlsx</t>
+  </si>
+  <si>
+    <t>Ajuste bueno</t>
+  </si>
+  <si>
+    <t>Data CS 25 P. VALDES estanque 219.xlsx</t>
+  </si>
+  <si>
+    <t>AMBOS</t>
+  </si>
+  <si>
+    <t>Ajuste decente para ambos, no excelente pero bueno</t>
   </si>
 </sst>
 </file>
@@ -1129,7 +1147,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="248">
+  <cellXfs count="246">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1427,6 +1445,37 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="170" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1457,6 +1506,15 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1469,51 +1527,9 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2217,25 +2233,25 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B2" s="216" t="s">
+      <c r="B2" s="231" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="215" t="s">
+      <c r="C2" s="230" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="215"/>
-      <c r="E2" s="215"/>
-      <c r="F2" s="215"/>
-      <c r="G2" s="218" t="s">
+      <c r="D2" s="230"/>
+      <c r="E2" s="230"/>
+      <c r="F2" s="230"/>
+      <c r="G2" s="233" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="218" t="s">
+      <c r="H2" s="233" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="218" t="s">
+      <c r="I2" s="233" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="213" t="s">
+      <c r="J2" s="228" t="s">
         <v>6</v>
       </c>
       <c r="L2" t="s">
@@ -2243,7 +2259,7 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="217"/>
+      <c r="B3" s="232"/>
       <c r="C3" s="16" t="s">
         <v>3</v>
       </c>
@@ -2256,10 +2272,10 @@
       <c r="F3" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="219"/>
-      <c r="H3" s="219"/>
-      <c r="I3" s="219"/>
-      <c r="J3" s="220"/>
+      <c r="G3" s="234"/>
+      <c r="H3" s="234"/>
+      <c r="I3" s="234"/>
+      <c r="J3" s="235"/>
       <c r="L3" t="s">
         <v>15</v>
       </c>
@@ -3767,30 +3783,30 @@
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B71" s="216" t="s">
+      <c r="B71" s="231" t="s">
         <v>1</v>
       </c>
-      <c r="C71" s="215" t="s">
+      <c r="C71" s="230" t="s">
         <v>2</v>
       </c>
-      <c r="D71" s="215"/>
-      <c r="E71" s="215"/>
-      <c r="F71" s="215"/>
-      <c r="G71" s="218" t="s">
+      <c r="D71" s="230"/>
+      <c r="E71" s="230"/>
+      <c r="F71" s="230"/>
+      <c r="G71" s="233" t="s">
         <v>12</v>
       </c>
-      <c r="H71" s="218" t="s">
+      <c r="H71" s="233" t="s">
         <v>9</v>
       </c>
-      <c r="I71" s="218" t="s">
+      <c r="I71" s="233" t="s">
         <v>10</v>
       </c>
-      <c r="J71" s="213" t="s">
+      <c r="J71" s="228" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="72" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B72" s="221"/>
+      <c r="B72" s="236"/>
       <c r="C72" s="7" t="s">
         <v>3</v>
       </c>
@@ -3803,10 +3819,10 @@
       <c r="F72" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G72" s="222"/>
-      <c r="H72" s="222"/>
-      <c r="I72" s="222"/>
-      <c r="J72" s="214"/>
+      <c r="G72" s="237"/>
+      <c r="H72" s="237"/>
+      <c r="I72" s="237"/>
+      <c r="J72" s="229"/>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B73" s="8" t="s">
@@ -4050,48 +4066,48 @@
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="B2" s="227" t="s">
+      <c r="B2" s="239" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="230" t="s">
+      <c r="C2" s="240" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="230"/>
-      <c r="E2" s="230"/>
-      <c r="F2" s="230"/>
-      <c r="G2" s="227" t="s">
+      <c r="D2" s="240"/>
+      <c r="E2" s="240"/>
+      <c r="F2" s="240"/>
+      <c r="G2" s="239" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="227" t="s">
+      <c r="H2" s="239" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="227" t="s">
+      <c r="I2" s="239" t="s">
         <v>34</v>
       </c>
-      <c r="N2" s="227" t="s">
+      <c r="N2" s="239" t="s">
         <v>40</v>
       </c>
-      <c r="O2" s="228" t="s">
+      <c r="O2" s="245" t="s">
         <v>1</v>
       </c>
-      <c r="P2" s="224" t="s">
+      <c r="P2" s="242" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="225"/>
-      <c r="R2" s="225"/>
-      <c r="S2" s="226"/>
-      <c r="T2" s="222" t="s">
+      <c r="Q2" s="243"/>
+      <c r="R2" s="243"/>
+      <c r="S2" s="244"/>
+      <c r="T2" s="237" t="s">
         <v>9</v>
       </c>
-      <c r="U2" s="222" t="s">
+      <c r="U2" s="237" t="s">
         <v>6</v>
       </c>
-      <c r="V2" s="222" t="s">
+      <c r="V2" s="237" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="B3" s="227"/>
+      <c r="B3" s="239"/>
       <c r="C3" s="50" t="s">
         <v>3</v>
       </c>
@@ -4104,11 +4120,11 @@
       <c r="F3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="227"/>
-      <c r="H3" s="227"/>
-      <c r="I3" s="227"/>
-      <c r="N3" s="227"/>
-      <c r="O3" s="228"/>
+      <c r="G3" s="239"/>
+      <c r="H3" s="239"/>
+      <c r="I3" s="239"/>
+      <c r="N3" s="239"/>
+      <c r="O3" s="245"/>
       <c r="P3" s="50" t="s">
         <v>3</v>
       </c>
@@ -4121,9 +4137,9 @@
       <c r="S3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="T3" s="223"/>
-      <c r="U3" s="223"/>
-      <c r="V3" s="223"/>
+      <c r="T3" s="241"/>
+      <c r="U3" s="241"/>
+      <c r="V3" s="241"/>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
@@ -4545,27 +4561,27 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B21" s="227" t="s">
+      <c r="B21" s="239" t="s">
         <v>1</v>
       </c>
-      <c r="C21" s="230" t="s">
+      <c r="C21" s="240" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="230"/>
-      <c r="E21" s="230"/>
-      <c r="F21" s="230"/>
-      <c r="G21" s="227" t="s">
+      <c r="D21" s="240"/>
+      <c r="E21" s="240"/>
+      <c r="F21" s="240"/>
+      <c r="G21" s="239" t="s">
         <v>9</v>
       </c>
-      <c r="H21" s="227" t="s">
+      <c r="H21" s="239" t="s">
         <v>6</v>
       </c>
-      <c r="I21" s="227" t="s">
+      <c r="I21" s="239" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B22" s="227"/>
+      <c r="B22" s="239"/>
       <c r="C22" s="50" t="s">
         <v>3</v>
       </c>
@@ -4578,9 +4594,9 @@
       <c r="F22" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G22" s="227"/>
-      <c r="H22" s="227"/>
-      <c r="I22" s="227"/>
+      <c r="G22" s="239"/>
+      <c r="H22" s="239"/>
+      <c r="I22" s="239"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B23" s="2" t="s">
@@ -4832,28 +4848,28 @@
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B40" s="227" t="s">
+      <c r="B40" s="239" t="s">
         <v>1</v>
       </c>
-      <c r="C40" s="230" t="s">
+      <c r="C40" s="240" t="s">
         <v>2</v>
       </c>
-      <c r="D40" s="230"/>
-      <c r="E40" s="230"/>
-      <c r="F40" s="230"/>
-      <c r="G40" s="227" t="s">
+      <c r="D40" s="240"/>
+      <c r="E40" s="240"/>
+      <c r="F40" s="240"/>
+      <c r="G40" s="239" t="s">
         <v>9</v>
       </c>
-      <c r="H40" s="227" t="s">
+      <c r="H40" s="239" t="s">
         <v>6</v>
       </c>
-      <c r="I40" s="227" t="s">
+      <c r="I40" s="239" t="s">
         <v>34</v>
       </c>
-      <c r="J40" s="229"/>
+      <c r="J40" s="238"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B41" s="227"/>
+      <c r="B41" s="239"/>
       <c r="C41" s="50" t="s">
         <v>3</v>
       </c>
@@ -4866,10 +4882,10 @@
       <c r="F41" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G41" s="227"/>
-      <c r="H41" s="227"/>
-      <c r="I41" s="227"/>
-      <c r="J41" s="229"/>
+      <c r="G41" s="239"/>
+      <c r="H41" s="239"/>
+      <c r="I41" s="239"/>
+      <c r="J41" s="238"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B42" s="2" t="s">
@@ -4955,6 +4971,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="T2:T3"/>
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
     <mergeCell ref="J40:J41"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="B21:B22"/>
@@ -4971,12 +4993,6 @@
     <mergeCell ref="G40:G41"/>
     <mergeCell ref="H40:H41"/>
     <mergeCell ref="I40:I41"/>
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="T2:T3"/>
-    <mergeCell ref="P2:S2"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11871,7 +11887,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{382E0A3D-09D8-49EB-98BB-1A19629C4812}">
-  <dimension ref="A1:AB34"/>
+  <dimension ref="A1:AB40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="43.88671875" bestFit="1" customWidth="1"/>
@@ -11880,85 +11896,85 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="233" t="s">
+      <c r="A1" s="215" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="234" t="s">
+      <c r="B1" s="216" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="235" t="s">
+      <c r="C1" s="217" t="s">
         <v>109</v>
       </c>
-      <c r="D1" s="236" t="s">
+      <c r="D1" s="218" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="236" t="s">
+      <c r="E1" s="218" t="s">
         <v>46</v>
       </c>
-      <c r="F1" s="236" t="s">
+      <c r="F1" s="218" t="s">
         <v>48</v>
       </c>
-      <c r="G1" s="236" t="s">
+      <c r="G1" s="218" t="s">
         <v>49</v>
       </c>
-      <c r="H1" s="236" t="s">
+      <c r="H1" s="218" t="s">
         <v>50</v>
       </c>
-      <c r="I1" s="234" t="s">
+      <c r="I1" s="216" t="s">
         <v>104</v>
       </c>
-      <c r="J1" s="234" t="s">
+      <c r="J1" s="216" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="234" t="s">
+      <c r="K1" s="216" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="234" t="s">
+      <c r="L1" s="216" t="s">
         <v>34</v>
       </c>
-      <c r="M1" s="234" t="s">
+      <c r="M1" s="216" t="s">
         <v>113</v>
       </c>
-      <c r="N1" s="237" t="s">
+      <c r="N1" s="219" t="s">
         <v>52</v>
       </c>
-      <c r="O1" s="237" t="s">
+      <c r="O1" s="219" t="s">
         <v>53</v>
       </c>
-      <c r="P1" s="237" t="s">
+      <c r="P1" s="219" t="s">
         <v>54</v>
       </c>
-      <c r="Q1" s="238" t="s">
+      <c r="Q1" s="220" t="s">
         <v>55</v>
       </c>
-      <c r="R1" s="238" t="s">
+      <c r="R1" s="220" t="s">
         <v>56</v>
       </c>
-      <c r="S1" s="238" t="s">
+      <c r="S1" s="220" t="s">
         <v>57</v>
       </c>
-      <c r="T1" s="238" t="s">
+      <c r="T1" s="220" t="s">
         <v>58</v>
       </c>
-      <c r="U1" s="238" t="s">
+      <c r="U1" s="220" t="s">
         <v>59</v>
       </c>
-      <c r="V1" s="238" t="s">
+      <c r="V1" s="220" t="s">
         <v>60</v>
       </c>
-      <c r="W1" s="237" t="s">
+      <c r="W1" s="219" t="s">
         <v>61</v>
       </c>
-      <c r="X1" s="237" t="s">
+      <c r="X1" s="219" t="s">
         <v>65</v>
       </c>
-      <c r="Y1" s="239" t="s">
+      <c r="Y1" s="221" t="s">
         <v>62</v>
       </c>
-      <c r="Z1" s="237" t="s">
+      <c r="Z1" s="219" t="s">
         <v>63</v>
       </c>
-      <c r="AA1" s="240" t="s">
+      <c r="AA1" s="222" t="s">
         <v>64</v>
       </c>
     </row>
@@ -11987,7 +12003,7 @@
       <c r="H2" s="9">
         <v>0.7</v>
       </c>
-      <c r="I2" s="231">
+      <c r="I2" s="213">
         <v>0.01</v>
       </c>
       <c r="J2" s="9">
@@ -12245,7 +12261,7 @@
       <c r="H5" s="6">
         <v>0.7</v>
       </c>
-      <c r="I5" s="232">
+      <c r="I5" s="214">
         <v>0.01</v>
       </c>
       <c r="J5" s="6">
@@ -12330,7 +12346,7 @@
       <c r="H6" s="9">
         <v>0.7</v>
       </c>
-      <c r="I6" s="231">
+      <c r="I6" s="213">
         <v>0.01</v>
       </c>
       <c r="J6" s="9">
@@ -12588,10 +12604,10 @@
       <c r="H9" s="23">
         <v>0.7</v>
       </c>
-      <c r="I9" s="241">
+      <c r="I9" s="223">
         <v>0.01</v>
       </c>
-      <c r="J9" s="242">
+      <c r="J9" s="224">
         <v>2.0583968975858001E-3</v>
       </c>
       <c r="K9" s="23">
@@ -12605,7 +12621,7 @@
       <c r="M9" s="23">
         <v>279</v>
       </c>
-      <c r="N9" s="242">
+      <c r="N9" s="224">
         <v>8.8806501677895E-2</v>
       </c>
       <c r="O9" s="117">
@@ -12673,7 +12689,7 @@
       <c r="H10" s="9">
         <v>0.7</v>
       </c>
-      <c r="I10" s="231">
+      <c r="I10" s="213">
         <v>0.01</v>
       </c>
       <c r="J10" s="126">
@@ -12928,7 +12944,7 @@
       <c r="H13" s="6">
         <v>0.7</v>
       </c>
-      <c r="I13" s="232">
+      <c r="I13" s="214">
         <v>0.01</v>
       </c>
       <c r="J13" s="6">
@@ -12988,76 +13004,27 @@
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A14" s="243"/>
-      <c r="B14" s="243"/>
-      <c r="C14" s="243"/>
-      <c r="D14" s="243"/>
-      <c r="E14" s="243"/>
-      <c r="F14" s="243"/>
-      <c r="G14" s="243"/>
-      <c r="H14" s="243"/>
-      <c r="I14" s="244"/>
-      <c r="J14" s="243"/>
-      <c r="K14" s="243"/>
-      <c r="L14" s="243"/>
-      <c r="M14" s="243"/>
-      <c r="N14" s="243"/>
-      <c r="O14" s="243"/>
-      <c r="P14" s="243"/>
-      <c r="Q14" s="245"/>
-      <c r="R14" s="245"/>
-      <c r="S14" s="245"/>
-      <c r="T14" s="245"/>
-      <c r="U14" s="245"/>
-      <c r="V14" s="245"/>
-      <c r="W14" s="243"/>
-      <c r="X14" s="243"/>
-      <c r="Y14" s="245"/>
-      <c r="Z14" s="243"/>
-      <c r="AA14" s="243"/>
+      <c r="I14" s="225"/>
+      <c r="Q14" s="115"/>
+      <c r="R14" s="115"/>
+      <c r="S14" s="115"/>
+      <c r="T14" s="115"/>
+      <c r="U14" s="115"/>
+      <c r="V14" s="115"/>
+      <c r="Y14" s="115"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A15" s="243"/>
-      <c r="B15" s="243"/>
-      <c r="C15" s="243"/>
-      <c r="D15" s="243"/>
-      <c r="E15" s="243"/>
-      <c r="F15" s="243"/>
-      <c r="G15" s="243"/>
-      <c r="H15" s="243"/>
-      <c r="I15" s="244"/>
-      <c r="J15" s="243"/>
-      <c r="K15" s="243"/>
-      <c r="L15" s="243"/>
-      <c r="M15" s="243"/>
-      <c r="N15" s="243"/>
-      <c r="O15" s="243"/>
-      <c r="P15" s="243"/>
-      <c r="Q15" s="245"/>
-      <c r="R15" s="245"/>
-      <c r="S15" s="245"/>
-      <c r="T15" s="245"/>
-      <c r="U15" s="245"/>
-      <c r="V15" s="245"/>
-      <c r="W15" s="243"/>
-      <c r="X15" s="243"/>
-      <c r="Y15" s="245"/>
-      <c r="Z15" s="243"/>
-      <c r="AA15" s="243"/>
+      <c r="I15" s="225"/>
+      <c r="Q15" s="115"/>
+      <c r="R15" s="115"/>
+      <c r="S15" s="115"/>
+      <c r="T15" s="115"/>
+      <c r="U15" s="115"/>
+      <c r="V15" s="115"/>
+      <c r="Y15" s="115"/>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A16" s="243"/>
-      <c r="B16" s="243"/>
-      <c r="C16" s="243"/>
-      <c r="D16" s="243"/>
-      <c r="E16" s="243"/>
-      <c r="F16" s="243"/>
-      <c r="G16" s="243"/>
-      <c r="H16" s="243"/>
-      <c r="I16" s="244"/>
-      <c r="J16" s="243"/>
-      <c r="K16" s="243"/>
-      <c r="L16" s="243"/>
+      <c r="I16" s="225"/>
       <c r="M16" s="210" t="s">
         <v>127</v>
       </c>
@@ -13098,18 +13065,7 @@
       </c>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A17" s="243"/>
-      <c r="B17" s="243"/>
-      <c r="C17" s="243"/>
-      <c r="D17" s="243"/>
-      <c r="E17" s="243"/>
-      <c r="F17" s="243"/>
-      <c r="G17" s="243"/>
-      <c r="H17" s="243"/>
-      <c r="I17" s="244"/>
-      <c r="J17" s="243"/>
-      <c r="K17" s="243"/>
-      <c r="L17" s="243"/>
+      <c r="I17" s="225"/>
       <c r="M17" s="52" t="s">
         <v>126</v>
       </c>
@@ -13311,85 +13267,85 @@
     </row>
     <row r="24" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="25" spans="1:28" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="233" t="s">
+      <c r="A25" s="215" t="s">
         <v>133</v>
       </c>
-      <c r="B25" s="234" t="s">
+      <c r="B25" s="216" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="235" t="s">
+      <c r="C25" s="217" t="s">
         <v>109</v>
       </c>
-      <c r="D25" s="236" t="s">
+      <c r="D25" s="218" t="s">
         <v>47</v>
       </c>
-      <c r="E25" s="236" t="s">
+      <c r="E25" s="218" t="s">
         <v>46</v>
       </c>
-      <c r="F25" s="236" t="s">
+      <c r="F25" s="218" t="s">
         <v>48</v>
       </c>
-      <c r="G25" s="236" t="s">
+      <c r="G25" s="218" t="s">
         <v>49</v>
       </c>
-      <c r="H25" s="236" t="s">
+      <c r="H25" s="218" t="s">
         <v>50</v>
       </c>
-      <c r="I25" s="234" t="s">
+      <c r="I25" s="216" t="s">
         <v>104</v>
       </c>
-      <c r="J25" s="234" t="s">
+      <c r="J25" s="216" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="234" t="s">
+      <c r="K25" s="216" t="s">
         <v>6</v>
       </c>
-      <c r="L25" s="234" t="s">
+      <c r="L25" s="216" t="s">
         <v>34</v>
       </c>
-      <c r="M25" s="234" t="s">
+      <c r="M25" s="216" t="s">
         <v>113</v>
       </c>
-      <c r="N25" s="237" t="s">
+      <c r="N25" s="219" t="s">
         <v>52</v>
       </c>
-      <c r="O25" s="237" t="s">
+      <c r="O25" s="219" t="s">
         <v>53</v>
       </c>
-      <c r="P25" s="237" t="s">
+      <c r="P25" s="219" t="s">
         <v>54</v>
       </c>
-      <c r="Q25" s="238" t="s">
+      <c r="Q25" s="220" t="s">
         <v>55</v>
       </c>
-      <c r="R25" s="238" t="s">
+      <c r="R25" s="220" t="s">
         <v>56</v>
       </c>
-      <c r="S25" s="238" t="s">
+      <c r="S25" s="220" t="s">
         <v>57</v>
       </c>
-      <c r="T25" s="238" t="s">
+      <c r="T25" s="220" t="s">
         <v>58</v>
       </c>
-      <c r="U25" s="238" t="s">
+      <c r="U25" s="220" t="s">
         <v>59</v>
       </c>
-      <c r="V25" s="238" t="s">
+      <c r="V25" s="220" t="s">
         <v>60</v>
       </c>
-      <c r="W25" s="237" t="s">
+      <c r="W25" s="219" t="s">
         <v>61</v>
       </c>
-      <c r="X25" s="237" t="s">
+      <c r="X25" s="219" t="s">
         <v>65</v>
       </c>
-      <c r="Y25" s="239" t="s">
+      <c r="Y25" s="221" t="s">
         <v>62</v>
       </c>
-      <c r="Z25" s="237" t="s">
+      <c r="Z25" s="219" t="s">
         <v>63</v>
       </c>
-      <c r="AA25" s="240" t="s">
+      <c r="AA25" s="222" t="s">
         <v>64</v>
       </c>
     </row>
@@ -13418,7 +13374,7 @@
       <c r="H26" s="9">
         <v>0.7</v>
       </c>
-      <c r="I26" s="231">
+      <c r="I26" s="213">
         <v>0.01</v>
       </c>
       <c r="J26" s="9">
@@ -13509,7 +13465,7 @@
       <c r="I27" s="208">
         <v>0.01</v>
       </c>
-      <c r="J27" s="246">
+      <c r="J27" s="226">
         <v>1.05437471085419E-3</v>
       </c>
       <c r="K27" s="2">
@@ -13594,7 +13550,7 @@
       <c r="I28" s="208">
         <v>0.01</v>
       </c>
-      <c r="J28" s="246">
+      <c r="J28" s="226">
         <v>7.5686483089474103E-4</v>
       </c>
       <c r="K28" s="2">
@@ -13676,10 +13632,10 @@
       <c r="H29" s="6">
         <v>0.7</v>
       </c>
-      <c r="I29" s="232">
+      <c r="I29" s="214">
         <v>0.01</v>
       </c>
-      <c r="J29" s="247">
+      <c r="J29" s="227">
         <v>6.4367444323311796E-4</v>
       </c>
       <c r="K29" s="6">
@@ -13816,8 +13772,359 @@
         <v>0.24939449922529852</v>
       </c>
     </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:28" x14ac:dyDescent="0.3">
       <c r="C34" s="209"/>
+    </row>
+    <row r="35" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="36" spans="1:28" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="215" t="s">
+        <v>141</v>
+      </c>
+      <c r="B36" s="216" t="s">
+        <v>45</v>
+      </c>
+      <c r="C36" s="217" t="s">
+        <v>109</v>
+      </c>
+      <c r="D36" s="218" t="s">
+        <v>47</v>
+      </c>
+      <c r="E36" s="218" t="s">
+        <v>46</v>
+      </c>
+      <c r="F36" s="218" t="s">
+        <v>48</v>
+      </c>
+      <c r="G36" s="218" t="s">
+        <v>49</v>
+      </c>
+      <c r="H36" s="218" t="s">
+        <v>50</v>
+      </c>
+      <c r="I36" s="216" t="s">
+        <v>104</v>
+      </c>
+      <c r="J36" s="216" t="s">
+        <v>9</v>
+      </c>
+      <c r="K36" s="216" t="s">
+        <v>6</v>
+      </c>
+      <c r="L36" s="216" t="s">
+        <v>34</v>
+      </c>
+      <c r="M36" s="216" t="s">
+        <v>113</v>
+      </c>
+      <c r="N36" s="219" t="s">
+        <v>52</v>
+      </c>
+      <c r="O36" s="219" t="s">
+        <v>53</v>
+      </c>
+      <c r="P36" s="219" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q36" s="220" t="s">
+        <v>55</v>
+      </c>
+      <c r="R36" s="220" t="s">
+        <v>56</v>
+      </c>
+      <c r="S36" s="220" t="s">
+        <v>57</v>
+      </c>
+      <c r="T36" s="220" t="s">
+        <v>58</v>
+      </c>
+      <c r="U36" s="220" t="s">
+        <v>59</v>
+      </c>
+      <c r="V36" s="220" t="s">
+        <v>60</v>
+      </c>
+      <c r="W36" s="219" t="s">
+        <v>61</v>
+      </c>
+      <c r="X36" s="219" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y36" s="221" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z36" s="219" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA36" s="222" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="37" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D37" s="9">
+        <v>1000</v>
+      </c>
+      <c r="E37" s="9">
+        <v>25</v>
+      </c>
+      <c r="F37" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="G37" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="H37" s="9">
+        <v>0.7</v>
+      </c>
+      <c r="I37" s="213">
+        <v>0.01</v>
+      </c>
+      <c r="J37" s="9">
+        <v>4.6512217008985301E-4</v>
+      </c>
+      <c r="K37" s="9">
+        <f>2*60+36.05</f>
+        <v>156.05000000000001</v>
+      </c>
+      <c r="L37" s="66">
+        <f>K37/60</f>
+        <v>2.6008333333333336</v>
+      </c>
+      <c r="M37" s="9">
+        <v>182</v>
+      </c>
+      <c r="N37" s="9">
+        <v>0.14882356306359101</v>
+      </c>
+      <c r="O37" s="40">
+        <v>3.6317653028851802</v>
+      </c>
+      <c r="P37" s="40">
+        <v>6.7282743450862199</v>
+      </c>
+      <c r="Q37" s="68">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R37" s="68">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S37" s="68">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T37" s="68">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U37" s="68">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V37" s="68">
+        <v>1E-4</v>
+      </c>
+      <c r="W37" s="40">
+        <v>0.99338431203216104</v>
+      </c>
+      <c r="X37" s="40">
+        <v>8.6284330530030697</v>
+      </c>
+      <c r="Y37" s="68">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z37" s="9">
+        <v>0.183051092616763</v>
+      </c>
+      <c r="AA37" s="11">
+        <v>0.40000253058091401</v>
+      </c>
+      <c r="AB37" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="38" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A38" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D38" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E38" s="2">
+        <v>25</v>
+      </c>
+      <c r="F38" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="G38" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="H38" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I38" s="208">
+        <v>0.01</v>
+      </c>
+      <c r="J38" s="101">
+        <v>1.22603838543025E-3</v>
+      </c>
+      <c r="K38" s="2">
+        <f>1*60+31.78</f>
+        <v>91.78</v>
+      </c>
+      <c r="L38" s="51">
+        <f>K38/60</f>
+        <v>1.5296666666666667</v>
+      </c>
+      <c r="M38" s="2">
+        <v>156</v>
+      </c>
+      <c r="N38" s="101">
+        <v>8.3946395282575498E-2</v>
+      </c>
+      <c r="O38" s="28">
+        <v>1.06816405493272</v>
+      </c>
+      <c r="P38" s="28">
+        <v>4.9298156910074296</v>
+      </c>
+      <c r="Q38" s="64">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R38" s="64">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S38" s="64">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T38" s="64">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U38" s="64">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V38" s="64">
+        <v>1E-4</v>
+      </c>
+      <c r="W38" s="28">
+        <v>1.8164079195785801</v>
+      </c>
+      <c r="X38" s="28">
+        <v>9.7927483750326196</v>
+      </c>
+      <c r="Y38" s="64">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z38" s="2">
+        <v>0.10186605360654</v>
+      </c>
+      <c r="AA38" s="146">
+        <v>1.27253263771213</v>
+      </c>
+      <c r="AB38" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="39" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D39" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E39" s="6">
+        <v>25</v>
+      </c>
+      <c r="F39" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="G39" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="H39" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="I39" s="214">
+        <v>0.01</v>
+      </c>
+      <c r="J39" s="132">
+        <v>1.35902765893188E-2</v>
+      </c>
+      <c r="K39" s="6">
+        <f>1*60+31.91</f>
+        <v>91.91</v>
+      </c>
+      <c r="L39" s="172">
+        <f>K39/60</f>
+        <v>1.5318333333333334</v>
+      </c>
+      <c r="M39" s="6">
+        <v>84</v>
+      </c>
+      <c r="N39" s="6">
+        <v>5.8703388704025403E-2</v>
+      </c>
+      <c r="O39" s="131">
+        <v>2.3331981745618799</v>
+      </c>
+      <c r="P39" s="131">
+        <v>3.7463864736288</v>
+      </c>
+      <c r="Q39" s="130">
+        <v>9.6469999999999993E-3</v>
+      </c>
+      <c r="R39" s="130">
+        <v>8.5518540000000005</v>
+      </c>
+      <c r="S39" s="130">
+        <v>7.1656500000000003</v>
+      </c>
+      <c r="T39" s="130">
+        <v>44.150669999999998</v>
+      </c>
+      <c r="U39" s="130">
+        <v>42.528283999999999</v>
+      </c>
+      <c r="V39" s="130">
+        <v>1E-4</v>
+      </c>
+      <c r="W39" s="131">
+        <v>2.4398515851898499</v>
+      </c>
+      <c r="X39" s="131">
+        <v>6.4923644669931102</v>
+      </c>
+      <c r="Y39" s="130">
+        <v>1.6426339999999999</v>
+      </c>
+      <c r="Z39" s="131">
+        <v>0.10000734498067899</v>
+      </c>
+      <c r="AA39" s="207">
+        <v>1.1808221240099701</v>
+      </c>
+      <c r="AB39" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="40" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="AB40" s="209"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AA1" xr:uid="{382E0A3D-09D8-49EB-98BB-1A19629C4812}">

</xml_diff>

<commit_message>
Actualización post primera prueba de hiperparámetros con w y pop_size
</commit_message>
<xml_diff>
--- a/Optimizacion/Resultados optimizadores.xlsx
+++ b/Optimizacion/Resultados optimizadores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p-mfolch\Documents\Proyecto_Tintos_CyT\Optimizacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9CC0535-B6C7-4935-A033-045E019AA903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D725696-A2C7-4A62-A6D2-62F7867DE935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="687" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="687" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -24,62 +24,62 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pruebas PSO'!$A$2:$X$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Pruebas variedades'!$A$1:$AF$1</definedName>
-    <definedName name="_xlchart.v1.0" hidden="1">'Pruebas variedades'!$C$10</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'Pruebas variedades'!$C$14</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">'Pruebas variedades'!$C$2</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">'Pruebas variedades'!$C$6</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">'Pruebas variedades'!$T$10:$T$13</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">'Pruebas variedades'!$T$14:$T$17</definedName>
-    <definedName name="_xlchart.v1.14" hidden="1">'Pruebas variedades'!$T$2:$T$5</definedName>
-    <definedName name="_xlchart.v1.15" hidden="1">'Pruebas variedades'!$T$6:$T$9</definedName>
-    <definedName name="_xlchart.v1.16" hidden="1">'Pruebas variedades'!$C$10</definedName>
-    <definedName name="_xlchart.v1.17" hidden="1">'Pruebas variedades'!$C$14</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">'Pruebas variedades'!$C$2</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">'Pruebas variedades'!$C$6</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'Pruebas variedades'!$C$2</definedName>
-    <definedName name="_xlchart.v1.20" hidden="1">'Pruebas variedades'!$U$10:$U$13</definedName>
-    <definedName name="_xlchart.v1.21" hidden="1">'Pruebas variedades'!$U$14:$U$17</definedName>
-    <definedName name="_xlchart.v1.22" hidden="1">'Pruebas variedades'!$U$2:$U$5</definedName>
-    <definedName name="_xlchart.v1.23" hidden="1">'Pruebas variedades'!$U$6:$U$9</definedName>
-    <definedName name="_xlchart.v1.24" hidden="1">'Pruebas variedades'!$AB$10:$AB$13</definedName>
-    <definedName name="_xlchart.v1.25" hidden="1">'Pruebas variedades'!$AB$14:$AB$17</definedName>
-    <definedName name="_xlchart.v1.26" hidden="1">'Pruebas variedades'!$AB$2:$AB$5</definedName>
-    <definedName name="_xlchart.v1.27" hidden="1">'Pruebas variedades'!$AB$6:$AB$9</definedName>
-    <definedName name="_xlchart.v1.28" hidden="1">'Pruebas variedades'!$C$10</definedName>
-    <definedName name="_xlchart.v1.29" hidden="1">'Pruebas variedades'!$C$14</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'Pruebas variedades'!$C$6</definedName>
-    <definedName name="_xlchart.v1.30" hidden="1">'Pruebas variedades'!$C$2</definedName>
-    <definedName name="_xlchart.v1.31" hidden="1">'Pruebas variedades'!$C$6</definedName>
-    <definedName name="_xlchart.v1.32" hidden="1">'Pruebas variedades'!$AE$10:$AE$13</definedName>
-    <definedName name="_xlchart.v1.33" hidden="1">'Pruebas variedades'!$AE$14:$AE$17</definedName>
-    <definedName name="_xlchart.v1.34" hidden="1">'Pruebas variedades'!$AE$2:$AE$5</definedName>
-    <definedName name="_xlchart.v1.35" hidden="1">'Pruebas variedades'!$AE$6:$AE$9</definedName>
-    <definedName name="_xlchart.v1.36" hidden="1">'Pruebas variedades'!$C$10</definedName>
-    <definedName name="_xlchart.v1.37" hidden="1">'Pruebas variedades'!$C$14</definedName>
-    <definedName name="_xlchart.v1.38" hidden="1">'Pruebas variedades'!$C$2</definedName>
-    <definedName name="_xlchart.v1.39" hidden="1">'Pruebas variedades'!$C$6</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">'Pruebas variedades'!$S$10:$S$13</definedName>
-    <definedName name="_xlchart.v1.40" hidden="1">'Pruebas variedades'!$AC$10:$AC$13</definedName>
-    <definedName name="_xlchart.v1.41" hidden="1">'Pruebas variedades'!$AC$14:$AC$17</definedName>
-    <definedName name="_xlchart.v1.42" hidden="1">'Pruebas variedades'!$AC$2:$AC$5</definedName>
-    <definedName name="_xlchart.v1.43" hidden="1">'Pruebas variedades'!$AC$6:$AC$9</definedName>
-    <definedName name="_xlchart.v1.44" hidden="1">'Pruebas variedades'!$C$10</definedName>
-    <definedName name="_xlchart.v1.45" hidden="1">'Pruebas variedades'!$C$14</definedName>
-    <definedName name="_xlchart.v1.46" hidden="1">'Pruebas variedades'!$C$2</definedName>
-    <definedName name="_xlchart.v1.47" hidden="1">'Pruebas variedades'!$C$6</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">'Pruebas variedades'!$AB$10:$AB$13</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'Pruebas variedades'!$AB$14:$AB$17</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">'Pruebas variedades'!$AE$2:$AE$5</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">'Pruebas variedades'!$AE$6:$AE$9</definedName>
+    <definedName name="_xlchart.v1.12" hidden="1">'Pruebas variedades'!$C$10</definedName>
+    <definedName name="_xlchart.v1.13" hidden="1">'Pruebas variedades'!$C$14</definedName>
+    <definedName name="_xlchart.v1.14" hidden="1">'Pruebas variedades'!$C$2</definedName>
+    <definedName name="_xlchart.v1.15" hidden="1">'Pruebas variedades'!$C$6</definedName>
+    <definedName name="_xlchart.v1.16" hidden="1">'Pruebas variedades'!$AC$10:$AC$13</definedName>
+    <definedName name="_xlchart.v1.17" hidden="1">'Pruebas variedades'!$AC$14:$AC$17</definedName>
+    <definedName name="_xlchart.v1.18" hidden="1">'Pruebas variedades'!$AC$2:$AC$5</definedName>
+    <definedName name="_xlchart.v1.19" hidden="1">'Pruebas variedades'!$AC$6:$AC$9</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'Pruebas variedades'!$AB$2:$AB$5</definedName>
+    <definedName name="_xlchart.v1.20" hidden="1">'Pruebas variedades'!$C$10</definedName>
+    <definedName name="_xlchart.v1.21" hidden="1">'Pruebas variedades'!$C$14</definedName>
+    <definedName name="_xlchart.v1.22" hidden="1">'Pruebas variedades'!$C$2</definedName>
+    <definedName name="_xlchart.v1.23" hidden="1">'Pruebas variedades'!$C$6</definedName>
+    <definedName name="_xlchart.v1.24" hidden="1">'Pruebas variedades'!$C$10</definedName>
+    <definedName name="_xlchart.v1.25" hidden="1">'Pruebas variedades'!$C$14</definedName>
+    <definedName name="_xlchart.v1.26" hidden="1">'Pruebas variedades'!$C$2</definedName>
+    <definedName name="_xlchart.v1.27" hidden="1">'Pruebas variedades'!$C$6</definedName>
+    <definedName name="_xlchart.v1.28" hidden="1">'Pruebas variedades'!$S$10:$S$13</definedName>
+    <definedName name="_xlchart.v1.29" hidden="1">'Pruebas variedades'!$S$14:$S$17</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'Pruebas variedades'!$AB$6:$AB$9</definedName>
+    <definedName name="_xlchart.v1.30" hidden="1">'Pruebas variedades'!$S$2:$S$5</definedName>
+    <definedName name="_xlchart.v1.31" hidden="1">'Pruebas variedades'!$S$6:$S$9</definedName>
+    <definedName name="_xlchart.v1.32" hidden="1">'Pruebas variedades'!$C$10</definedName>
+    <definedName name="_xlchart.v1.33" hidden="1">'Pruebas variedades'!$C$14</definedName>
+    <definedName name="_xlchart.v1.34" hidden="1">'Pruebas variedades'!$C$2</definedName>
+    <definedName name="_xlchart.v1.35" hidden="1">'Pruebas variedades'!$C$6</definedName>
+    <definedName name="_xlchart.v1.36" hidden="1">'Pruebas variedades'!$U$10:$U$13</definedName>
+    <definedName name="_xlchart.v1.37" hidden="1">'Pruebas variedades'!$U$14:$U$17</definedName>
+    <definedName name="_xlchart.v1.38" hidden="1">'Pruebas variedades'!$U$2:$U$5</definedName>
+    <definedName name="_xlchart.v1.39" hidden="1">'Pruebas variedades'!$U$6:$U$9</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">'Pruebas variedades'!$C$10</definedName>
+    <definedName name="_xlchart.v1.40" hidden="1">'Pruebas variedades'!$C$10</definedName>
+    <definedName name="_xlchart.v1.41" hidden="1">'Pruebas variedades'!$C$14</definedName>
+    <definedName name="_xlchart.v1.42" hidden="1">'Pruebas variedades'!$C$2</definedName>
+    <definedName name="_xlchart.v1.43" hidden="1">'Pruebas variedades'!$C$6</definedName>
+    <definedName name="_xlchart.v1.44" hidden="1">'Pruebas variedades'!$T$10:$T$13</definedName>
+    <definedName name="_xlchart.v1.45" hidden="1">'Pruebas variedades'!$T$14:$T$17</definedName>
+    <definedName name="_xlchart.v1.46" hidden="1">'Pruebas variedades'!$T$2:$T$5</definedName>
+    <definedName name="_xlchart.v1.47" hidden="1">'Pruebas variedades'!$T$6:$T$9</definedName>
     <definedName name="_xlchart.v1.48" hidden="1">'Pruebas variedades'!$AF$10:$AF$13</definedName>
     <definedName name="_xlchart.v1.49" hidden="1">'Pruebas variedades'!$AF$14:$AF$17</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">'Pruebas variedades'!$S$14:$S$17</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">'Pruebas variedades'!$C$14</definedName>
     <definedName name="_xlchart.v1.50" hidden="1">'Pruebas variedades'!$AF$2:$AF$5</definedName>
     <definedName name="_xlchart.v1.51" hidden="1">'Pruebas variedades'!$AF$6:$AF$9</definedName>
     <definedName name="_xlchart.v1.52" hidden="1">'Pruebas variedades'!$C$10</definedName>
     <definedName name="_xlchart.v1.53" hidden="1">'Pruebas variedades'!$C$14</definedName>
     <definedName name="_xlchart.v1.54" hidden="1">'Pruebas variedades'!$C$2</definedName>
     <definedName name="_xlchart.v1.55" hidden="1">'Pruebas variedades'!$C$6</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">'Pruebas variedades'!$S$2:$S$5</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">'Pruebas variedades'!$S$6:$S$9</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">'Pruebas variedades'!$C$10</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">'Pruebas variedades'!$C$14</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">'Pruebas variedades'!$C$2</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">'Pruebas variedades'!$C$6</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">'Pruebas variedades'!$AE$10:$AE$13</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">'Pruebas variedades'!$AE$14:$AE$17</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -165,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="180">
   <si>
     <t>Set de datos:</t>
   </si>
@@ -696,6 +696,15 @@
   </si>
   <si>
     <t>p-value</t>
+  </si>
+  <si>
+    <t>100 K</t>
+  </si>
+  <si>
+    <t>52,4 K</t>
+  </si>
+  <si>
+    <t>100 - 52,4</t>
   </si>
 </sst>
 </file>
@@ -1388,7 +1397,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="307">
+  <cellXfs count="309">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1814,12 +1823,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1850,15 +1853,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1871,15 +1865,76 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1918,22 +1973,22 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.6</cx:f>
+        <cx:f>_xlchart.v1.30</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.7</cx:f>
+        <cx:f>_xlchart.v1.31</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.4</cx:f>
+        <cx:f>_xlchart.v1.28</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.5</cx:f>
+        <cx:f>_xlchart.v1.29</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1971,7 +2026,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000001-F3AE-4AF7-90E7-B6ECE0CB8583}" formatIdx="1">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.2</cx:f>
+              <cx:f>_xlchart.v1.26</cx:f>
               <cx:v>Cabernet Sauvignon</cx:v>
             </cx:txData>
           </cx:tx>
@@ -1983,7 +2038,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000002-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.3</cx:f>
+              <cx:f>_xlchart.v1.27</cx:f>
               <cx:v>Syrah</cx:v>
             </cx:txData>
           </cx:tx>
@@ -1995,7 +2050,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000003-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.0</cx:f>
+              <cx:f>_xlchart.v1.24</cx:f>
               <cx:v>Merlot</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2007,7 +2062,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000004-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.1</cx:f>
+              <cx:f>_xlchart.v1.25</cx:f>
               <cx:v>Carmenere</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2037,22 +2092,22 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.14</cx:f>
+        <cx:f>_xlchart.v1.46</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.15</cx:f>
+        <cx:f>_xlchart.v1.47</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.12</cx:f>
+        <cx:f>_xlchart.v1.44</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.13</cx:f>
+        <cx:f>_xlchart.v1.45</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -2090,7 +2145,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000001-F3AE-4AF7-90E7-B6ECE0CB8583}" formatIdx="1">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.10</cx:f>
+              <cx:f>_xlchart.v1.42</cx:f>
               <cx:v>Cabernet Sauvignon</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2102,7 +2157,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000002-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.11</cx:f>
+              <cx:f>_xlchart.v1.43</cx:f>
               <cx:v>Syrah</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2114,7 +2169,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000003-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.8</cx:f>
+              <cx:f>_xlchart.v1.40</cx:f>
               <cx:v>Merlot</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2126,7 +2181,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000004-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.9</cx:f>
+              <cx:f>_xlchart.v1.41</cx:f>
               <cx:v>Carmenere</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2157,22 +2212,22 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.22</cx:f>
+        <cx:f>_xlchart.v1.38</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.23</cx:f>
+        <cx:f>_xlchart.v1.39</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.20</cx:f>
+        <cx:f>_xlchart.v1.36</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.21</cx:f>
+        <cx:f>_xlchart.v1.37</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -2210,7 +2265,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000001-F3AE-4AF7-90E7-B6ECE0CB8583}" formatIdx="1">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.18</cx:f>
+              <cx:f>_xlchart.v1.34</cx:f>
               <cx:v>Cabernet Sauvignon</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2222,7 +2277,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000002-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.19</cx:f>
+              <cx:f>_xlchart.v1.35</cx:f>
               <cx:v>Syrah</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2234,7 +2289,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000003-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.16</cx:f>
+              <cx:f>_xlchart.v1.32</cx:f>
               <cx:v>Merlot</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2246,7 +2301,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000004-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.17</cx:f>
+              <cx:f>_xlchart.v1.33</cx:f>
               <cx:v>Carmenere</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2277,22 +2332,22 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.26</cx:f>
+        <cx:f>_xlchart.v1.2</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.27</cx:f>
+        <cx:f>_xlchart.v1.3</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.24</cx:f>
+        <cx:f>_xlchart.v1.0</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.25</cx:f>
+        <cx:f>_xlchart.v1.1</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -2330,7 +2385,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000001-F3AE-4AF7-90E7-B6ECE0CB8583}" formatIdx="1">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.30</cx:f>
+              <cx:f>_xlchart.v1.6</cx:f>
               <cx:v>Cabernet Sauvignon</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2342,7 +2397,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000002-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.31</cx:f>
+              <cx:f>_xlchart.v1.7</cx:f>
               <cx:v>Syrah</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2354,7 +2409,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000003-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.28</cx:f>
+              <cx:f>_xlchart.v1.4</cx:f>
               <cx:v>Merlot</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2366,7 +2421,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000004-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.29</cx:f>
+              <cx:f>_xlchart.v1.5</cx:f>
               <cx:v>Carmenere</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2397,22 +2452,22 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.42</cx:f>
+        <cx:f>_xlchart.v1.18</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.43</cx:f>
+        <cx:f>_xlchart.v1.19</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.40</cx:f>
+        <cx:f>_xlchart.v1.16</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.41</cx:f>
+        <cx:f>_xlchart.v1.17</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -2450,7 +2505,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000001-F3AE-4AF7-90E7-B6ECE0CB8583}" formatIdx="1">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.46</cx:f>
+              <cx:f>_xlchart.v1.22</cx:f>
               <cx:v>Cabernet Sauvignon</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2462,7 +2517,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000002-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.47</cx:f>
+              <cx:f>_xlchart.v1.23</cx:f>
               <cx:v>Syrah</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2474,7 +2529,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000003-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.44</cx:f>
+              <cx:f>_xlchart.v1.20</cx:f>
               <cx:v>Merlot</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2486,7 +2541,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000004-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.45</cx:f>
+              <cx:f>_xlchart.v1.21</cx:f>
               <cx:v>Carmenere</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2517,22 +2572,22 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.34</cx:f>
+        <cx:f>_xlchart.v1.10</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.35</cx:f>
+        <cx:f>_xlchart.v1.11</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.32</cx:f>
+        <cx:f>_xlchart.v1.8</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.33</cx:f>
+        <cx:f>_xlchart.v1.9</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -2570,7 +2625,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000001-F3AE-4AF7-90E7-B6ECE0CB8583}" formatIdx="1">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.38</cx:f>
+              <cx:f>_xlchart.v1.14</cx:f>
               <cx:v>Cabernet Sauvignon</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2582,7 +2637,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000002-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.39</cx:f>
+              <cx:f>_xlchart.v1.15</cx:f>
               <cx:v>Syrah</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2594,7 +2649,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000003-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.36</cx:f>
+              <cx:f>_xlchart.v1.12</cx:f>
               <cx:v>Merlot</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2606,7 +2661,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000004-F3AE-4AF7-90E7-B6ECE0CB8583}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.37</cx:f>
+              <cx:f>_xlchart.v1.13</cx:f>
               <cx:v>Carmenere</cx:v>
             </cx:txData>
           </cx:tx>
@@ -7023,8 +7078,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="10919460" y="171450"/>
-              <a:ext cx="4572000" cy="2743200"/>
+              <a:off x="10896600" y="167640"/>
+              <a:ext cx="4562475" cy="2714625"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7101,8 +7156,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="15552420" y="182880"/>
-              <a:ext cx="4572000" cy="2743200"/>
+              <a:off x="15516225" y="180975"/>
+              <a:ext cx="4562475" cy="2714625"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7179,8 +7234,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="20223480" y="198120"/>
-              <a:ext cx="4572000" cy="2743200"/>
+              <a:off x="20183475" y="200025"/>
+              <a:ext cx="4552950" cy="2714625"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7257,8 +7312,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="15537180" y="3048000"/>
-              <a:ext cx="4572000" cy="2743200"/>
+              <a:off x="15506700" y="3019425"/>
+              <a:ext cx="4562475" cy="2714625"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7335,8 +7390,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="20200620" y="3048000"/>
-              <a:ext cx="4572000" cy="2743200"/>
+              <a:off x="20154900" y="3019425"/>
+              <a:ext cx="4562475" cy="2714625"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7413,8 +7468,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="15529560" y="6012180"/>
-              <a:ext cx="4572000" cy="2743200"/>
+              <a:off x="15497175" y="5953125"/>
+              <a:ext cx="4562475" cy="2714625"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7491,8 +7546,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="20193000" y="5958840"/>
-              <a:ext cx="4572000" cy="2743200"/>
+              <a:off x="20145375" y="5895975"/>
+              <a:ext cx="4562475" cy="2714625"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -9601,25 +9656,25 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B2" s="292" t="s">
+      <c r="B2" s="290" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="291" t="s">
+      <c r="C2" s="289" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="291"/>
-      <c r="E2" s="291"/>
-      <c r="F2" s="291"/>
-      <c r="G2" s="294" t="s">
+      <c r="D2" s="289"/>
+      <c r="E2" s="289"/>
+      <c r="F2" s="289"/>
+      <c r="G2" s="292" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="294" t="s">
+      <c r="H2" s="292" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="294" t="s">
+      <c r="I2" s="292" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="289" t="s">
+      <c r="J2" s="287" t="s">
         <v>6</v>
       </c>
       <c r="L2" t="s">
@@ -9627,7 +9682,7 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="293"/>
+      <c r="B3" s="291"/>
       <c r="C3" s="16" t="s">
         <v>3</v>
       </c>
@@ -9640,10 +9695,10 @@
       <c r="F3" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="295"/>
-      <c r="H3" s="295"/>
-      <c r="I3" s="295"/>
-      <c r="J3" s="296"/>
+      <c r="G3" s="293"/>
+      <c r="H3" s="293"/>
+      <c r="I3" s="293"/>
+      <c r="J3" s="294"/>
       <c r="L3" t="s">
         <v>15</v>
       </c>
@@ -11151,30 +11206,30 @@
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B71" s="292" t="s">
+      <c r="B71" s="290" t="s">
         <v>1</v>
       </c>
-      <c r="C71" s="291" t="s">
+      <c r="C71" s="289" t="s">
         <v>2</v>
       </c>
-      <c r="D71" s="291"/>
-      <c r="E71" s="291"/>
-      <c r="F71" s="291"/>
-      <c r="G71" s="294" t="s">
+      <c r="D71" s="289"/>
+      <c r="E71" s="289"/>
+      <c r="F71" s="289"/>
+      <c r="G71" s="292" t="s">
         <v>12</v>
       </c>
-      <c r="H71" s="294" t="s">
+      <c r="H71" s="292" t="s">
         <v>9</v>
       </c>
-      <c r="I71" s="294" t="s">
+      <c r="I71" s="292" t="s">
         <v>10</v>
       </c>
-      <c r="J71" s="289" t="s">
+      <c r="J71" s="287" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="72" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B72" s="297"/>
+      <c r="B72" s="295"/>
       <c r="C72" s="7" t="s">
         <v>3</v>
       </c>
@@ -11187,10 +11242,10 @@
       <c r="F72" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G72" s="298"/>
-      <c r="H72" s="298"/>
-      <c r="I72" s="298"/>
-      <c r="J72" s="290"/>
+      <c r="G72" s="296"/>
+      <c r="H72" s="296"/>
+      <c r="I72" s="296"/>
+      <c r="J72" s="288"/>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B73" s="8" t="s">
@@ -11434,48 +11489,48 @@
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="B2" s="300" t="s">
+      <c r="B2" s="301" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="301" t="s">
+      <c r="C2" s="304" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="301"/>
-      <c r="E2" s="301"/>
-      <c r="F2" s="301"/>
-      <c r="G2" s="300" t="s">
+      <c r="D2" s="304"/>
+      <c r="E2" s="304"/>
+      <c r="F2" s="304"/>
+      <c r="G2" s="301" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="300" t="s">
+      <c r="H2" s="301" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="300" t="s">
+      <c r="I2" s="301" t="s">
         <v>34</v>
       </c>
-      <c r="N2" s="300" t="s">
+      <c r="N2" s="301" t="s">
         <v>40</v>
       </c>
-      <c r="O2" s="306" t="s">
+      <c r="O2" s="302" t="s">
         <v>1</v>
       </c>
-      <c r="P2" s="303" t="s">
+      <c r="P2" s="298" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="304"/>
-      <c r="R2" s="304"/>
-      <c r="S2" s="305"/>
-      <c r="T2" s="298" t="s">
+      <c r="Q2" s="299"/>
+      <c r="R2" s="299"/>
+      <c r="S2" s="300"/>
+      <c r="T2" s="296" t="s">
         <v>9</v>
       </c>
-      <c r="U2" s="298" t="s">
+      <c r="U2" s="296" t="s">
         <v>6</v>
       </c>
-      <c r="V2" s="298" t="s">
+      <c r="V2" s="296" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="B3" s="300"/>
+      <c r="B3" s="301"/>
       <c r="C3" s="50" t="s">
         <v>3</v>
       </c>
@@ -11488,11 +11543,11 @@
       <c r="F3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="300"/>
-      <c r="H3" s="300"/>
-      <c r="I3" s="300"/>
-      <c r="N3" s="300"/>
-      <c r="O3" s="306"/>
+      <c r="G3" s="301"/>
+      <c r="H3" s="301"/>
+      <c r="I3" s="301"/>
+      <c r="N3" s="301"/>
+      <c r="O3" s="302"/>
       <c r="P3" s="50" t="s">
         <v>3</v>
       </c>
@@ -11505,9 +11560,9 @@
       <c r="S3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="T3" s="302"/>
-      <c r="U3" s="302"/>
-      <c r="V3" s="302"/>
+      <c r="T3" s="297"/>
+      <c r="U3" s="297"/>
+      <c r="V3" s="297"/>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
@@ -11929,27 +11984,27 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B21" s="300" t="s">
+      <c r="B21" s="301" t="s">
         <v>1</v>
       </c>
-      <c r="C21" s="301" t="s">
+      <c r="C21" s="304" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="301"/>
-      <c r="E21" s="301"/>
-      <c r="F21" s="301"/>
-      <c r="G21" s="300" t="s">
+      <c r="D21" s="304"/>
+      <c r="E21" s="304"/>
+      <c r="F21" s="304"/>
+      <c r="G21" s="301" t="s">
         <v>9</v>
       </c>
-      <c r="H21" s="300" t="s">
+      <c r="H21" s="301" t="s">
         <v>6</v>
       </c>
-      <c r="I21" s="300" t="s">
+      <c r="I21" s="301" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B22" s="300"/>
+      <c r="B22" s="301"/>
       <c r="C22" s="50" t="s">
         <v>3</v>
       </c>
@@ -11962,9 +12017,9 @@
       <c r="F22" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G22" s="300"/>
-      <c r="H22" s="300"/>
-      <c r="I22" s="300"/>
+      <c r="G22" s="301"/>
+      <c r="H22" s="301"/>
+      <c r="I22" s="301"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B23" s="2" t="s">
@@ -12216,28 +12271,28 @@
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B40" s="300" t="s">
+      <c r="B40" s="301" t="s">
         <v>1</v>
       </c>
-      <c r="C40" s="301" t="s">
+      <c r="C40" s="304" t="s">
         <v>2</v>
       </c>
-      <c r="D40" s="301"/>
-      <c r="E40" s="301"/>
-      <c r="F40" s="301"/>
-      <c r="G40" s="300" t="s">
+      <c r="D40" s="304"/>
+      <c r="E40" s="304"/>
+      <c r="F40" s="304"/>
+      <c r="G40" s="301" t="s">
         <v>9</v>
       </c>
-      <c r="H40" s="300" t="s">
+      <c r="H40" s="301" t="s">
         <v>6</v>
       </c>
-      <c r="I40" s="300" t="s">
+      <c r="I40" s="301" t="s">
         <v>34</v>
       </c>
-      <c r="J40" s="299"/>
+      <c r="J40" s="303"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B41" s="300"/>
+      <c r="B41" s="301"/>
       <c r="C41" s="50" t="s">
         <v>3</v>
       </c>
@@ -12250,10 +12305,10 @@
       <c r="F41" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G41" s="300"/>
-      <c r="H41" s="300"/>
-      <c r="I41" s="300"/>
-      <c r="J41" s="299"/>
+      <c r="G41" s="301"/>
+      <c r="H41" s="301"/>
+      <c r="I41" s="301"/>
+      <c r="J41" s="303"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B42" s="2" t="s">
@@ -12339,12 +12394,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="T2:T3"/>
-    <mergeCell ref="P2:S2"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
     <mergeCell ref="J40:J41"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="B21:B22"/>
@@ -12361,6 +12410,12 @@
     <mergeCell ref="G40:G41"/>
     <mergeCell ref="H40:H41"/>
     <mergeCell ref="I40:I41"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="T2:T3"/>
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -23307,7 +23362,7 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="287" t="s">
+      <c r="A15" s="305" t="s">
         <v>171</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -23343,7 +23398,7 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="287"/>
+      <c r="A16" s="305"/>
       <c r="B16" s="2" t="s">
         <v>166</v>
       </c>
@@ -23377,7 +23432,7 @@
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="287"/>
+      <c r="A17" s="305"/>
       <c r="B17" s="2" t="s">
         <v>167</v>
       </c>
@@ -23411,7 +23466,7 @@
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="287"/>
+      <c r="A18" s="305"/>
       <c r="B18" s="2" t="s">
         <v>168</v>
       </c>
@@ -23445,7 +23500,7 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="287"/>
+      <c r="A19" s="305"/>
       <c r="B19" s="2" t="s">
         <v>169</v>
       </c>
@@ -23479,7 +23534,7 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="287"/>
+      <c r="A20" s="305"/>
       <c r="B20" s="2" t="s">
         <v>170</v>
       </c>
@@ -23513,7 +23568,7 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="288" t="s">
+      <c r="A21" s="306" t="s">
         <v>173</v>
       </c>
       <c r="B21" s="2" t="s">
@@ -23549,7 +23604,7 @@
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="288"/>
+      <c r="A22" s="306"/>
       <c r="B22" s="2" t="s">
         <v>166</v>
       </c>
@@ -23583,7 +23638,7 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="288"/>
+      <c r="A23" s="306"/>
       <c r="B23" s="2" t="s">
         <v>167</v>
       </c>
@@ -23617,7 +23672,7 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="288"/>
+      <c r="A24" s="306"/>
       <c r="B24" s="2" t="s">
         <v>168</v>
       </c>
@@ -23651,7 +23706,7 @@
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="288"/>
+      <c r="A25" s="306"/>
       <c r="B25" s="2" t="s">
         <v>169</v>
       </c>
@@ -23685,7 +23740,7 @@
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="288"/>
+      <c r="A26" s="306"/>
       <c r="B26" s="2" t="s">
         <v>170</v>
       </c>
@@ -23719,7 +23774,7 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="287" t="s">
+      <c r="A27" s="305" t="s">
         <v>176</v>
       </c>
       <c r="B27" s="2" t="s">
@@ -23755,7 +23810,7 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="287"/>
+      <c r="A28" s="305"/>
       <c r="B28" s="2" t="s">
         <v>166</v>
       </c>
@@ -23789,7 +23844,7 @@
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" s="287"/>
+      <c r="A29" s="305"/>
       <c r="B29" s="2" t="s">
         <v>167</v>
       </c>
@@ -23823,7 +23878,7 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="287"/>
+      <c r="A30" s="305"/>
       <c r="B30" s="2" t="s">
         <v>168</v>
       </c>
@@ -23857,7 +23912,7 @@
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" s="287"/>
+      <c r="A31" s="305"/>
       <c r="B31" s="2" t="s">
         <v>169</v>
       </c>
@@ -23891,7 +23946,7 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="287"/>
+      <c r="A32" s="305"/>
       <c r="B32" s="2" t="s">
         <v>170</v>
       </c>
@@ -23931,10 +23986,10 @@
     <mergeCell ref="A27:A32"/>
   </mergeCells>
   <conditionalFormatting sqref="C27:I32">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
       <formula>0.05</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
       <formula>0.05</formula>
     </cfRule>
   </conditionalFormatting>
@@ -23946,9 +24001,362 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{623BAF27-CEDB-4C6E-9684-D0A7DA63A489}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="L1" t="s">
+        <v>175</v>
+      </c>
+      <c r="M1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C2" s="104" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="104" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" s="104" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" s="104" t="s">
+        <v>61</v>
+      </c>
+      <c r="G2" s="104" t="s">
+        <v>65</v>
+      </c>
+      <c r="H2" s="104" t="s">
+        <v>63</v>
+      </c>
+      <c r="I2" s="104" t="s">
+        <v>64</v>
+      </c>
+      <c r="J2" s="104" t="s">
+        <v>164</v>
+      </c>
+      <c r="K2" s="104" t="s">
+        <v>172</v>
+      </c>
+      <c r="L2" s="104" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" s="307" t="s">
+        <v>177</v>
+      </c>
+      <c r="B3" s="231" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3" s="2">
+        <f>'Pruebas variedades'!S20</f>
+        <v>9.2298363684499451E-2</v>
+      </c>
+      <c r="D3" s="2">
+        <f>'Pruebas variedades'!T20</f>
+        <v>1.4329067184418673</v>
+      </c>
+      <c r="E3" s="2">
+        <f>'Pruebas variedades'!U20</f>
+        <v>5.7996119857887543</v>
+      </c>
+      <c r="F3" s="2">
+        <f>'Pruebas variedades'!AB20</f>
+        <v>3.5090837563444373</v>
+      </c>
+      <c r="G3" s="2">
+        <f>'Pruebas variedades'!AC20</f>
+        <v>6.4898138659096531</v>
+      </c>
+      <c r="H3" s="2">
+        <f>'Pruebas variedades'!AE20</f>
+        <v>0.35703827704971747</v>
+      </c>
+      <c r="I3" s="2">
+        <f>'Pruebas variedades'!AF20</f>
+        <v>0.6505524194218153</v>
+      </c>
+      <c r="J3" s="2">
+        <f>'Pruebas variedades'!H20+4</f>
+        <v>207</v>
+      </c>
+      <c r="K3" s="2">
+        <v>4</v>
+      </c>
+      <c r="L3" s="2">
+        <f>J3-$M$1</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" s="307"/>
+      <c r="B4" s="258" t="s">
+        <v>126</v>
+      </c>
+      <c r="C4" s="2">
+        <f>'Pruebas variedades'!S21</f>
+        <v>5.6623375029387607E-2</v>
+      </c>
+      <c r="D4" s="2">
+        <f>'Pruebas variedades'!T21</f>
+        <v>1.0674755455728331</v>
+      </c>
+      <c r="E4" s="2">
+        <f>'Pruebas variedades'!U21</f>
+        <v>3.7373191145113278</v>
+      </c>
+      <c r="F4" s="2">
+        <f>'Pruebas variedades'!AB21</f>
+        <v>2.1862359325412095</v>
+      </c>
+      <c r="G4" s="2">
+        <f>'Pruebas variedades'!AC21</f>
+        <v>1.7784686194618968</v>
+      </c>
+      <c r="H4" s="2">
+        <f>'Pruebas variedades'!AE21</f>
+        <v>0.42569788985141976</v>
+      </c>
+      <c r="I4" s="2">
+        <f>'Pruebas variedades'!AF21</f>
+        <v>0.31051964173200736</v>
+      </c>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" s="308" t="s">
+        <v>178</v>
+      </c>
+      <c r="B5" s="231" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" s="2">
+        <f>'Pruebas variedades'!S57</f>
+        <v>0.2355949551118362</v>
+      </c>
+      <c r="D5" s="2">
+        <f>'Pruebas variedades'!T57</f>
+        <v>1.973789012508822</v>
+      </c>
+      <c r="E5" s="2">
+        <f>'Pruebas variedades'!U57</f>
+        <v>1.8453025658142468</v>
+      </c>
+      <c r="F5" s="2">
+        <f>'Pruebas variedades'!AB57</f>
+        <v>3.9990542652753476</v>
+      </c>
+      <c r="G5" s="2">
+        <f>'Pruebas variedades'!AC57</f>
+        <v>3.3050793553530129</v>
+      </c>
+      <c r="H5" s="2">
+        <f>'Pruebas variedades'!AE57</f>
+        <v>0.45254688471599674</v>
+      </c>
+      <c r="I5" s="2">
+        <f>'Pruebas variedades'!AF57</f>
+        <v>0.50152131860861004</v>
+      </c>
+      <c r="J5" s="2">
+        <f>'Pruebas variedades'!H22+4</f>
+        <v>150</v>
+      </c>
+      <c r="K5" s="2">
+        <v>4</v>
+      </c>
+      <c r="L5" s="2">
+        <f>J5-$M$1</f>
+        <v>143</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" s="308"/>
+      <c r="B6" s="258" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" s="101">
+        <f>'Pruebas variedades'!S58</f>
+        <v>0.30040960079264961</v>
+      </c>
+      <c r="D6" s="2">
+        <f>'Pruebas variedades'!T58</f>
+        <v>2.2384131517421531</v>
+      </c>
+      <c r="E6" s="2">
+        <f>'Pruebas variedades'!U58</f>
+        <v>0.84220084028758913</v>
+      </c>
+      <c r="F6" s="2">
+        <f>'Pruebas variedades'!AB58</f>
+        <v>2.0186505471776366</v>
+      </c>
+      <c r="G6" s="2">
+        <f>'Pruebas variedades'!AC58</f>
+        <v>4.2058978534079605</v>
+      </c>
+      <c r="H6" s="2">
+        <f>'Pruebas variedades'!AE58</f>
+        <v>0.39413496827723071</v>
+      </c>
+      <c r="I6" s="101">
+        <f>'Pruebas variedades'!AF58</f>
+        <v>0.24939449922529852</v>
+      </c>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C13" s="179" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="179" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="179" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="179" t="s">
+        <v>61</v>
+      </c>
+      <c r="G13" s="179" t="s">
+        <v>65</v>
+      </c>
+      <c r="H13" s="179" t="s">
+        <v>63</v>
+      </c>
+      <c r="I13" s="179" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B14" s="308" t="s">
+        <v>179</v>
+      </c>
+      <c r="C14" s="2">
+        <f>(C3-C5)/(SQRT(C4^2+C6^2))</f>
+        <v>-0.46874996308960598</v>
+      </c>
+      <c r="D14" s="2">
+        <f t="shared" ref="D14:I14" si="0">(D3-D5)/(SQRT(D4^2+D6^2))</f>
+        <v>-0.21810483642857845</v>
+      </c>
+      <c r="E14" s="2">
+        <f t="shared" si="0"/>
+        <v>1.0321768789242416</v>
+      </c>
+      <c r="F14" s="2">
+        <f t="shared" si="0"/>
+        <v>-0.16465920606646894</v>
+      </c>
+      <c r="G14" s="2">
+        <f t="shared" si="0"/>
+        <v>0.6974191752318577</v>
+      </c>
+      <c r="H14" s="2">
+        <f t="shared" si="0"/>
+        <v>-0.16463060577754765</v>
+      </c>
+      <c r="I14" s="2">
+        <f t="shared" si="0"/>
+        <v>0.37419488680900143</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B15" s="308"/>
+      <c r="C15" s="2">
+        <f>(C4^2+C6^2)^2/(C4^4/$L$3+C6^4/$L$5)</f>
+        <v>153.20308011950746</v>
+      </c>
+      <c r="D15" s="2">
+        <f t="shared" ref="D15:I15" si="1">(D4^2+D6^2)^2/(D4^4/$L$3+D6^4/$L$5)</f>
+        <v>207.75629171825344</v>
+      </c>
+      <c r="E15" s="2">
+        <f t="shared" si="1"/>
+        <v>220.03500904366837</v>
+      </c>
+      <c r="F15" s="2">
+        <f t="shared" si="1"/>
+        <v>340.37500181005515</v>
+      </c>
+      <c r="G15" s="2">
+        <f t="shared" si="1"/>
+        <v>194.268689666532</v>
+      </c>
+      <c r="H15" s="2">
+        <f t="shared" si="1"/>
+        <v>340.21017923061174</v>
+      </c>
+      <c r="I15" s="2">
+        <f t="shared" si="1"/>
+        <v>342.1349003972461</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B16" s="308"/>
+      <c r="C16" s="2">
+        <f>_xlfn.T.DIST.2T(ABS(C14),C15)</f>
+        <v>0.63991555954669144</v>
+      </c>
+      <c r="D16" s="2">
+        <f t="shared" ref="D16:I16" si="2">_xlfn.T.DIST.2T(ABS(D14),D15)</f>
+        <v>0.82756228902040641</v>
+      </c>
+      <c r="E16" s="2">
+        <f t="shared" si="2"/>
+        <v>0.30312261130172646</v>
+      </c>
+      <c r="F16" s="2">
+        <f t="shared" si="2"/>
+        <v>0.86931007602368837</v>
+      </c>
+      <c r="G16" s="2">
+        <f t="shared" si="2"/>
+        <v>0.48637545875939847</v>
+      </c>
+      <c r="H16" s="2">
+        <f t="shared" si="2"/>
+        <v>0.86933257110954354</v>
+      </c>
+      <c r="I16" s="2">
+        <f t="shared" si="2"/>
+        <v>0.70849121751365174</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B14:B16"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C16:I16">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
+      <formula>0.05</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
+      <formula>0.05</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>